<commit_message>
Update: Synchronisation des derniers rapports Excel et JSON
</commit_message>
<xml_diff>
--- a/data/cyber_security_catalogues.xlsx
+++ b/data/cyber_security_catalogues.xlsx
@@ -456,7 +456,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>228182</v>
+        <v>228183</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -475,7 +475,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-06-13T17:45:03Z</t>
+          <t>2026-06-13T17:52:59Z</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3396,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-06-12T16:16:40Z</t>
+          <t>2026-06-13T17:49:34Z</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Hack-with-Github/Awesome-Security-Gists</t>
+          <t>tcostam/awesome-command-control</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -4060,12 +4060,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>A collection of various GitHub gists for hackers, pentesters and security researchers</t>
+          <t>A collection of awesome Command &amp; Control (C2) frameworks, tools and resources for post-exploitation and red teaming assignments.</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://github.com/Hack-with-Github/Awesome-Security-Gists</t>
+          <t>https://github.com/tcostam/awesome-command-control</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -4075,14 +4075,14 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-06-08T15:44:24Z</t>
+          <t>2026-06-05T20:33:11Z</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>tcostam/awesome-command-control</t>
+          <t>Hack-with-Github/Awesome-Security-Gists</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -4090,12 +4090,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>A collection of awesome Command &amp; Control (C2) frameworks, tools and resources for post-exploitation and red teaming assignments.</t>
+          <t>A collection of various GitHub gists for hackers, pentesters and security researchers</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://github.com/tcostam/awesome-command-control</t>
+          <t>https://github.com/Hack-with-Github/Awesome-Security-Gists</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-06-05T20:33:11Z</t>
+          <t>2026-06-08T15:44:24Z</t>
         </is>
       </c>
     </row>
@@ -5912,7 +5912,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>netero1010/ScheduleRunner</t>
+          <t>ImAyrix/cut-cdn</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -5920,29 +5920,29 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>A C# tool with more flexibility to customize scheduled task for both persistence and lateral movement in red team operation</t>
+          <t>✂️ Removing CDN IPs from the list of IP addresses</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>https://github.com/netero1010/ScheduleRunner</t>
+          <t>https://github.com/ImAyrix/cut-cdn</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>C#</t>
+          <t>Go</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>2026-06-11T01:48:00Z</t>
+          <t>2026-06-13T14:50:23Z</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ImAyrix/cut-cdn</t>
+          <t>netero1010/ScheduleRunner</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -5950,29 +5950,29 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>✂️ Removing CDN IPs from the list of IP addresses</t>
+          <t>A C# tool with more flexibility to customize scheduled task for both persistence and lateral movement in red team operation</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>https://github.com/ImAyrix/cut-cdn</t>
+          <t>https://github.com/netero1010/ScheduleRunner</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Go</t>
+          <t>C#</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>2026-06-13T14:50:23Z</t>
+          <t>2026-06-11T01:48:00Z</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>noraj/rawsec-cybersecurity-inventory</t>
+          <t>trustedsec/artillery</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -5980,29 +5980,29 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>An inventory of tools and resources about CyberSecurity that  aims to help people to find everything related to CyberSecurity.</t>
+          <t>The Artillery Project is an open-source blue team tool designed to protect Linux and Windows operating systems through multiple methods.</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>https://github.com/noraj/rawsec-cybersecurity-inventory</t>
+          <t>https://github.com/trustedsec/artillery</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>JavaScript</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>2026-06-05T06:16:50Z</t>
+          <t>2026-05-04T13:07:07Z</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>trustedsec/artillery</t>
+          <t>noraj/rawsec-cybersecurity-inventory</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -6010,22 +6010,22 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>The Artillery Project is an open-source blue team tool designed to protect Linux and Windows operating systems through multiple methods.</t>
+          <t>An inventory of tools and resources about CyberSecurity that  aims to help people to find everything related to CyberSecurity.</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>https://github.com/trustedsec/artillery</t>
+          <t>https://github.com/noraj/rawsec-cybersecurity-inventory</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>JavaScript</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>2026-05-04T13:07:07Z</t>
+          <t>2026-06-05T06:16:50Z</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>yeahhub/Kali-Linux-Ebooks</t>
+          <t>cyberark/Evasor</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -6130,29 +6130,29 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Top 20 Kali Linux Related E-books (Free Download)</t>
+          <t>A tool to be used in post exploitation phase for blue and red teams to bypass APPLICATIONCONTROL policies</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>https://github.com/yeahhub/Kali-Linux-Ebooks</t>
+          <t>https://github.com/cyberark/Evasor</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>C#</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>2026-05-07T18:07:53Z</t>
+          <t>2026-05-26T23:42:40Z</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>cyberark/Evasor</t>
+          <t>yeahhub/Kali-Linux-Ebooks</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -6160,22 +6160,22 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>A tool to be used in post exploitation phase for blue and red teams to bypass APPLICATIONCONTROL policies</t>
+          <t>Top 20 Kali Linux Related E-books (Free Download)</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>https://github.com/cyberark/Evasor</t>
+          <t>https://github.com/yeahhub/Kali-Linux-Ebooks</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>C#</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>2026-05-26T23:42:40Z</t>
+          <t>2026-05-07T18:07:53Z</t>
         </is>
       </c>
     </row>
@@ -6242,7 +6242,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>zer0yu/Berserker</t>
+          <t>m4xx101/cryptex-oss</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -6250,29 +6250,29 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>A list of useful payloads for Web Application Security and Pentest/CTF</t>
+          <t>Open-source LLM red-teaming technique toolkit (162 transforms, 36 mutators, 25 tool surfaces). MIT.</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>https://github.com/zer0yu/Berserker</t>
+          <t>https://github.com/m4xx101/cryptex-oss</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>2026-06-01T19:42:38Z</t>
+          <t>2026-06-13T14:43:30Z</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>m4xx101/cryptex-oss</t>
+          <t>zer0yu/Berserker</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -6280,22 +6280,22 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Open-source LLM red-teaming technique toolkit (162 transforms, 36 mutators, 25 tool surfaces). MIT.</t>
+          <t>A list of useful payloads for Web Application Security and Pentest/CTF</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>https://github.com/m4xx101/cryptex-oss</t>
+          <t>https://github.com/zer0yu/Berserker</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>2026-06-13T14:43:30Z</t>
+          <t>2026-06-01T19:42:38Z</t>
         </is>
       </c>
     </row>
@@ -6362,7 +6362,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Eyadkelleh/awesome-skills-security</t>
+          <t>madhuakula/hacker-container</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -6370,29 +6370,29 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Security testing toolkit for AI Agent: curated SecLists wordlists, injection payloads, and expert agents for authorized pentesting, CTFs, and bug bounties</t>
+          <t>The Swiss Army Container for Cloud Native Security. Container with all the list of useful tools/commands while hacking and securing Containers, Kubernetes Clusters, and Cloud Native workloads.</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>https://github.com/Eyadkelleh/awesome-skills-security</t>
+          <t>https://github.com/madhuakula/hacker-container</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>Dockerfile</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-06-10T16:52:31Z</t>
+          <t>2026-06-08T15:46:43Z</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>madhuakula/hacker-container</t>
+          <t>Eyadkelleh/awesome-skills-security</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -6400,22 +6400,22 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>The Swiss Army Container for Cloud Native Security. Container with all the list of useful tools/commands while hacking and securing Containers, Kubernetes Clusters, and Cloud Native workloads.</t>
+          <t>Security testing toolkit for AI Agent: curated SecLists wordlists, injection payloads, and expert agents for authorized pentesting, CTFs, and bug bounties</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>https://github.com/madhuakula/hacker-container</t>
+          <t>https://github.com/Eyadkelleh/awesome-skills-security</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Dockerfile</t>
+          <t>PHP</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>2026-06-08T15:46:43Z</t>
+          <t>2026-06-10T16:52:31Z</t>
         </is>
       </c>
     </row>
@@ -6692,7 +6692,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Coff0xc/AutoRedTeam-Orchestrator</t>
+          <t>0xdea/blindsight</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -6700,29 +6700,29 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Enterprise AI Red Team Platform | 企业级AI红队平台 | 132 MCP Tools | Pure Python Engines | SDK+CLI+MCP | Auto-Download sqlmap/nuclei/ffuf | Production C2 | LLM Enhanced | Docker Sandbox | SARIF CI/CD | 1980 Tests</t>
+          <t>Red teaming tool to dump LSASS memory, bypassing basic countermeasures.</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>https://github.com/Coff0xc/AutoRedTeam-Orchestrator</t>
+          <t>https://github.com/0xdea/blindsight</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Rust</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>2026-06-12T01:48:22Z</t>
+          <t>2026-06-07T23:06:03Z</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>0xdea/blindsight</t>
+          <t>blackhatethicalhacking/SecretOpt1c</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -6730,29 +6730,29 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Red teaming tool to dump LSASS memory, bypassing basic countermeasures.</t>
+          <t>SecretOpt1c is a Red Team tool that helps uncover sensitive information in websites using ACTIVE and PASSIVE Techniques for Superior Accuracy!</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>https://github.com/0xdea/blindsight</t>
+          <t>https://github.com/blackhatethicalhacking/SecretOpt1c</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Rust</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>2026-06-07T23:06:03Z</t>
+          <t>2026-06-10T00:48:04Z</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>blackhatethicalhacking/SecretOpt1c</t>
+          <t>Coff0xc/AutoRedTeam-Orchestrator</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -6760,22 +6760,22 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>SecretOpt1c is a Red Team tool that helps uncover sensitive information in websites using ACTIVE and PASSIVE Techniques for Superior Accuracy!</t>
+          <t>Enterprise AI Red Team Platform | 企业级AI红队平台 | 132 MCP Tools | Pure Python Engines | SDK+CLI+MCP | Auto-Download sqlmap/nuclei/ffuf | Production C2 | LLM Enhanced | Docker Sandbox | SARIF CI/CD | 1980 Tests</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>https://github.com/blackhatethicalhacking/SecretOpt1c</t>
+          <t>https://github.com/Coff0xc/AutoRedTeam-Orchestrator</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>2026-06-10T00:48:04Z</t>
+          <t>2026-06-12T01:48:22Z</t>
         </is>
       </c>
     </row>
@@ -7352,7 +7352,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>security-prince/Resources-for-Application-Security</t>
+          <t>kh4sh3i/cloud-penetration-testing</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -7360,12 +7360,12 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Some good resources for getting started with application security</t>
+          <t>A curated list of cloud pentesting resource, contains AWS, Azure, Google Cloud</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>https://github.com/security-prince/Resources-for-Application-Security</t>
+          <t>https://github.com/kh4sh3i/cloud-penetration-testing</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -7375,14 +7375,14 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-06-10T02:32:41Z</t>
+          <t>2026-05-19T12:08:10Z</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>kh4sh3i/cloud-penetration-testing</t>
+          <t>security-prince/Resources-for-Application-Security</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -7390,12 +7390,12 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>A curated list of cloud pentesting resource, contains AWS, Azure, Google Cloud</t>
+          <t>Some good resources for getting started with application security</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>https://github.com/kh4sh3i/cloud-penetration-testing</t>
+          <t>https://github.com/security-prince/Resources-for-Application-Security</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -7405,7 +7405,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>2026-05-19T12:08:10Z</t>
+          <t>2026-06-10T02:32:41Z</t>
         </is>
       </c>
     </row>
@@ -7562,7 +7562,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>7WaySecurity/cloud_osint</t>
+          <t>FADL285/LINUX-BASICS-FOR-HACKERS-Book</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -7570,12 +7570,12 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>☁️ Curated Cloud OSINT resources — dorks, tools, and techniques for AWS, Azure, GCP, Oracle Cloud, and other major providers reconnaissance</t>
+          <t xml:space="preserve">Summary for Linux Basics For Hackers Book </t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>https://github.com/7WaySecurity/cloud_osint</t>
+          <t>https://github.com/FADL285/LINUX-BASICS-FOR-HACKERS-Book</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -7585,14 +7585,14 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>2026-06-03T00:08:36Z</t>
+          <t>2026-06-13T08:19:13Z</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>FADL285/LINUX-BASICS-FOR-HACKERS-Book</t>
+          <t>7WaySecurity/cloud_osint</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -7600,12 +7600,12 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Summary for Linux Basics For Hackers Book </t>
+          <t>☁️ Curated Cloud OSINT resources — dorks, tools, and techniques for AWS, Azure, GCP, Oracle Cloud, and other major providers reconnaissance</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>https://github.com/FADL285/LINUX-BASICS-FOR-HACKERS-Book</t>
+          <t>https://github.com/7WaySecurity/cloud_osint</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -7615,7 +7615,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>2026-06-13T08:19:13Z</t>
+          <t>2026-06-03T00:08:36Z</t>
         </is>
       </c>
     </row>
@@ -7682,7 +7682,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>cedowens/MacShellSwift</t>
+          <t>JoasASantos/Awesome-PenTest-Practice</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -7690,29 +7690,29 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Proof of concept MacOS post exploitation tool written in Swift. Designed as a POC for blue teams to build macOS detections. Author: Cedric Owens</t>
+          <t>Hackthebox, Vulnhub, TryHackMe and Real World PenTest</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>https://github.com/cedowens/MacShellSwift</t>
+          <t>https://github.com/JoasASantos/Awesome-PenTest-Practice</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Swift</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>2026-04-07T15:05:39Z</t>
+          <t>2026-06-01T21:22:55Z</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>pathakabhi24/CyberSecurity-Books</t>
+          <t>cedowens/MacShellSwift</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -7720,29 +7720,29 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>This repository has E-books on Cybersecs</t>
+          <t>Proof of concept MacOS post exploitation tool written in Swift. Designed as a POC for blue teams to build macOS detections. Author: Cedric Owens</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>https://github.com/pathakabhi24/CyberSecurity-Books</t>
+          <t>https://github.com/cedowens/MacShellSwift</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Swift</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>2026-06-08T15:34:06Z</t>
+          <t>2026-04-07T15:05:39Z</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>JoasASantos/Awesome-PenTest-Practice</t>
+          <t>pathakabhi24/CyberSecurity-Books</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -7750,12 +7750,12 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Hackthebox, Vulnhub, TryHackMe and Real World PenTest</t>
+          <t>This repository has E-books on Cybersecs</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>https://github.com/JoasASantos/Awesome-PenTest-Practice</t>
+          <t>https://github.com/pathakabhi24/CyberSecurity-Books</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
@@ -7765,7 +7765,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>2026-06-01T21:22:55Z</t>
+          <t>2026-06-08T15:34:06Z</t>
         </is>
       </c>
     </row>
@@ -7922,7 +7922,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>FabioBaroni/awesome-chinese-infosec-websites</t>
+          <t>CyDefOps/project-killchain</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -7930,29 +7930,29 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>A curated list of Chinese websites and personal blogs about ethical hacking and pentesting</t>
+          <t xml:space="preserve"> Welcome to Project KillChain, a comprehensive GitHub repository for Red and Blue Teams. This repository houses tools, scripts, techniques, and Indicators of Compromise (IOCs) aiding in cybersecurity operations. It facilitates penetration testing, incident response, digital forensics, and threat hunting.</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>https://github.com/FabioBaroni/awesome-chinese-infosec-websites</t>
+          <t>https://github.com/CyDefOps/project-killchain</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>2026-06-05T10:27:10Z</t>
+          <t>2026-04-15T12:11:21Z</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>CyDefOps/project-killchain</t>
+          <t>FabioBaroni/awesome-chinese-infosec-websites</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -7960,22 +7960,22 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Welcome to Project KillChain, a comprehensive GitHub repository for Red and Blue Teams. This repository houses tools, scripts, techniques, and Indicators of Compromise (IOCs) aiding in cybersecurity operations. It facilitates penetration testing, incident response, digital forensics, and threat hunting.</t>
+          <t>A curated list of Chinese websites and personal blogs about ethical hacking and pentesting</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>https://github.com/CyDefOps/project-killchain</t>
+          <t>https://github.com/FabioBaroni/awesome-chinese-infosec-websites</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>2026-04-15T12:11:21Z</t>
+          <t>2026-06-05T10:27:10Z</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>0x00ctrl/CyberSec-Books</t>
+          <t>swati1024/torrents</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -8110,12 +8110,12 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Some useful books related to Cybersecurity, Linux and more.</t>
+          <t>Skip to content   Search… All gists Back to GitHub Sign in Sign up Instantly share code, notes, and snippets.  @giansalex giansalex/torrent-courses-download-list.md forked from M-Younus/torrent courses download-list Last active 2 days ago 15188  Code Revisions 15 Stars 151 Forks 88 &lt;script src="https://gist.github.com/giansalex/4cd3631e94433bbbd71bf07aedb33a7b.js"&gt;&lt;/script&gt;     torrent-courses-download-list.md Torrent Courses List Download  http://kickass.to/infiniteskills-learning-jquery-mobile-working-files-t7967156.html http://kickass.to/lynda-bootstrap-3-advanced-web-development-2013-eng-t8167587.html http://kickass.to/lynda-css-advanced-typographic-techniques-t7928210.html http://kickass.to/lynda-html5-projects-interactive-charts-2013-eng-t8167670.html http://kickass.to/vtc-html5-css3-responsive-web-design-course-t7922533.html http://kickass.to/10gen-m101js-mongodb-for-node-js-developers-2013-eng-t8165205.html http://kickass.to/cbt-nuggets-amazon-web-services-aws-foundations-t7839734.html http://kickass.to/cbt-nuggets-apache-hadoop-t8027965.html http://kickass.to/cbt-nuggets-backtrack-and-kali-linux-t7677281.html http://kickass.to/cbt-nuggets-ccda-desgn-640-864-t8300917.html http://kickass.to/cbt-nuggets-ccna-wireless-iuwne-640-722-t8300389.html http://kickass.to/cbt-nuggets-cisco-ccna-labs-cisco-for-the-real-world-bonus-t6154766.html http://kickass.to/cbt-nuggets-cisco-ccnp-security-firewall-v2-0-642-618-azazredhat-t6955696.html http://kickass.to/cbt-nuggets-cisco-ccnp-security-secure-642-637-azazredhat-t6955710.html http://kickass.to/cbt-nuggets-comptia-network-videos-2010-gurufuel-t4648514.html http://kickass.to/cbt-nuggets-definitive-guide-to-working-with-gns3-by-keith-bar-t8301349.html http://kickass.to/cbt-nuggets-ec-council-certified-ethical-hacker-v7-0-t6801120.html http://kickass.to/cbt-nuggets-exam-walkthrough-cisco-icnd1ccent-100-101-t8516719.html http://kickass.to/cbt-nuggets-exam-walkthrough-cisco-icnd2ccna-200-101-t8524803.html http://kickass.to/cbt-nuggets-linux-in-the-real-world-with-shawn-powers-t7718107.html http://kickass.to/cbt-nuggets-linux-series-video-tutorial-t485320.html http://kickass.to/cbt-nuggets-lpi-linux-lpic-1-101-and-comptia-linux-t8031864.html http://kickass.to/cbt-nuggets-lpi-linux-lpic-1-102-and-comptia-linux-t8031871.html http://kickass.to/cbt-nuggets-mastering-vmware-view-5-and-preparing-for-the-vcp510-dt-exam-t8301829.html http://kickass.to/cbt-nuggets-vmware-virtualization-vcp-vsphere-5-t8300512.html http://kickass.to/cbt-nuggets-wireshark-with-keith-barker-t8040855.html http://kickass.to/comptia-network-n10-005-collection-t8319928.html http://kickass.to/developing-in-html5-with-javascript-and-css3-jump-start-t8277565.html http://kickass.to/eli-the-computer-guy-linux-t8647714.html http://kickass.to/foundations-of-programming-test-driven-development-t7522376.html http://kickass.to/infiniteskills-advanced-html5-programming-t7463355.html http://kickass.to/infiniteskills-cisco-ccna-certification-bundle-2013-t7645010.html http://kickass.to/infiniteskills-css3-transformations-and-animations-t7930047.html http://kickass.to/infiniteskills-learning-javascript-programming-t7625039.html http://kickass.to/infiniteskills-learning-python-programming-t7107001.html http://kickass.to/infiniteskills-learning-regular-expressions-t8028765.html http://kickass.to/infiniteskills-learning-whitehat-hacking-and-penetration-testing-t8303725.html http://kickass.to/infiniteskills-microsoft-windows-server-2012-certification-training-exam-70-410-t7379360.html http://kickass.to/infiniteskills-php-security-t8046511.html http://kickass.to/learning-vmware-esxi-and-vsphere-5-1-administration-training-t8030885.html http://kickass.to/linuxcbt-basic-security-edition-d3x-t7650913.html http://kickass.to/linuxcbt-config-mgmt-edition-d3x-t7650929.html http://kickass.to/linuxcbthttpdxil-edition-d3x-t7653897.html http://kickass.to/linuxcbt-vbox-edition-d3x-t7653916.html http://kickass.to/linuxcbt-webscan-edition-d3x-t7653922.html http://kickass.to/linuxcbt-winpython-edition-d3x-t7653942.html http://kickass.to/linuxcbt-xenvm-edition-d3x-t7653948.html http://kickass.to/lynda-com-foundations-of-programming-code-efficiency-t8604312.html http://kickass.to/lynda-com-foundations-of-programming-databases-t8596357.html http://kickass.to/lynda-com-foundations-of-programming-design-patterns-t8692867.html http://kickass.to/lynda-com-foundations-of-programming-fundamentals-t7600288.html http://kickass.to/lynda-com-foundations-of-programming-web-services-including-exercise-files-torrenters-t7797117.html http://kickass.to/lynda-com-ruby-on-rails-4-essential-training-dec-2013-t8438392.html http://kickass.to/lynda-foundations-of-programming-refactoring-code-t7524343.html http://kickass.to/lynda-foundations-of-programming-software-quality-assurance-sum1-here-silverrg-t8043799.html http://kickass.to/lynda-javascript-events-t7893809.html http://kickass.to/lynda-leading-with-emotional-intelligence-t8157240.html http://kickass.to/lynda-management-tips-t8154761.html http://kickass.to/mysql-database-tutorials-by-bucky-thenewboston-org-1-33-t8224550.html http://kickass.to/packtpub-advanced-penetration-testing-for-highly-secured-environments-t8300620.html http://kickass.to/pluralsight-mysql-query-optimization-and-performance-tuning-with-pinal-dave-t8553369.html http://kickass.to/pluralsight-relational-database-design-t8551479.html http://kickass.to/ruby-tutorial-bucky-totally-for-beginner-t8699509.html http://kickass.to/trainsignal-vmware-vcloud-director-5-1-essentials-t7495660.html http://kickass.to/trainsignal-vmware-vsphere-optimize-and-scale-vcap5-dca-t7495659.html http://kickass.to/trainsignal-vmware-workstation-9-for-the-it-admin-t7495658.html http://kickass.to/tutsplus-advanced-command-line-techniques-t7632228.html http://kickass.to/tutsplus-advanced-javascript-fundamentals-t6739742.html http://kickass.to/tutsplus-agile-design-patterns-2012-t6992118.html http://kickass.to/tutsplus-cleaner-code-with-coffeescript-t6741625.html http://kickass.to/tutsplus-detecting-code-smells-t8128341.html http://kickass.to/tutsplus-firebug-white-to-black-belt-v413hav-t7154501.html http://kickass.to/tutsplus-foundational-flask-creating-your-own-static-blog-generator-t8356996.html http://kickass.to/tutsplus-freelance-bootcamp-t6832678.html http://kickass.to/tutsplus-premium-e-book-mega-pack-v413hav-t7178526.html http://kickass.to/tutsplus-pro-workflow-for-web-designers-t6854268.html http://kickass.to/tutsplus-riding-ruby-on-rails-t6728201.html http://kickass.to/tutsplus-sql-essentials-t6746851.html http://kickass.to/tutsplus-tools-of-the-modern-web-developer-t8107617.html http://kickass.to/tutsplus-video-fundamentals-t6752217.html http://kickass.to/ine-ccna-wireless-640-722-iuwne-t8301376.html http://kickass.to/learn-metasploit-t8174472.html http://kickass.to/lynda-ruby-on-rails-essential-training-t7630711.html http://kickass.to/lynda-up-and-running-with-python-2013-eng-t8167709.html http://kickass.to/build-flat-responsive-website-from-scratch-complete-course-t8604527.html http://kickass.to/canvas-essentials-t8550909.html http://kickass.to/cbt-nuggets-70-331-microsoft-sharepoint-server-2013-x264-mkv-encod3r-t8595423.html http://kickass.to/cbt-nuggets-98-365-windows-server-admin-fundamentals-encod3r-t8613009.html http://kickass.to/cbt-nuggets-ccie-combo-pack-t271107.html http://kickass.to/cbt-nuggets-ccna-certification-videos-material-2010-gurufu-t4648321.html http://kickass.to/cbt-nuggets-juniper-networks-certified-specialist-security-jncis-sec-jn0-332-t8028083.html http://kickass.to/cehv7-cbt-nuggets-instructor-slides-tools-video-tools-study-guide-rar-t8705752.html http://kickass.to/cisco-ccna-initial-router-and-switch-configuration-t8648377.html http://kickass.to/cisco-ccna-security-aaa-and-ip-security-t8648378.html http://kickass.to/cisco-ccna-security-introduction-to-network-security-t8648381.html http://kickass.to/cisco-ccna-voice-configuration-and-advanced-features-t8648387.html http://kickass.to/cisco-ccna-voice-voice-overview-and-lab-setup-t8648386.html http://kickass.to/cisco-press-ccna-security-640-554-official-cert-guide-videos-t8648384.html http://kickass.to/coursera-neural-networks-and-machine-learning-geoffrey-hinton-university-of-toronto-t8568642.html http://kickass.to/eli-the-computer-guy-hacking-t8647661.html http://kickass.to/ine-ccie-data-center-storage-t8029396.html http://kickass.to/infinite-skills-learning-cloud-computing-with-amazon-web-services-2013-eng-t8703045.html http://kickass.to/infiniteskills-learning-tcp-ip-t8303739.html http://kickass.to/lynda-bootstrap-3-new-features-and-migration-t7958409.html http://kickass.to/lynda-bootstrap-adding-interactivity-to-your-site-t7519306.html http://kickass.to/lynda-com-jquery-ui-widgets-t8172743.html http://kickass.to/lynda-essential-training-t8157222.html http://kickass.to/lynda-foundation-incorporating-sass-and-compass-t7953037.html http://kickass.to/lynda-html5-projects-advanced-to-do-list-t7855578.html http://kickass.to/lynda-html5-projects-creating-a-responsive-presentation-2013-eng-t8167660.html http://kickass.to/lynda-online-presentations-with-reveal-js-2013-eng-t8167575.html http://kickass.to/lynda-teacher-tips-t8157202.html http://kickass.to/lynda-up-and-running-with-angularjs-t7982840.html http://kickass.to/lynda-up-and-running-with-bootstrap-3-t8011198.html http://kickass.to/lynda-up-and-running-with-cakephp-t7963854.html http://kickass.to/lynda-up-and-running-with-google-apps-script-t7917458.html http://kickass.to/lynda-up-and-running-with-php-codeigniter-t7849968.html http://kickass.to/lynda-web-semantics-t7899223.html http://kickass.to/lynda-wordpress-essential-training-2013-tutorial-t8270624.html http://kickass.to/pluralsight-aws-developer-fundamentals-2013-eng-t8703013.html http://kickass.to/pluralsight-bootstrap-3-t8214168.html http://kickass.to/pluralsight-cisco-ccie-routing-and-switching-implement-bgp-t8648391.html http://kickass.to/pluralsight-cisco-ccna-advanced-ethernet-and-file-management-t8051456.html http://kickass.to/pluralsight-cisco-ccna-security-firewalls-and-vpns-t8648393.html http://kickass.to/pluralsight-cisco-ccna-wan-technologies-learn-wide-area-network-wan-technologies-and-configuration-t7882351.html http://kickass.to/pluralsight-javascript-from-scratch-t7612372.html http://kickass.to/pluralsight-sublime-text-3-from-scratch-2013-eng-t8153034.html http://kickass.to/ten-ton-wordpress-mastery-video-t8452016.html http://kickass.to/trainsignal-microsoft-network-monitoring-t8028791.html http://kickass.to/tuts-plus-2013-bdd-in-rails-psiclone-t8474590.html http://kickass.to/tutsplus-advanced-css3-animations-t7791566.html http://kickass.to/tutsplus-an-introduction-to-node-js-t6744596.html http://kickass.to/tutsplus-better-statistics-with-google-charts-t7983386.html http://kickass.to/tutsplus-bootstrap-for-web-design-t8210956.html http://kickass.to/tutsplus-com-advanced-ui-techniques-2013-t7072722.html http://kickass.to/tutsplus-com-build-a-cms-in-codeigniter-2013-t7072644.html http://kickass.to/tutsplus-com-learning-mongodb-2013-t7072653.html http://kickass.to/tutsplus-computer-networks-distilled-v413hav-t7630795.html http://kickass.to/tutsplus-css-3d-essentials-t8027191.html http://kickass.to/tutsplus-css-noob-to-ninja-v413hav-t7475010.html http://kickass.to/tutsplus-css-tips-and-tricks-t8292119.html http://kickass.to/tutsplus-css3-essentials-t6608214.html http://kickass.to/tutsplus-css3-typography-techniques-t7882076.html http://kickass.to/tutsplus-design-patterns-in-ruby-t8354740.html http://kickass.to/tutsplus-fundamentals-of-design-t6645691.html http://kickass.to/tutsplus-fundamentals-of-print-design-t6667261.html http://kickass.to/tutsplus-fundamentals-of-ux-design-t6710443.html http://kickass.to/tutsplus-html-kickstart-essentials-t7969388.html http://kickass.to/tutsplus-html-tips-and-tricks-t8224648.html http://kickass.to/tutsplus-introduction-to-web-typography-t6662386.html http://kickass.to/tutsplus-javascript-fundamentals-101-t6738976.html http://kickass.to/tutsplus-jquery-ui-101-the-essentials-2013-eng-t8165125.html http://kickass.to/tutsplus-jquery-ui-101-the-essentials-t7791579.html http://kickass.to/tutsplus-jquery-ui-201-beyond-the-basics-t7791583.html http://kickass.to/tutsplus-jquery-ui-301-the-widget-factory-2013-eng-t8165109.html http://kickass.to/tutsplus-jquery-ui-301-the-widget-factory-working-files-2013-eng-t8180547.html http://kickass.to/tutsplus-laravel-essentials-t6722386.html http://kickass.to/tutsplus-logo-design-fundamentals-with-gary-simon-swatiate-t7867377.html http://kickass.to/tutsplus-mastering-corporate-design-v413hav-t7586047.html http://kickass.to/tutsplus-mastering-flat-design-v413hav-t7781777.html http://kickass.to/tutsplus-mastering-retro-web-design-v413hav-t7343186.html http://kickass.to/tutsplus-object-oriented-javascript-t6863065.html http://kickass.to/tutsplus-perfect-workflow-in-sublime-text-2-t6794850.html http://kickass.to/tutsplus-php-fundamentals-t6671312.html http://kickass.to/tutsplus-php-security-pitfalls-t7835091.html http://kickass.to/tutsplus-relational-databases-t8023530.html http://kickass.to/tutsplus-responsive-web-design-for-beginners-v413hav-t7385876.html http://kickass.to/tutsplus-responsive-web-design-techniques-t8103476.html http://kickass.to/tutsplus-responsive-web-design-with-foundation-t8103477.html http://kickass.to/tutsplus-simple-development-with-jquery-mobile-t6735499.html http://kickass.to/tutsplus-solid-design-patterns-t8208974.html http://kickass.to/tutsplus-test-driven-php-in-action-t6851704.html http://kickass.to/tutsplus-testing-tricks-for-php-and-laravel-developers-t7844807.html http://kickass.to/tutsplus-web-form-design-and-development-t8020800.html http://kickass.to/tutsplus-wordpress-plugin-development-essentials-t6615050.html http://kickass.to/udemy-build-an-instantly-updating-dynamic-website-with-jquery-ajax-t8415746.html http://kickass.to/udemy-psd-to-html5-css3-hand-code-a-beautiful-website-in-4-hours-t7740752.html http://kickass.to/video2brain-drupal-power-workshop-t6811365.html http://kickass.to/video2brain-exploring-css-positioning-t6683727.html http://kickass.to/video2brain-getting-started-with-joomla-t6600909.html http://kickass.to/video2brain-html5-for-beginners-learn-by-video-t6686185.html http://kickass.to/video2brain-html5-power-workshop-t6689166.html http://kickass.to/video2brain-php-5-3-advanced-web-application-programming-t6681560.html http://kickass.to/vtc-mysql-5-development-part-1-of-2-t7502575.html http://kickass.to/vtc-mysql-5-development-part-2-of-2-t7502576.html  https://thepiratebay.se/torrent/6113010/Linux_CBT_Scripting_BASH__PERL__PYTHON__PHP https://thepiratebay.se/torrent/7667241/CBT.Nuggets.Python.Programming.Python.Language-PLATO https://thepiratebay.se/torrent/8608894/InfiniteSkills_-_Web_Programming_With_Python https://thepiratebay.se/torrent/7838122/Lynda.com_-_Python_3_Essential_Training https://thepiratebay.se/torrent/7837732/python_book_collection https://thepiratebay.se/torrent/9549614/Pluralsight.com_-_Python_Fundamentals https://thepiratebay.se/torrent/5134755/LiveLessons.Python.Fundamentals.DVDR-HELL https://thepiratebay.se/torrent/7112525/The_New_Boston_-_Python_Programming_Tutorials http://kickass.to/lynda-up-and-running-with-python-2013-eng-t8167709.html  http://www.seedpeer.me/details/5730405/CBT-Nuggets---COMPTIA-SECURITY-SY0-201-WITH-SY0-301,-JK0-018-UPDATES.html http://www.seedpeer.me/details/6411686/CBT.Nuggets----IPv6.html http://www.seedpeer.me/details/6421814/CBT-Nuggets---Ubuntu.html http://www.seedpeer.me/details/6107414/LinuxCBT.Awk.Sed.Edition.html http://www.seedpeer.me/details/6107522/LinuxCBT-BASH-II-Edition-d3x.html http://www.seedpeer.me/details/4799869/LinuxCBT---Berkeley-Packet-Filters-BPF-Edition.html http://www.seedpeer.me/details/6881816/LinuxCBT--HTTPD-Edition.html http://www.seedpeer.me/details/6559038/LinuxCBT-Key-Files-edition.html http://www.seedpeer.me/details/6107600/LinuxCBT.MemCacheD.Edition-d3x.html http://www.seedpeer.me/details/5870507/LinuxCBT-Monitoring-Edition-feat-Nagios.html http://www.seedpeer.me/details/6107677/LinuxCBT-NIDS-Edition-d3x.html http://www.seedpeer.me/details/5925487/LinuxCBT-OpenLDAP-Edition.html http://www.seedpeer.me/details/6107558/LinuxCBT.OpenPGP.Edition-d3x.html http://www.seedpeer.me/details/6107692/LinuxCBT-OpenSSHv2-Edition-d3x.html http://www.seedpeer.me/details/6107699/LinuxCBT-PDNS-Edition-d3x.html http://www.seedpeer.me/details/2595080/LinuxCBT-Proxy-Edition-Feat-Squid-AG-torrent-[twistedtorrents2-com].html http://www.seedpeer.me/details/6110590/LinuxCBT-Samba-Edition-d3x.html http://www.seedpeer.me/details/6110595/LinuxCBT-SELinux-Edition-d3x.html http://www.seedpeer.me/details/4799871/LinuxCBT---SFTP-Edition.html http://www.seedpeer.me/details/6110602/LinuxCBT-SQLite-Edition-d3x.html http://www.seedpeer.me/details/5408265/LinuxCBT---Ubuntu-12.04-LTS.html http://www.seedpeer.me/details/4799857/LinuxCBT---UnixCBT-BSD8x-Edition-FreeBSD-8.2.html http://www.seedpeer.me/details/6110504/LinuxCBT.WinPerl.Edition-d3x.html http://www.seedpeer.me/details/6562861/Lynda-com---CMS-Fundamentals.html http://www.seedpeer.me/details/5247098/Lynda.com---Creating-an-Effective-Resume.html http://www.seedpeer.me/details/4989808/Lynda.com---CSS-with-LESS-and-SASS.html http://www.seedpeer.me/details/5340566/Lynda.com---Fundamentals-of-Software-Version-Control-Nov.-2012.html http://www.seedpeer.me/details/5569955/Lynda.com-GMail-For-Power-Users-V413HAV.html http://www.seedpeer.me/details/4631148/Lynda.com-Invaluable-Becoming-a-Leading-Authority.html http://www.seedpeer.me/details/4631108/Lynda.com-Invaluable-Building-Professional-Connections.html http://www.seedpeer.me/details/4623697/Lynda.com---Managing-a-Hosted-Website.html http://www.seedpeer.me/details/5236946/Lynda.com---PayPal-Essential-Training.html http://www.seedpeer.me/details/4596519/Lynda.com---PostgreSQL-9-With-PHP-Essential-Training-iRONiSO.html http://www.seedpeer.me/details/5016023/Lynda.com---Ruby-Essential-Training-with-Kevin-Skoglund.html http://www.seedpeer.me/details/4931186/Lynda.com---Using-Regular-Expressions.html http://www.seedpeer.me/details/6675342/Lynda---Git-Essential-Training.html http://www.seedpeer.me/details/6698556/Lynda---Leading-Change.html http://www.seedpeer.me/details/6973932/PluralSight-Refactoring-Fundamentals.html http://www.seedpeer.me/details/6661700/Tutsplus---Building-Ribbit-in-Rails.html http://www.seedpeer.me/details/6101172/Tutsplus---Cross-Platform-Browser-Testing-V413HAV.html http://www.seedpeer.me/details/5266314/TutsPlus---Git-Essentials.html http://www.seedpeer.me/details/4848412/TutsPlus---How-to-Be-a-Terminal-Pro.html http://www.seedpeer.me/details/4848374/TutsPlus---How-To-Customize-Your-Terminal.html http://www.seedpeer.me/details/4848299/TutsPlus---Maintainable-CSS-With-Sass-and-Compass.html http://www.seedpeer.me/details/4856068/TutsPlus---Regular-Expressions---Up-and-Running.html http://www.seedpeer.me/details/4816386/TutsPlus---The-Fundamentals-of-Ruby.html http://www.seedpeer.me/details/4848281/TutsPlus---The-Ultimate-Guide-for-Learning-Mootools.html http://www.seedpeer.me/details/4935147/CBT-Nuggets---Intermediate-to-Advanced-Linux-Series.html http://www.seedpeer.me/details/6251428/CBT-Nuggets---IPv6gidbcn.html http://www.seedpeer.me/details/5124174/CBT-Nuggets---LINUX-SERIES.html http://www.seedpeer.me/details/2891954/LinuxCBT-Deb5x-Edition-DVD-YUM.html http://www.seedpeer.me/details/4799921/LinuxCBT---Enterprise-Linux-4-Edition.html http://www.seedpeer.me/details/6290791/LinuxCBT-Network-Intrusion-Detection-System.html http://www.seedpeer.me/details/6107569/LinuxCBT.PackCapAnal.Edition-d3x.html http://www.seedpeer.me/details/6107588/LinuxCBT.PAM.Edition-d3x.html http://www.seedpeer.me/details/6110616/LinuxCBT-Win-Awk-Sed-Edition-d3x.html http://www.seedpeer.me/details/6666824/Packtpub-BackTrack-5-Wireless-Penetration-Testing-[Video].html http://www.seedpeer.me/details/6668649/Packtpub-Getting-started-with-Apache-Solr-Search-Server-[Video].html http://www.seedpeer.me/details/6668652/Packtpub-Getting-Started-with-Citrix-XenApp-6.5-[Video].html http://www.seedpeer.me/details/6668669/Packtpub-Kali-Linux---Backtrack-Evolved-Assuring-Security-by-Penetration-Testing.html http://www.seedpeer.me/details/6415199/Pluralsight-com-Installing-and-Configuring-Apache-Web-Server-iNKiSO.html http://www.seedpeer.me/details/6271468/Pluralsight---MySQL-Indexing-for-Performance-2013.html http://www.seedpeer.me/details/6228283/Pluralsight---Web-Performance-Course.html http://www.seedpeer.me/details/6376899/TutsPlus---Documentation-in-Ruby.html http://www.seedpeer.me/details/5661723/CBT-Nuggets-&amp;acirc;%EF%BF%BD%EF%BF%BD-Cisco-CCENT-CCNA-ICND1-100-101.html http://www.seedpeer.me/details/5825975/CBT-Nuggets-CCNA-200-101-mp4.html http://www.seedpeer.me/details/5513622/CBT-Nuggets---Cisco-CCNA-Security-640-554.html http://www.seedpeer.me/details/5890097/CBT-Nuggets---Citrix-XenApp-6.5.html http://www.seedpeer.me/details/6187994/CBT-Nuggets----CompTIA-A-220-801-&amp;amp;-220-802-Update-2012-iso.html http://www.seedpeer.me/details/6353101/CBT-Nuggets---CompTIA-Security.rar.html http://www.seedpeer.me/details/5243830/CBT-Nuggets---Oracle-Certified-Professional-1Z0-053-OCP.html http://www.seedpeer.me/details/4935122/CBT-Nuggets---Oracle-Database-11g-DBA-1-1Z0-052.html http://www.seedpeer.me/details/7222524/CBT.Nuggets----Oracle.Database.11G.DBA.1Z0-053-EnCod3r.html http://www.seedpeer.me/details/4935128/CBT-Nuggets---Oracle-Database-11g-SQL-Fundamentals-1-1Z0-051.html http://www.seedpeer.me/details/5863952/CBTNuggets-VMware-View-5.iso.html http://www.seedpeer.me/details/6199576/CBT-Nuggets---Web-Development.html http://www.seedpeer.me/details/4825729/LinuxCBT---CentOS6x-Edition.html http://www.seedpeer.me/details/1520287/linuxCBT---DBMS-mysql-5-Training.html http://www.seedpeer.me/details/4799864/LinuxCBT---Deb6x-Edition.html http://www.seedpeer.me/details/4799881/LinuxCBT---Debian-Edition.html http://www.seedpeer.me/details/1548037/LINUXCBT-FEAT-SUSE-10-ENTERPRISE-EDITION-JGTiSO[www.thepeerhub.com].html http://www.seedpeer.me/details/6107551/LinuxCBT-KornShell-Edition-d3x.html http://www.seedpeer.me/details/4261635/Linuxcbt-Redhat-6-Enterprise-Tutorials.html http://www.seedpeer.me/details/1662106/LinuxCBT---RHEL5.html http://www.seedpeer.me/details/6110601/LinuxCBT-SLES-10-Edition-d3x.html http://www.seedpeer.me/details/4799923/LinuxCBT---SLES-11-Edition-SUSE-11-Enterprise.html http://www.seedpeer.me/details/6964916/Lynda---ASP.NET-MVC-4-Essential-Training.html http://www.seedpeer.me/details/7253647/Lynda---Building-Facebook-Applications-with-PHP-and-MySQL.html http://www.seedpeer.me/details/5552857/Lynda.com---Applied-Responsive-Design-Mar,-2013.html http://www.seedpeer.me/details/4657790/Lynda.com-Building-Facebook-Applications-with-HTML-and-JavaScript.html http://www.seedpeer.me/details/4986911/Lynda.com---C&amp;amp;C-Essential-Training.html http://www.seedpeer.me/details/4504272/Lynda.com-Choosing-Using-Web-Fonts.html http://www.seedpeer.me/details/6554622/Lynda.com---Designing-Resume.html http://www.seedpeer.me/details/5332552/Lynda.com---Drupal-7-Advanced-Training---TestOrToast.html http://www.seedpeer.me/details/7051972/Lynda.com---Drupal-7--Creating-and-Editing-Custom-Themes---with-Chaz-Chumley[Isaac-9].html http://www.seedpeer.me/details/5565633/Lynda.com---JavaScript-and-JSON-Mar,-2013.html http://www.seedpeer.me/details/6664728/Lynda.com-JavaScript-for-Web-Designers[2013].html http://www.seedpeer.me/details/6664733/Lynda.com-Node.js-Essential-Training[2013].html http://www.seedpeer.me/details/4591597/Lynda.com---Practical-and-Effective-JavaScript.html http://www.seedpeer.me/details/5256920/Lynda.com-Responsive-Design-with-Joomla--Exercice-Files.html http://www.seedpeer.me/details/5374680/Lynda.com---Simplified-Drupal-Sites-with-Drush---TestOrToast.html http://www.seedpeer.me/details/4795822/Lynda.com---Unix-for-Mac-OS-X-Users.html http://www.seedpeer.me/details/6716808/[Lynda.com]-Up-and-Running-with-Amazon-Web-Services-[2013,-ENG].html http://www.seedpeer.me/details/4593746/Lynda.com-Web-Form-Design-Best-Practices.html http://www.seedpeer.me/details/4850397/Lynda---Create-Your-First-Online-Store-with-Drupal-Commerce.html http://www.seedpeer.me/details/4850389/Lynda---Drupal-7-:-Essential-Training.html http://www.seedpeer.me/details/4850540/Lynda---Drupal-7-New-Features.html http://www.seedpeer.me/details/4850393/Lynda---Drupal-7-:-Reporting-and-Visualizing-Data.html http://www.seedpeer.me/details/5996422/Lynda---Up-and-Running-with-Backbone.js.html http://www.seedpeer.me/details/6971211/Lynda---Up-and-Running-with-CakePHP.html http://www.seedpeer.me/details/6666828/Packtpub-Beginning-Yii-[Video].html http://www.seedpeer.me/details/6666832/Packtpub-Building-a-Website-with-Drupal-[Video].html http://www.seedpeer.me/details/6668107/Packtpub-Drupal-7-Module-Development-[Video].html http://www.seedpeer.me/details/6668679/Packtpub-Learning-Joomla-3-Extension-Development-[Video].html http://www.seedpeer.me/details/7101071/Pluralsight---AngularJS-Fundamentals-[OGNADROL].html http://www.seedpeer.me/details/7268422/[Pluralsight]-AWS-Developer-Fundamentals-[2013,-ENG].html http://www.seedpeer.me/details/6695354/Pluralsight---Beginning-HTML5-Game-Development-With-Quintus.html http://www.seedpeer.me/details/6370939/Pluralsight---Cisco-CCNA-WAN-Technologies---Learn-wide-area-network-WAN-technologies-and-configuration.html http://www.seedpeer.me/details/6383616/Pluralsight-Introduction-to-Spring-MVC2013.html http://www.seedpeer.me/details/6228297/Pluralsight---Introduction-to-the-Facebook-Graph-API.html http://www.seedpeer.me/details/6294391/Pluralsight---Optimizing-and-Managing-Distributed-Systems-on-AWS-2013.html http://www.seedpeer.me/details/6698563/[Pluralsight]-Sublime-Text-3-From-Scratch-[2013,-ENG].html http://www.seedpeer.me/details/5056370/Tutsplus---Advanced-Backbone-Patterns-and-Techniques-2012.html http://www.seedpeer.me/details/7233352/Tutsplus---Become-a-Professional-JavaScript-Developer-Basics.html http://www.seedpeer.me/details/4848277/TutsPlus---Build-Web-Apps-in-Node-and-Express.html http://www.seedpeer.me/details/5683153/Tutsplus---Catch-Up-with-Ruby-on-Rails-4.html http://www.seedpeer.me/details/4918947/TutsPlus---CodeIgniter-Essentials.html http://www.seedpeer.me/details/5069781/TutsPlus---Connected-to-the-Backbone.html http://www.seedpeer.me/details/5513056/Tutsplus---Designing-Professional-Resumes.html http://www.seedpeer.me/details/5706815/Tutsplus-Easier-JavaScript-Apps-with-AngularJS.html http://www.seedpeer.me/details/6462415/TutsPlus---Easier-JavaScript-with-TypeScript.html http://www.seedpeer.me/details/5868293/TutsPlus---Getting-Started-With-Windows-8-Development-Using-HTML,-CSS-&amp;amp;-JavaScript-V413HAV.html http://www.seedpeer.me/details/6150521/TutsPlus-HTML5-Video-Essentials-PRODEV.html http://www.seedpeer.me/details/4841911/TutsPlus---JavaScript-Testing-With-Jasmine.html http://www.seedpeer.me/details/6593486/TutsPlus---Less-is-More.html http://www.seedpeer.me/details/6571637/TutsPlus---Modern-Testing-in-PHP-with-Codeception.html http://www.seedpeer.me/details/6095651/Tutsplus---Parallax-Scrolling-for-Web-Design.html http://www.seedpeer.me/details/6574591/TutsPlus---Say-Yo-to-Yeoman.html http://www.seedpeer.me/details/4811335/Tutsplus---Test-Driven-Development-in-Ruby.html http://www.seedpeer.me/details/6268980/TutsPlus-Test-Driven-Development-With-CoffeeScript-and-Jasmine.html http://www.seedpeer.me/details/6185755/TutsPlus---The-MVC-Mindser-Jeffery-Way---ICARUS.html http://www.seedpeer.me/details/5024493/TutsPlus---Venture-Into-Vim.html http://www.seedpeer.me/details/6286416/Tutsplus---Vim-for-Advanced-Users.html http://www.seedpeer.me/details/6585031/Tutsplus---WordPress-Hackers-Guide-to-the-Galaxy.html http://www.seedpeer.me/details/4848477/TutsPlus---Writing-Modular-JavaScript.html  @giansalex Owner Author giansalex commented on 26 Feb 2018 •  SOLID http://www.allitebooks.com/beginning-solid-principles-and-design-patterns-for-asp-net-developers/  @giansalex Owner Author giansalex commented on 7 Mar 2018 Udemy: AWS Arquitecto de Soluciones Certificado Asociado  https://mega.co.nz/#!ZzhGWSAL!wuthFca0SdJBjmaP5lFX0QF6PeMsrdclKFXlZL1Rsi4 Pass: gratismas.org  @giansalex Owner Author giansalex commented on 7 Mar 2018 Go lang Complete https://www.freetutorials.us/wp-content/uploads/2017/11/FreeTutorials.Us-Udemy-go-the-complete-developers-guide.torrent  @GCPBigData GCPBigData commented on 15 Jul 2018 go books https://drive.google.com/open?id=1d6OsFAn8kpHCXtw0bcoYuyHqrAdGZva0  @freisrael freisrael commented on 14 Aug 2018 giansalex thanks for sharing. I am looking for learning phython with Joe Marini. It would be great if you post it.  @FirstBoy1 FirstBoy1 commented on 25 May 2019 Can anyone provide this book "Getting started with Spring Framework: covers Spring 5" by " J Sharma (Author), Ashish Sarin ". Thanks in advance  @okreka okreka commented on 31 May 2019 Can anyone provide "Windows Presentation Foundation Masterclass" course from Udemy. Thanks in advance  @singhaltanvi singhaltanvi commented on 8 Aug 2019 can anyone provide 'sedimentology and petroleum geology' course from Udemy. Thanks in advance.  @kumarsreenivas051 kumarsreenivas051 commented on 9 Sep 2019 Can anyone provide "Programming languages A,B and C" course from Coursera. Thanks in advance.  @BrunoMoreno BrunoMoreno commented on 11 Sep 2019 The link for the torrents in piratebay, now is .org to the correct url.  @sany2k8 sany2k8 commented on 24 Sep 2019 Can anyone add this The Complete Hands-On Course to Master Apache Airflow  @pharaoh1 pharaoh1 commented on 30 Sep 2019 can you pls add this course to your list https://www.udemy.com/course/advanced-python3/  @SushantDhote936 SushantDhote936 commented on 1 Oct 2019 Can you add Plural Sight CISSP  @allayGerald allayGerald commented on 1 Oct 2019 open directive for lynda courses: https://drive.google.com/drive/folders/1zQan1cq1ZnqXmueRF5IqKoOtpFxl6Y4G  @ezekielskottarathil ezekielskottarathil commented on 3 Oct 2019 can anyone provide 'sedimentology and petroleum geology' course from Udemy. Thanks in advance.  "wrong place boy"  @pulkitd2699 pulkitd2699 commented on 8 Oct 2019 Does anyone has a link for 'Cyber security: Python and web applications' course? Thanks  @mohanrajrc mohanrajrc commented on 19 Oct 2019 •  Can anyone provide torrent file for Mastering React By Mosh Hamedani. Thanks https://codewithmosh.com/p/mastering-react  @evilprince2009 evilprince2009 commented on 27 Oct 2019 Can you please add these two below ? https://codewithmosh.com/p/the-ultimate-java-mastery-series https://codewithmosh.com/p/data-structures-algorithms-part-2  @nunusandio nunusandio commented on 30 Oct 2019 Can anyone post torrent file for ASP.NET Authentication: The Big Picture https://app.pluralsight.com/library/courses/aspdotnet-authentication-big-picture/table-of-contents  @EslamElmadny EslamElmadny commented on 9 Dec 2019 Can you please add these two below ? https://codewithmosh.com/p/the-ultimate-java-mastery-series https://codewithmosh.com/p/data-structures-algorithms-part-2  any luck ?  @Genius-K-SL Genius-K-SL commented on 14 Dec 2019 hay brother! do you have html5 game development with javascript course ?  @Genius-K-SL Genius-K-SL commented on 14 Dec 2019 This link is not working brother! http://www.seedpeer.me/details/4657790/Lynda.com-Building-Facebook-Applications-with-HTML-and-JavaScript.html  @smithtuka smithtuka commented on 20 Dec 2019 Can you please add these two below ? https://codewithmosh.com/p/the-ultimate-java-mastery-series https://codewithmosh.com/p/data-structures-algorithms-part-2  any luck ?  Has this come through by any chances?  @AbdOoSaed AbdOoSaed commented on 22 Dec 2019 Can you please add these two below ? https://codewithmosh.com/p/the-ultimate-java-mastery-series https://codewithmosh.com/p/data-structures-algorithms-part</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>https://github.com/0x00ctrl/CyberSec-Books</t>
+          <t>https://github.com/swati1024/torrents</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -8125,14 +8125,14 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-06-13T00:45:17Z</t>
+          <t>2026-05-17T09:49:47Z</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>swati1024/torrents</t>
+          <t>0x00ctrl/CyberSec-Books</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -8140,12 +8140,12 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Skip to content   Search… All gists Back to GitHub Sign in Sign up Instantly share code, notes, and snippets.  @giansalex giansalex/torrent-courses-download-list.md forked from M-Younus/torrent courses download-list Last active 2 days ago 15188  Code Revisions 15 Stars 151 Forks 88 &lt;script src="https://gist.github.com/giansalex/4cd3631e94433bbbd71bf07aedb33a7b.js"&gt;&lt;/script&gt;     torrent-courses-download-list.md Torrent Courses List Download  http://kickass.to/infiniteskills-learning-jquery-mobile-working-files-t7967156.html http://kickass.to/lynda-bootstrap-3-advanced-web-development-2013-eng-t8167587.html http://kickass.to/lynda-css-advanced-typographic-techniques-t7928210.html http://kickass.to/lynda-html5-projects-interactive-charts-2013-eng-t8167670.html http://kickass.to/vtc-html5-css3-responsive-web-design-course-t7922533.html http://kickass.to/10gen-m101js-mongodb-for-node-js-developers-2013-eng-t8165205.html http://kickass.to/cbt-nuggets-amazon-web-services-aws-foundations-t7839734.html http://kickass.to/cbt-nuggets-apache-hadoop-t8027965.html http://kickass.to/cbt-nuggets-backtrack-and-kali-linux-t7677281.html http://kickass.to/cbt-nuggets-ccda-desgn-640-864-t8300917.html http://kickass.to/cbt-nuggets-ccna-wireless-iuwne-640-722-t8300389.html http://kickass.to/cbt-nuggets-cisco-ccna-labs-cisco-for-the-real-world-bonus-t6154766.html http://kickass.to/cbt-nuggets-cisco-ccnp-security-firewall-v2-0-642-618-azazredhat-t6955696.html http://kickass.to/cbt-nuggets-cisco-ccnp-security-secure-642-637-azazredhat-t6955710.html http://kickass.to/cbt-nuggets-comptia-network-videos-2010-gurufuel-t4648514.html http://kickass.to/cbt-nuggets-definitive-guide-to-working-with-gns3-by-keith-bar-t8301349.html http://kickass.to/cbt-nuggets-ec-council-certified-ethical-hacker-v7-0-t6801120.html http://kickass.to/cbt-nuggets-exam-walkthrough-cisco-icnd1ccent-100-101-t8516719.html http://kickass.to/cbt-nuggets-exam-walkthrough-cisco-icnd2ccna-200-101-t8524803.html http://kickass.to/cbt-nuggets-linux-in-the-real-world-with-shawn-powers-t7718107.html http://kickass.to/cbt-nuggets-linux-series-video-tutorial-t485320.html http://kickass.to/cbt-nuggets-lpi-linux-lpic-1-101-and-comptia-linux-t8031864.html http://kickass.to/cbt-nuggets-lpi-linux-lpic-1-102-and-comptia-linux-t8031871.html http://kickass.to/cbt-nuggets-mastering-vmware-view-5-and-preparing-for-the-vcp510-dt-exam-t8301829.html http://kickass.to/cbt-nuggets-vmware-virtualization-vcp-vsphere-5-t8300512.html http://kickass.to/cbt-nuggets-wireshark-with-keith-barker-t8040855.html http://kickass.to/comptia-network-n10-005-collection-t8319928.html http://kickass.to/developing-in-html5-with-javascript-and-css3-jump-start-t8277565.html http://kickass.to/eli-the-computer-guy-linux-t8647714.html http://kickass.to/foundations-of-programming-test-driven-development-t7522376.html http://kickass.to/infiniteskills-advanced-html5-programming-t7463355.html http://kickass.to/infiniteskills-cisco-ccna-certification-bundle-2013-t7645010.html http://kickass.to/infiniteskills-css3-transformations-and-animations-t7930047.html http://kickass.to/infiniteskills-learning-javascript-programming-t7625039.html http://kickass.to/infiniteskills-learning-python-programming-t7107001.html http://kickass.to/infiniteskills-learning-regular-expressions-t8028765.html http://kickass.to/infiniteskills-learning-whitehat-hacking-and-penetration-testing-t8303725.html http://kickass.to/infiniteskills-microsoft-windows-server-2012-certification-training-exam-70-410-t7379360.html http://kickass.to/infiniteskills-php-security-t8046511.html http://kickass.to/learning-vmware-esxi-and-vsphere-5-1-administration-training-t8030885.html http://kickass.to/linuxcbt-basic-security-edition-d3x-t7650913.html http://kickass.to/linuxcbt-config-mgmt-edition-d3x-t7650929.html http://kickass.to/linuxcbthttpdxil-edition-d3x-t7653897.html http://kickass.to/linuxcbt-vbox-edition-d3x-t7653916.html http://kickass.to/linuxcbt-webscan-edition-d3x-t7653922.html http://kickass.to/linuxcbt-winpython-edition-d3x-t7653942.html http://kickass.to/linuxcbt-xenvm-edition-d3x-t7653948.html http://kickass.to/lynda-com-foundations-of-programming-code-efficiency-t8604312.html http://kickass.to/lynda-com-foundations-of-programming-databases-t8596357.html http://kickass.to/lynda-com-foundations-of-programming-design-patterns-t8692867.html http://kickass.to/lynda-com-foundations-of-programming-fundamentals-t7600288.html http://kickass.to/lynda-com-foundations-of-programming-web-services-including-exercise-files-torrenters-t7797117.html http://kickass.to/lynda-com-ruby-on-rails-4-essential-training-dec-2013-t8438392.html http://kickass.to/lynda-foundations-of-programming-refactoring-code-t7524343.html http://kickass.to/lynda-foundations-of-programming-software-quality-assurance-sum1-here-silverrg-t8043799.html http://kickass.to/lynda-javascript-events-t7893809.html http://kickass.to/lynda-leading-with-emotional-intelligence-t8157240.html http://kickass.to/lynda-management-tips-t8154761.html http://kickass.to/mysql-database-tutorials-by-bucky-thenewboston-org-1-33-t8224550.html http://kickass.to/packtpub-advanced-penetration-testing-for-highly-secured-environments-t8300620.html http://kickass.to/pluralsight-mysql-query-optimization-and-performance-tuning-with-pinal-dave-t8553369.html http://kickass.to/pluralsight-relational-database-design-t8551479.html http://kickass.to/ruby-tutorial-bucky-totally-for-beginner-t8699509.html http://kickass.to/trainsignal-vmware-vcloud-director-5-1-essentials-t7495660.html http://kickass.to/trainsignal-vmware-vsphere-optimize-and-scale-vcap5-dca-t7495659.html http://kickass.to/trainsignal-vmware-workstation-9-for-the-it-admin-t7495658.html http://kickass.to/tutsplus-advanced-command-line-techniques-t7632228.html http://kickass.to/tutsplus-advanced-javascript-fundamentals-t6739742.html http://kickass.to/tutsplus-agile-design-patterns-2012-t6992118.html http://kickass.to/tutsplus-cleaner-code-with-coffeescript-t6741625.html http://kickass.to/tutsplus-detecting-code-smells-t8128341.html http://kickass.to/tutsplus-firebug-white-to-black-belt-v413hav-t7154501.html http://kickass.to/tutsplus-foundational-flask-creating-your-own-static-blog-generator-t8356996.html http://kickass.to/tutsplus-freelance-bootcamp-t6832678.html http://kickass.to/tutsplus-premium-e-book-mega-pack-v413hav-t7178526.html http://kickass.to/tutsplus-pro-workflow-for-web-designers-t6854268.html http://kickass.to/tutsplus-riding-ruby-on-rails-t6728201.html http://kickass.to/tutsplus-sql-essentials-t6746851.html http://kickass.to/tutsplus-tools-of-the-modern-web-developer-t8107617.html http://kickass.to/tutsplus-video-fundamentals-t6752217.html http://kickass.to/ine-ccna-wireless-640-722-iuwne-t8301376.html http://kickass.to/learn-metasploit-t8174472.html http://kickass.to/lynda-ruby-on-rails-essential-training-t7630711.html http://kickass.to/lynda-up-and-running-with-python-2013-eng-t8167709.html http://kickass.to/build-flat-responsive-website-from-scratch-complete-course-t8604527.html http://kickass.to/canvas-essentials-t8550909.html http://kickass.to/cbt-nuggets-70-331-microsoft-sharepoint-server-2013-x264-mkv-encod3r-t8595423.html http://kickass.to/cbt-nuggets-98-365-windows-server-admin-fundamentals-encod3r-t8613009.html http://kickass.to/cbt-nuggets-ccie-combo-pack-t271107.html http://kickass.to/cbt-nuggets-ccna-certification-videos-material-2010-gurufu-t4648321.html http://kickass.to/cbt-nuggets-juniper-networks-certified-specialist-security-jncis-sec-jn0-332-t8028083.html http://kickass.to/cehv7-cbt-nuggets-instructor-slides-tools-video-tools-study-guide-rar-t8705752.html http://kickass.to/cisco-ccna-initial-router-and-switch-configuration-t8648377.html http://kickass.to/cisco-ccna-security-aaa-and-ip-security-t8648378.html http://kickass.to/cisco-ccna-security-introduction-to-network-security-t8648381.html http://kickass.to/cisco-ccna-voice-configuration-and-advanced-features-t8648387.html http://kickass.to/cisco-ccna-voice-voice-overview-and-lab-setup-t8648386.html http://kickass.to/cisco-press-ccna-security-640-554-official-cert-guide-videos-t8648384.html http://kickass.to/coursera-neural-networks-and-machine-learning-geoffrey-hinton-university-of-toronto-t8568642.html http://kickass.to/eli-the-computer-guy-hacking-t8647661.html http://kickass.to/ine-ccie-data-center-storage-t8029396.html http://kickass.to/infinite-skills-learning-cloud-computing-with-amazon-web-services-2013-eng-t8703045.html http://kickass.to/infiniteskills-learning-tcp-ip-t8303739.html http://kickass.to/lynda-bootstrap-3-new-features-and-migration-t7958409.html http://kickass.to/lynda-bootstrap-adding-interactivity-to-your-site-t7519306.html http://kickass.to/lynda-com-jquery-ui-widgets-t8172743.html http://kickass.to/lynda-essential-training-t8157222.html http://kickass.to/lynda-foundation-incorporating-sass-and-compass-t7953037.html http://kickass.to/lynda-html5-projects-advanced-to-do-list-t7855578.html http://kickass.to/lynda-html5-projects-creating-a-responsive-presentation-2013-eng-t8167660.html http://kickass.to/lynda-online-presentations-with-reveal-js-2013-eng-t8167575.html http://kickass.to/lynda-teacher-tips-t8157202.html http://kickass.to/lynda-up-and-running-with-angularjs-t7982840.html http://kickass.to/lynda-up-and-running-with-bootstrap-3-t8011198.html http://kickass.to/lynda-up-and-running-with-cakephp-t7963854.html http://kickass.to/lynda-up-and-running-with-google-apps-script-t7917458.html http://kickass.to/lynda-up-and-running-with-php-codeigniter-t7849968.html http://kickass.to/lynda-web-semantics-t7899223.html http://kickass.to/lynda-wordpress-essential-training-2013-tutorial-t8270624.html http://kickass.to/pluralsight-aws-developer-fundamentals-2013-eng-t8703013.html http://kickass.to/pluralsight-bootstrap-3-t8214168.html http://kickass.to/pluralsight-cisco-ccie-routing-and-switching-implement-bgp-t8648391.html http://kickass.to/pluralsight-cisco-ccna-advanced-ethernet-and-file-management-t8051456.html http://kickass.to/pluralsight-cisco-ccna-security-firewalls-and-vpns-t8648393.html http://kickass.to/pluralsight-cisco-ccna-wan-technologies-learn-wide-area-network-wan-technologies-and-configuration-t7882351.html http://kickass.to/pluralsight-javascript-from-scratch-t7612372.html http://kickass.to/pluralsight-sublime-text-3-from-scratch-2013-eng-t8153034.html http://kickass.to/ten-ton-wordpress-mastery-video-t8452016.html http://kickass.to/trainsignal-microsoft-network-monitoring-t8028791.html http://kickass.to/tuts-plus-2013-bdd-in-rails-psiclone-t8474590.html http://kickass.to/tutsplus-advanced-css3-animations-t7791566.html http://kickass.to/tutsplus-an-introduction-to-node-js-t6744596.html http://kickass.to/tutsplus-better-statistics-with-google-charts-t7983386.html http://kickass.to/tutsplus-bootstrap-for-web-design-t8210956.html http://kickass.to/tutsplus-com-advanced-ui-techniques-2013-t7072722.html http://kickass.to/tutsplus-com-build-a-cms-in-codeigniter-2013-t7072644.html http://kickass.to/tutsplus-com-learning-mongodb-2013-t7072653.html http://kickass.to/tutsplus-computer-networks-distilled-v413hav-t7630795.html http://kickass.to/tutsplus-css-3d-essentials-t8027191.html http://kickass.to/tutsplus-css-noob-to-ninja-v413hav-t7475010.html http://kickass.to/tutsplus-css-tips-and-tricks-t8292119.html http://kickass.to/tutsplus-css3-essentials-t6608214.html http://kickass.to/tutsplus-css3-typography-techniques-t7882076.html http://kickass.to/tutsplus-design-patterns-in-ruby-t8354740.html http://kickass.to/tutsplus-fundamentals-of-design-t6645691.html http://kickass.to/tutsplus-fundamentals-of-print-design-t6667261.html http://kickass.to/tutsplus-fundamentals-of-ux-design-t6710443.html http://kickass.to/tutsplus-html-kickstart-essentials-t7969388.html http://kickass.to/tutsplus-html-tips-and-tricks-t8224648.html http://kickass.to/tutsplus-introduction-to-web-typography-t6662386.html http://kickass.to/tutsplus-javascript-fundamentals-101-t6738976.html http://kickass.to/tutsplus-jquery-ui-101-the-essentials-2013-eng-t8165125.html http://kickass.to/tutsplus-jquery-ui-101-the-essentials-t7791579.html http://kickass.to/tutsplus-jquery-ui-201-beyond-the-basics-t7791583.html http://kickass.to/tutsplus-jquery-ui-301-the-widget-factory-2013-eng-t8165109.html http://kickass.to/tutsplus-jquery-ui-301-the-widget-factory-working-files-2013-eng-t8180547.html http://kickass.to/tutsplus-laravel-essentials-t6722386.html http://kickass.to/tutsplus-logo-design-fundamentals-with-gary-simon-swatiate-t7867377.html http://kickass.to/tutsplus-mastering-corporate-design-v413hav-t7586047.html http://kickass.to/tutsplus-mastering-flat-design-v413hav-t7781777.html http://kickass.to/tutsplus-mastering-retro-web-design-v413hav-t7343186.html http://kickass.to/tutsplus-object-oriented-javascript-t6863065.html http://kickass.to/tutsplus-perfect-workflow-in-sublime-text-2-t6794850.html http://kickass.to/tutsplus-php-fundamentals-t6671312.html http://kickass.to/tutsplus-php-security-pitfalls-t7835091.html http://kickass.to/tutsplus-relational-databases-t8023530.html http://kickass.to/tutsplus-responsive-web-design-for-beginners-v413hav-t7385876.html http://kickass.to/tutsplus-responsive-web-design-techniques-t8103476.html http://kickass.to/tutsplus-responsive-web-design-with-foundation-t8103477.html http://kickass.to/tutsplus-simple-development-with-jquery-mobile-t6735499.html http://kickass.to/tutsplus-solid-design-patterns-t8208974.html http://kickass.to/tutsplus-test-driven-php-in-action-t6851704.html http://kickass.to/tutsplus-testing-tricks-for-php-and-laravel-developers-t7844807.html http://kickass.to/tutsplus-web-form-design-and-development-t8020800.html http://kickass.to/tutsplus-wordpress-plugin-development-essentials-t6615050.html http://kickass.to/udemy-build-an-instantly-updating-dynamic-website-with-jquery-ajax-t8415746.html http://kickass.to/udemy-psd-to-html5-css3-hand-code-a-beautiful-website-in-4-hours-t7740752.html http://kickass.to/video2brain-drupal-power-workshop-t6811365.html http://kickass.to/video2brain-exploring-css-positioning-t6683727.html http://kickass.to/video2brain-getting-started-with-joomla-t6600909.html http://kickass.to/video2brain-html5-for-beginners-learn-by-video-t6686185.html http://kickass.to/video2brain-html5-power-workshop-t6689166.html http://kickass.to/video2brain-php-5-3-advanced-web-application-programming-t6681560.html http://kickass.to/vtc-mysql-5-development-part-1-of-2-t7502575.html http://kickass.to/vtc-mysql-5-development-part-2-of-2-t7502576.html  https://thepiratebay.se/torrent/6113010/Linux_CBT_Scripting_BASH__PERL__PYTHON__PHP https://thepiratebay.se/torrent/7667241/CBT.Nuggets.Python.Programming.Python.Language-PLATO https://thepiratebay.se/torrent/8608894/InfiniteSkills_-_Web_Programming_With_Python https://thepiratebay.se/torrent/7838122/Lynda.com_-_Python_3_Essential_Training https://thepiratebay.se/torrent/7837732/python_book_collection https://thepiratebay.se/torrent/9549614/Pluralsight.com_-_Python_Fundamentals https://thepiratebay.se/torrent/5134755/LiveLessons.Python.Fundamentals.DVDR-HELL https://thepiratebay.se/torrent/7112525/The_New_Boston_-_Python_Programming_Tutorials http://kickass.to/lynda-up-and-running-with-python-2013-eng-t8167709.html  http://www.seedpeer.me/details/5730405/CBT-Nuggets---COMPTIA-SECURITY-SY0-201-WITH-SY0-301,-JK0-018-UPDATES.html http://www.seedpeer.me/details/6411686/CBT.Nuggets----IPv6.html http://www.seedpeer.me/details/6421814/CBT-Nuggets---Ubuntu.html http://www.seedpeer.me/details/6107414/LinuxCBT.Awk.Sed.Edition.html http://www.seedpeer.me/details/6107522/LinuxCBT-BASH-II-Edition-d3x.html http://www.seedpeer.me/details/4799869/LinuxCBT---Berkeley-Packet-Filters-BPF-Edition.html http://www.seedpeer.me/details/6881816/LinuxCBT--HTTPD-Edition.html http://www.seedpeer.me/details/6559038/LinuxCBT-Key-Files-edition.html http://www.seedpeer.me/details/6107600/LinuxCBT.MemCacheD.Edition-d3x.html http://www.seedpeer.me/details/5870507/LinuxCBT-Monitoring-Edition-feat-Nagios.html http://www.seedpeer.me/details/6107677/LinuxCBT-NIDS-Edition-d3x.html http://www.seedpeer.me/details/5925487/LinuxCBT-OpenLDAP-Edition.html http://www.seedpeer.me/details/6107558/LinuxCBT.OpenPGP.Edition-d3x.html http://www.seedpeer.me/details/6107692/LinuxCBT-OpenSSHv2-Edition-d3x.html http://www.seedpeer.me/details/6107699/LinuxCBT-PDNS-Edition-d3x.html http://www.seedpeer.me/details/2595080/LinuxCBT-Proxy-Edition-Feat-Squid-AG-torrent-[twistedtorrents2-com].html http://www.seedpeer.me/details/6110590/LinuxCBT-Samba-Edition-d3x.html http://www.seedpeer.me/details/6110595/LinuxCBT-SELinux-Edition-d3x.html http://www.seedpeer.me/details/4799871/LinuxCBT---SFTP-Edition.html http://www.seedpeer.me/details/6110602/LinuxCBT-SQLite-Edition-d3x.html http://www.seedpeer.me/details/5408265/LinuxCBT---Ubuntu-12.04-LTS.html http://www.seedpeer.me/details/4799857/LinuxCBT---UnixCBT-BSD8x-Edition-FreeBSD-8.2.html http://www.seedpeer.me/details/6110504/LinuxCBT.WinPerl.Edition-d3x.html http://www.seedpeer.me/details/6562861/Lynda-com---CMS-Fundamentals.html http://www.seedpeer.me/details/5247098/Lynda.com---Creating-an-Effective-Resume.html http://www.seedpeer.me/details/4989808/Lynda.com---CSS-with-LESS-and-SASS.html http://www.seedpeer.me/details/5340566/Lynda.com---Fundamentals-of-Software-Version-Control-Nov.-2012.html http://www.seedpeer.me/details/5569955/Lynda.com-GMail-For-Power-Users-V413HAV.html http://www.seedpeer.me/details/4631148/Lynda.com-Invaluable-Becoming-a-Leading-Authority.html http://www.seedpeer.me/details/4631108/Lynda.com-Invaluable-Building-Professional-Connections.html http://www.seedpeer.me/details/4623697/Lynda.com---Managing-a-Hosted-Website.html http://www.seedpeer.me/details/5236946/Lynda.com---PayPal-Essential-Training.html http://www.seedpeer.me/details/4596519/Lynda.com---PostgreSQL-9-With-PHP-Essential-Training-iRONiSO.html http://www.seedpeer.me/details/5016023/Lynda.com---Ruby-Essential-Training-with-Kevin-Skoglund.html http://www.seedpeer.me/details/4931186/Lynda.com---Using-Regular-Expressions.html http://www.seedpeer.me/details/6675342/Lynda---Git-Essential-Training.html http://www.seedpeer.me/details/6698556/Lynda---Leading-Change.html http://www.seedpeer.me/details/6973932/PluralSight-Refactoring-Fundamentals.html http://www.seedpeer.me/details/6661700/Tutsplus---Building-Ribbit-in-Rails.html http://www.seedpeer.me/details/6101172/Tutsplus---Cross-Platform-Browser-Testing-V413HAV.html http://www.seedpeer.me/details/5266314/TutsPlus---Git-Essentials.html http://www.seedpeer.me/details/4848412/TutsPlus---How-to-Be-a-Terminal-Pro.html http://www.seedpeer.me/details/4848374/TutsPlus---How-To-Customize-Your-Terminal.html http://www.seedpeer.me/details/4848299/TutsPlus---Maintainable-CSS-With-Sass-and-Compass.html http://www.seedpeer.me/details/4856068/TutsPlus---Regular-Expressions---Up-and-Running.html http://www.seedpeer.me/details/4816386/TutsPlus---The-Fundamentals-of-Ruby.html http://www.seedpeer.me/details/4848281/TutsPlus---The-Ultimate-Guide-for-Learning-Mootools.html http://www.seedpeer.me/details/4935147/CBT-Nuggets---Intermediate-to-Advanced-Linux-Series.html http://www.seedpeer.me/details/6251428/CBT-Nuggets---IPv6gidbcn.html http://www.seedpeer.me/details/5124174/CBT-Nuggets---LINUX-SERIES.html http://www.seedpeer.me/details/2891954/LinuxCBT-Deb5x-Edition-DVD-YUM.html http://www.seedpeer.me/details/4799921/LinuxCBT---Enterprise-Linux-4-Edition.html http://www.seedpeer.me/details/6290791/LinuxCBT-Network-Intrusion-Detection-System.html http://www.seedpeer.me/details/6107569/LinuxCBT.PackCapAnal.Edition-d3x.html http://www.seedpeer.me/details/6107588/LinuxCBT.PAM.Edition-d3x.html http://www.seedpeer.me/details/6110616/LinuxCBT-Win-Awk-Sed-Edition-d3x.html http://www.seedpeer.me/details/6666824/Packtpub-BackTrack-5-Wireless-Penetration-Testing-[Video].html http://www.seedpeer.me/details/6668649/Packtpub-Getting-started-with-Apache-Solr-Search-Server-[Video].html http://www.seedpeer.me/details/6668652/Packtpub-Getting-Started-with-Citrix-XenApp-6.5-[Video].html http://www.seedpeer.me/details/6668669/Packtpub-Kali-Linux---Backtrack-Evolved-Assuring-Security-by-Penetration-Testing.html http://www.seedpeer.me/details/6415199/Pluralsight-com-Installing-and-Configuring-Apache-Web-Server-iNKiSO.html http://www.seedpeer.me/details/6271468/Pluralsight---MySQL-Indexing-for-Performance-2013.html http://www.seedpeer.me/details/6228283/Pluralsight---Web-Performance-Course.html http://www.seedpeer.me/details/6376899/TutsPlus---Documentation-in-Ruby.html http://www.seedpeer.me/details/5661723/CBT-Nuggets-&amp;acirc;%EF%BF%BD%EF%BF%BD-Cisco-CCENT-CCNA-ICND1-100-101.html http://www.seedpeer.me/details/5825975/CBT-Nuggets-CCNA-200-101-mp4.html http://www.seedpeer.me/details/5513622/CBT-Nuggets---Cisco-CCNA-Security-640-554.html http://www.seedpeer.me/details/5890097/CBT-Nuggets---Citrix-XenApp-6.5.html http://www.seedpeer.me/details/6187994/CBT-Nuggets----CompTIA-A-220-801-&amp;amp;-220-802-Update-2012-iso.html http://www.seedpeer.me/details/6353101/CBT-Nuggets---CompTIA-Security.rar.html http://www.seedpeer.me/details/5243830/CBT-Nuggets---Oracle-Certified-Professional-1Z0-053-OCP.html http://www.seedpeer.me/details/4935122/CBT-Nuggets---Oracle-Database-11g-DBA-1-1Z0-052.html http://www.seedpeer.me/details/7222524/CBT.Nuggets----Oracle.Database.11G.DBA.1Z0-053-EnCod3r.html http://www.seedpeer.me/details/4935128/CBT-Nuggets---Oracle-Database-11g-SQL-Fundamentals-1-1Z0-051.html http://www.seedpeer.me/details/5863952/CBTNuggets-VMware-View-5.iso.html http://www.seedpeer.me/details/6199576/CBT-Nuggets---Web-Development.html http://www.seedpeer.me/details/4825729/LinuxCBT---CentOS6x-Edition.html http://www.seedpeer.me/details/1520287/linuxCBT---DBMS-mysql-5-Training.html http://www.seedpeer.me/details/4799864/LinuxCBT---Deb6x-Edition.html http://www.seedpeer.me/details/4799881/LinuxCBT---Debian-Edition.html http://www.seedpeer.me/details/1548037/LINUXCBT-FEAT-SUSE-10-ENTERPRISE-EDITION-JGTiSO[www.thepeerhub.com].html http://www.seedpeer.me/details/6107551/LinuxCBT-KornShell-Edition-d3x.html http://www.seedpeer.me/details/4261635/Linuxcbt-Redhat-6-Enterprise-Tutorials.html http://www.seedpeer.me/details/1662106/LinuxCBT---RHEL5.html http://www.seedpeer.me/details/6110601/LinuxCBT-SLES-10-Edition-d3x.html http://www.seedpeer.me/details/4799923/LinuxCBT---SLES-11-Edition-SUSE-11-Enterprise.html http://www.seedpeer.me/details/6964916/Lynda---ASP.NET-MVC-4-Essential-Training.html http://www.seedpeer.me/details/7253647/Lynda---Building-Facebook-Applications-with-PHP-and-MySQL.html http://www.seedpeer.me/details/5552857/Lynda.com---Applied-Responsive-Design-Mar,-2013.html http://www.seedpeer.me/details/4657790/Lynda.com-Building-Facebook-Applications-with-HTML-and-JavaScript.html http://www.seedpeer.me/details/4986911/Lynda.com---C&amp;amp;C-Essential-Training.html http://www.seedpeer.me/details/4504272/Lynda.com-Choosing-Using-Web-Fonts.html http://www.seedpeer.me/details/6554622/Lynda.com---Designing-Resume.html http://www.seedpeer.me/details/5332552/Lynda.com---Drupal-7-Advanced-Training---TestOrToast.html http://www.seedpeer.me/details/7051972/Lynda.com---Drupal-7--Creating-and-Editing-Custom-Themes---with-Chaz-Chumley[Isaac-9].html http://www.seedpeer.me/details/5565633/Lynda.com---JavaScript-and-JSON-Mar,-2013.html http://www.seedpeer.me/details/6664728/Lynda.com-JavaScript-for-Web-Designers[2013].html http://www.seedpeer.me/details/6664733/Lynda.com-Node.js-Essential-Training[2013].html http://www.seedpeer.me/details/4591597/Lynda.com---Practical-and-Effective-JavaScript.html http://www.seedpeer.me/details/5256920/Lynda.com-Responsive-Design-with-Joomla--Exercice-Files.html http://www.seedpeer.me/details/5374680/Lynda.com---Simplified-Drupal-Sites-with-Drush---TestOrToast.html http://www.seedpeer.me/details/4795822/Lynda.com---Unix-for-Mac-OS-X-Users.html http://www.seedpeer.me/details/6716808/[Lynda.com]-Up-and-Running-with-Amazon-Web-Services-[2013,-ENG].html http://www.seedpeer.me/details/4593746/Lynda.com-Web-Form-Design-Best-Practices.html http://www.seedpeer.me/details/4850397/Lynda---Create-Your-First-Online-Store-with-Drupal-Commerce.html http://www.seedpeer.me/details/4850389/Lynda---Drupal-7-:-Essential-Training.html http://www.seedpeer.me/details/4850540/Lynda---Drupal-7-New-Features.html http://www.seedpeer.me/details/4850393/Lynda---Drupal-7-:-Reporting-and-Visualizing-Data.html http://www.seedpeer.me/details/5996422/Lynda---Up-and-Running-with-Backbone.js.html http://www.seedpeer.me/details/6971211/Lynda---Up-and-Running-with-CakePHP.html http://www.seedpeer.me/details/6666828/Packtpub-Beginning-Yii-[Video].html http://www.seedpeer.me/details/6666832/Packtpub-Building-a-Website-with-Drupal-[Video].html http://www.seedpeer.me/details/6668107/Packtpub-Drupal-7-Module-Development-[Video].html http://www.seedpeer.me/details/6668679/Packtpub-Learning-Joomla-3-Extension-Development-[Video].html http://www.seedpeer.me/details/7101071/Pluralsight---AngularJS-Fundamentals-[OGNADROL].html http://www.seedpeer.me/details/7268422/[Pluralsight]-AWS-Developer-Fundamentals-[2013,-ENG].html http://www.seedpeer.me/details/6695354/Pluralsight---Beginning-HTML5-Game-Development-With-Quintus.html http://www.seedpeer.me/details/6370939/Pluralsight---Cisco-CCNA-WAN-Technologies---Learn-wide-area-network-WAN-technologies-and-configuration.html http://www.seedpeer.me/details/6383616/Pluralsight-Introduction-to-Spring-MVC2013.html http://www.seedpeer.me/details/6228297/Pluralsight---Introduction-to-the-Facebook-Graph-API.html http://www.seedpeer.me/details/6294391/Pluralsight---Optimizing-and-Managing-Distributed-Systems-on-AWS-2013.html http://www.seedpeer.me/details/6698563/[Pluralsight]-Sublime-Text-3-From-Scratch-[2013,-ENG].html http://www.seedpeer.me/details/5056370/Tutsplus---Advanced-Backbone-Patterns-and-Techniques-2012.html http://www.seedpeer.me/details/7233352/Tutsplus---Become-a-Professional-JavaScript-Developer-Basics.html http://www.seedpeer.me/details/4848277/TutsPlus---Build-Web-Apps-in-Node-and-Express.html http://www.seedpeer.me/details/5683153/Tutsplus---Catch-Up-with-Ruby-on-Rails-4.html http://www.seedpeer.me/details/4918947/TutsPlus---CodeIgniter-Essentials.html http://www.seedpeer.me/details/5069781/TutsPlus---Connected-to-the-Backbone.html http://www.seedpeer.me/details/5513056/Tutsplus---Designing-Professional-Resumes.html http://www.seedpeer.me/details/5706815/Tutsplus-Easier-JavaScript-Apps-with-AngularJS.html http://www.seedpeer.me/details/6462415/TutsPlus---Easier-JavaScript-with-TypeScript.html http://www.seedpeer.me/details/5868293/TutsPlus---Getting-Started-With-Windows-8-Development-Using-HTML,-CSS-&amp;amp;-JavaScript-V413HAV.html http://www.seedpeer.me/details/6150521/TutsPlus-HTML5-Video-Essentials-PRODEV.html http://www.seedpeer.me/details/4841911/TutsPlus---JavaScript-Testing-With-Jasmine.html http://www.seedpeer.me/details/6593486/TutsPlus---Less-is-More.html http://www.seedpeer.me/details/6571637/TutsPlus---Modern-Testing-in-PHP-with-Codeception.html http://www.seedpeer.me/details/6095651/Tutsplus---Parallax-Scrolling-for-Web-Design.html http://www.seedpeer.me/details/6574591/TutsPlus---Say-Yo-to-Yeoman.html http://www.seedpeer.me/details/4811335/Tutsplus---Test-Driven-Development-in-Ruby.html http://www.seedpeer.me/details/6268980/TutsPlus-Test-Driven-Development-With-CoffeeScript-and-Jasmine.html http://www.seedpeer.me/details/6185755/TutsPlus---The-MVC-Mindser-Jeffery-Way---ICARUS.html http://www.seedpeer.me/details/5024493/TutsPlus---Venture-Into-Vim.html http://www.seedpeer.me/details/6286416/Tutsplus---Vim-for-Advanced-Users.html http://www.seedpeer.me/details/6585031/Tutsplus---WordPress-Hackers-Guide-to-the-Galaxy.html http://www.seedpeer.me/details/4848477/TutsPlus---Writing-Modular-JavaScript.html  @giansalex Owner Author giansalex commented on 26 Feb 2018 •  SOLID http://www.allitebooks.com/beginning-solid-principles-and-design-patterns-for-asp-net-developers/  @giansalex Owner Author giansalex commented on 7 Mar 2018 Udemy: AWS Arquitecto de Soluciones Certificado Asociado  https://mega.co.nz/#!ZzhGWSAL!wuthFca0SdJBjmaP5lFX0QF6PeMsrdclKFXlZL1Rsi4 Pass: gratismas.org  @giansalex Owner Author giansalex commented on 7 Mar 2018 Go lang Complete https://www.freetutorials.us/wp-content/uploads/2017/11/FreeTutorials.Us-Udemy-go-the-complete-developers-guide.torrent  @GCPBigData GCPBigData commented on 15 Jul 2018 go books https://drive.google.com/open?id=1d6OsFAn8kpHCXtw0bcoYuyHqrAdGZva0  @freisrael freisrael commented on 14 Aug 2018 giansalex thanks for sharing. I am looking for learning phython with Joe Marini. It would be great if you post it.  @FirstBoy1 FirstBoy1 commented on 25 May 2019 Can anyone provide this book "Getting started with Spring Framework: covers Spring 5" by " J Sharma (Author), Ashish Sarin ". Thanks in advance  @okreka okreka commented on 31 May 2019 Can anyone provide "Windows Presentation Foundation Masterclass" course from Udemy. Thanks in advance  @singhaltanvi singhaltanvi commented on 8 Aug 2019 can anyone provide 'sedimentology and petroleum geology' course from Udemy. Thanks in advance.  @kumarsreenivas051 kumarsreenivas051 commented on 9 Sep 2019 Can anyone provide "Programming languages A,B and C" course from Coursera. Thanks in advance.  @BrunoMoreno BrunoMoreno commented on 11 Sep 2019 The link for the torrents in piratebay, now is .org to the correct url.  @sany2k8 sany2k8 commented on 24 Sep 2019 Can anyone add this The Complete Hands-On Course to Master Apache Airflow  @pharaoh1 pharaoh1 commented on 30 Sep 2019 can you pls add this course to your list https://www.udemy.com/course/advanced-python3/  @SushantDhote936 SushantDhote936 commented on 1 Oct 2019 Can you add Plural Sight CISSP  @allayGerald allayGerald commented on 1 Oct 2019 open directive for lynda courses: https://drive.google.com/drive/folders/1zQan1cq1ZnqXmueRF5IqKoOtpFxl6Y4G  @ezekielskottarathil ezekielskottarathil commented on 3 Oct 2019 can anyone provide 'sedimentology and petroleum geology' course from Udemy. Thanks in advance.  "wrong place boy"  @pulkitd2699 pulkitd2699 commented on 8 Oct 2019 Does anyone has a link for 'Cyber security: Python and web applications' course? Thanks  @mohanrajrc mohanrajrc commented on 19 Oct 2019 •  Can anyone provide torrent file for Mastering React By Mosh Hamedani. Thanks https://codewithmosh.com/p/mastering-react  @evilprince2009 evilprince2009 commented on 27 Oct 2019 Can you please add these two below ? https://codewithmosh.com/p/the-ultimate-java-mastery-series https://codewithmosh.com/p/data-structures-algorithms-part-2  @nunusandio nunusandio commented on 30 Oct 2019 Can anyone post torrent file for ASP.NET Authentication: The Big Picture https://app.pluralsight.com/library/courses/aspdotnet-authentication-big-picture/table-of-contents  @EslamElmadny EslamElmadny commented on 9 Dec 2019 Can you please add these two below ? https://codewithmosh.com/p/the-ultimate-java-mastery-series https://codewithmosh.com/p/data-structures-algorithms-part-2  any luck ?  @Genius-K-SL Genius-K-SL commented on 14 Dec 2019 hay brother! do you have html5 game development with javascript course ?  @Genius-K-SL Genius-K-SL commented on 14 Dec 2019 This link is not working brother! http://www.seedpeer.me/details/4657790/Lynda.com-Building-Facebook-Applications-with-HTML-and-JavaScript.html  @smithtuka smithtuka commented on 20 Dec 2019 Can you please add these two below ? https://codewithmosh.com/p/the-ultimate-java-mastery-series https://codewithmosh.com/p/data-structures-algorithms-part-2  any luck ?  Has this come through by any chances?  @AbdOoSaed AbdOoSaed commented on 22 Dec 2019 Can you please add these two below ? https://codewithmosh.com/p/the-ultimate-java-mastery-series https://codewithmosh.com/p/data-structures-algorithms-part</t>
+          <t>Some useful books related to Cybersecurity, Linux and more.</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>https://github.com/swati1024/torrents</t>
+          <t>https://github.com/0x00ctrl/CyberSec-Books</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>2026-05-17T09:49:47Z</t>
+          <t>2026-06-13T00:45:17Z</t>
         </is>
       </c>
     </row>
@@ -8192,7 +8192,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>BugBountyResources/Resources</t>
+          <t>jassics/awesome-cybersecurity-learning-resources</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -8200,12 +8200,12 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>A Storehouse of resources related to Bug Bounty Hunting collected from different sources. Latest guides, tools, methodology, platforms tips, and tricks curated by us.</t>
+          <t>Learning resources for cybersecurity including youtube, github, books, videos, courses, labs, articles etc. at one place</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>https://github.com/BugBountyResources/Resources</t>
+          <t>https://github.com/jassics/awesome-cybersecurity-learning-resources</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -8215,14 +8215,14 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>2026-05-08T11:48:50Z</t>
+          <t>2026-06-11T08:54:42Z</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>jassics/awesome-cybersecurity-learning-resources</t>
+          <t>BugBountyResources/Resources</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -8230,12 +8230,12 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Learning resources for cybersecurity including youtube, github, books, videos, courses, labs, articles etc. at one place</t>
+          <t>A Storehouse of resources related to Bug Bounty Hunting collected from different sources. Latest guides, tools, methodology, platforms tips, and tricks curated by us.</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>https://github.com/jassics/awesome-cybersecurity-learning-resources</t>
+          <t>https://github.com/BugBountyResources/Resources</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>2026-06-11T08:54:42Z</t>
+          <t>2026-05-08T11:48:50Z</t>
         </is>
       </c>
     </row>
@@ -8312,7 +8312,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>bL34cHig0/Pentest-Resources-Cheat-Sheets</t>
+          <t>Mr6MJT/LearnForFREE</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -8320,12 +8320,12 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>This repository contains a curated list of websites and repositories featuring pentest &amp; red-team resources such as cheatsheets, write-ups, tools, techniques, programming/scripting notes, and more. I documented them in this repo to provide like-minded offensive security enthusiasts and professionals easy access to these valuable resources.</t>
+          <t>These are some books that will help you in your learning,I got them in my cyber security career, These books for: pentesting, programming, networking, crypto, reverse engineering, web hacking...</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>https://github.com/bL34cHig0/Pentest-Resources-Cheat-Sheets</t>
+          <t>https://github.com/Mr6MJT/LearnForFREE</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -8335,14 +8335,14 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>2026-06-12T12:53:13Z</t>
+          <t>2026-05-13T18:20:18Z</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Mr6MJT/LearnForFREE</t>
+          <t>bL34cHig0/Pentest-Resources-Cheat-Sheets</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -8350,12 +8350,12 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>These are some books that will help you in your learning,I got them in my cyber security career, These books for: pentesting, programming, networking, crypto, reverse engineering, web hacking...</t>
+          <t>This repository contains a curated list of websites and repositories featuring pentest &amp; red-team resources such as cheatsheets, write-ups, tools, techniques, programming/scripting notes, and more. I documented them in this repo to provide like-minded offensive security enthusiasts and professionals easy access to these valuable resources.</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>https://github.com/Mr6MJT/LearnForFREE</t>
+          <t>https://github.com/bL34cHig0/Pentest-Resources-Cheat-Sheets</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-05-13T18:20:18Z</t>
+          <t>2026-06-12T12:53:13Z</t>
         </is>
       </c>
     </row>
@@ -8672,7 +8672,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>shabarkin/CodeAllTheThings</t>
+          <t>s0cm0nkey/Security-Reference-Guide</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -8680,29 +8680,29 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>A list of threat sinks used in the manual security source code review for application security</t>
+          <t>Curated cyber security resources for blue team, red team, DFIR, OSINT, AppSec, cloud security, security logging, and training.</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>https://github.com/shabarkin/CodeAllTheThings</t>
+          <t>https://github.com/s0cm0nkey/Security-Reference-Guide</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>HTML</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>2026-01-22T03:00:56Z</t>
+          <t>2026-06-10T08:25:34Z</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>s0cm0nkey/Security-Reference-Guide</t>
+          <t>shabarkin/CodeAllTheThings</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -8710,22 +8710,22 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Curated cyber security resources for blue team, red team, DFIR, OSINT, AppSec, cloud security, security logging, and training.</t>
+          <t>A list of threat sinks used in the manual security source code review for application security</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>https://github.com/s0cm0nkey/Security-Reference-Guide</t>
+          <t>https://github.com/shabarkin/CodeAllTheThings</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>2026-06-10T08:25:34Z</t>
+          <t>2026-01-22T03:00:56Z</t>
         </is>
       </c>
     </row>
@@ -8762,7 +8762,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>alparslanakyildiz/ChapterZero</t>
+          <t>mizazhaider-ceh/Security-Books</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -8770,12 +8770,12 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Welcome! I'm Alparslan Akyıldız, an author focusing on cybersecurity and technology. Explore my guides, books, and texts designed to simplify complex topics and make cybersecurity accessible for all. Happy reading!</t>
+          <t xml:space="preserve">🛡️ The Ultimate Cybersecurity Library | 160+ curated books, guides &amp; resources covering Ethical Hacking, Penetration Testing, Bug Bounty, Red/Blue Team, OSINT, Malware Analysis, CEH, OSCP, CISSP, CHFI, Network Security, Kali Linux, Web Security &amp; more. Free, organized, and clickable. Knowledge should be accessible to everyone. </t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>https://github.com/alparslanakyildiz/ChapterZero</t>
+          <t>https://github.com/mizazhaider-ceh/Security-Books</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -8785,14 +8785,14 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>2025-12-16T10:14:33Z</t>
+          <t>2026-06-13T15:28:29Z</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>mizazhaider-ceh/Security-Books</t>
+          <t>alparslanakyildiz/ChapterZero</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -8800,12 +8800,12 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t xml:space="preserve">🛡️ The Ultimate Cybersecurity Library | 160+ curated books, guides &amp; resources covering Ethical Hacking, Penetration Testing, Bug Bounty, Red/Blue Team, OSINT, Malware Analysis, CEH, OSCP, CISSP, CHFI, Network Security, Kali Linux, Web Security &amp; more. Free, organized, and clickable. Knowledge should be accessible to everyone. </t>
+          <t>Welcome! I'm Alparslan Akyıldız, an author focusing on cybersecurity and technology. Explore my guides, books, and texts designed to simplify complex topics and make cybersecurity accessible for all. Happy reading!</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>https://github.com/mizazhaider-ceh/Security-Books</t>
+          <t>https://github.com/alparslanakyildiz/ChapterZero</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -8815,7 +8815,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>2026-06-13T15:28:29Z</t>
+          <t>2025-12-16T10:14:33Z</t>
         </is>
       </c>
     </row>
@@ -8852,7 +8852,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Sh0ckFR/Infosec-Useful-Stuff</t>
+          <t>paulveillard/cybersecurity-build-your-own-x</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -8860,12 +8860,12 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>This repository is my own list of tools / useful stuff for pentest, defensive activities, programming, lockpicking and physical security</t>
+          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about building your own x in security.</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>https://github.com/Sh0ckFR/Infosec-Useful-Stuff</t>
+          <t>https://github.com/paulveillard/cybersecurity-build-your-own-x</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -8875,14 +8875,14 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>2026-06-08T16:20:35Z</t>
+          <t>2026-06-04T09:58:51Z</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-build-your-own-x</t>
+          <t>Sh0ckFR/Infosec-Useful-Stuff</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -8890,12 +8890,12 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about building your own x in security.</t>
+          <t>This repository is my own list of tools / useful stuff for pentest, defensive activities, programming, lockpicking and physical security</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-build-your-own-x</t>
+          <t>https://github.com/Sh0ckFR/Infosec-Useful-Stuff</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -8905,14 +8905,14 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>2026-06-04T09:58:51Z</t>
+          <t>2026-06-08T16:20:35Z</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-malware-analysis</t>
+          <t>cyver-core/ultimate-pentest-tools-list</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -8920,12 +8920,12 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>A collection of Malware Analysis software, materials, libraries, documents, books, resources  about malware analysis in Cybersecurity.</t>
+          <t xml:space="preserve">The following include a list of pentest tools available across the web. Many are free and even open source, others are premium tools and require a monthly or yearly subscription. We’ll note when pentest tools aren’t free. </t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-malware-analysis</t>
+          <t>https://github.com/cyver-core/ultimate-pentest-tools-list</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -8935,14 +8935,14 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>2026-06-09T23:54:08Z</t>
+          <t>2026-06-06T01:24:53Z</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>cyver-core/ultimate-pentest-tools-list</t>
+          <t>paulveillard/cybersecurity-malware-analysis</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -8950,12 +8950,12 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t xml:space="preserve">The following include a list of pentest tools available across the web. Many are free and even open source, others are premium tools and require a monthly or yearly subscription. We’ll note when pentest tools aren’t free. </t>
+          <t>A collection of Malware Analysis software, materials, libraries, documents, books, resources  about malware analysis in Cybersecurity.</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>https://github.com/cyver-core/ultimate-pentest-tools-list</t>
+          <t>https://github.com/paulveillard/cybersecurity-malware-analysis</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -8965,14 +8965,14 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>2026-06-06T01:24:53Z</t>
+          <t>2026-06-09T23:54:08Z</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-infosec</t>
+          <t>archanchoudhury/Davy-Jones-Locker</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -8980,29 +8980,29 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Information Security in Cybersecurity.</t>
+          <t>Getting FREE Cyber Security Resources have been a challenge always. Access Davy-Jones-Locker to get all what you might need to upskill yourself and create an impact in the InfoSec Community</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-infosec</t>
+          <t>https://github.com/archanchoudhury/Davy-Jones-Locker</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>2026-06-06T00:04:26Z</t>
+          <t>2026-01-05T06:02:30Z</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>archanchoudhury/Davy-Jones-Locker</t>
+          <t>paulveillard/cybersecurity-infosec</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -9010,22 +9010,22 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Getting FREE Cyber Security Resources have been a challenge always. Access Davy-Jones-Locker to get all what you might need to upskill yourself and create an impact in the InfoSec Community</t>
+          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Information Security in Cybersecurity.</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>https://github.com/archanchoudhury/Davy-Jones-Locker</t>
+          <t>https://github.com/paulveillard/cybersecurity-infosec</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>2026-01-05T06:02:30Z</t>
+          <t>2026-06-06T00:04:26Z</t>
         </is>
       </c>
     </row>
@@ -9392,7 +9392,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>glaucusec/awesome-repos</t>
+          <t>paulveillard/cybersecurity-threat-detection</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -9400,12 +9400,12 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Repositories, Links, Payloads, Blogs, Tools, etc.. which I think might be useful for pentesting and bug bounty</t>
+          <t>An ongoing &amp; curated collection of awesome software best practices and remediation techniques, libraries and frameworks, E-books and videos, Technical guidelines and important resources about Threat Detection &amp; Hunting.</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>https://github.com/glaucusec/awesome-repos</t>
+          <t>https://github.com/paulveillard/cybersecurity-threat-detection</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9415,7 +9415,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>2026-04-01T16:34:54Z</t>
+          <t>2026-05-18T03:20:40Z</t>
         </is>
       </c>
     </row>
@@ -9482,7 +9482,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-threat-detection</t>
+          <t>glaucusec/awesome-repos</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -9490,12 +9490,12 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>An ongoing &amp; curated collection of awesome software best practices and remediation techniques, libraries and frameworks, E-books and videos, Technical guidelines and important resources about Threat Detection &amp; Hunting.</t>
+          <t>Repositories, Links, Payloads, Blogs, Tools, etc.. which I think might be useful for pentesting and bug bounty</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-threat-detection</t>
+          <t>https://github.com/glaucusec/awesome-repos</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -9505,14 +9505,14 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>2026-05-18T03:20:40Z</t>
+          <t>2026-04-01T16:34:54Z</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>andripwn/PayloadsAll</t>
+          <t>Reconnaishawnce/Red-Team</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -9520,22 +9520,22 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>A list of useful payloads and bypass for Web Application Security and Pentest/CTF</t>
+          <t>Tools and Resources for Physical Security Red Teaming</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>https://github.com/andripwn/PayloadsAll</t>
+          <t>https://github.com/Reconnaishawnce/Red-Team</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>2026-02-28T22:44:21Z</t>
+          <t>2026-06-10T20:35:34Z</t>
         </is>
       </c>
     </row>
@@ -9572,7 +9572,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Reconnaishawnce/Red-Team</t>
+          <t>andripwn/PayloadsAll</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -9580,22 +9580,22 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Tools and Resources for Physical Security Red Teaming</t>
+          <t>A list of useful payloads and bypass for Web Application Security and Pentest/CTF</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>https://github.com/Reconnaishawnce/Red-Team</t>
+          <t>https://github.com/andripwn/PayloadsAll</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>HTML</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>2026-06-10T20:35:34Z</t>
+          <t>2026-02-28T22:44:21Z</t>
         </is>
       </c>
     </row>
@@ -9722,7 +9722,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-bug-bounty</t>
+          <t>BabyJ723/blast-ON</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -9730,29 +9730,29 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Bug Bounty in Cybersecurity.</t>
+          <t># Awesome Keycloak [![Awesome](https://cdn.rawgit.com/sindresorhus/awesome/d7305f38d29fed78fa85652e3a63e154dd8e8829/media/badge.svg)](https://github.com/sindresorhus/awesome)  # [&lt;img src="https://www.keycloak.org/resources/images/keycloak_logo_480x108.png"&gt;](https://github.com/thomasdarimont/awesome-keycloak)  &gt; Carefully curated list of awesome Keycloak resources.  A curated list of resources for learning about the Open Source Identity and Access Management solution Keycloak.  Contains books, websites, blog posts, links to github Repositories.    # Contributing Contributions welcome. Add links through pull requests or create an issue to start a discussion. [Please refer to the contributing guide for details](CONTRIBUTING.md).  # Contents  * [General](#general)   * [Documentation](#docs)     * [Keycloak Website](http://www.keycloak.org)     * [Current Documentation](http://www.keycloak.org/documentation.html)     * [Archived Documentation](http://www.keycloak.org/documentation-archive.html)   * [Mailing Lists](#mailing-lists)     * [User Mailing List](#user-mailing-list)     * [Developer Mailing List](#dev-mailing-list)     * [Mailing List Search](#mailing-list-search) * [Books](#books) * [Articles](#articles) * [Talks](#talks) * [Presentations](#presentations) * [Video Playlists](#video-playlists) * [Community Extensions](#community-extensions) * [Integrations](#integrations) * [Themes](#themes) * [Docker](#docker) * [Deployment Examples](#deployment-examples) * [Example Projects](#example-projects) * [Benchmarks](#benchmarks) * [Help](#help) * [Commercial Offerings](#commercial-offerings) * [Miscellaneous](#miscellaneous)  # General  ## Documentation  *  [Keycloak Website](http://www.keycloak.org/) *  [Current Documentation](http://www.keycloak.org/documentation.html) *  [Archived Documentation](http://www.keycloak.org/documentation-archive.html) *  [Product Documentation for Red Hat Single Sign-On](https://access.redhat.com/documentation/en/red-hat-single-sign-on/)  ## Discussion Groups and Mailing Lists *  [Keycloak Users Google Group](https://groups.google.com/forum/#!forum/keycloak-user) *  [Keycloak Developers Google Group](https://groups.google.com/forum/#!forum/keycloak-dev) *  [Keycloak Discourse Group](https://keycloak.discourse.group/) *  [Keycloak Developer Chat](https://keycloak.zulipchat.com) *  [Inactive - User Mailing List](https://lists.jboss.org/mailman/listinfo/keycloak-user) *  [Inactive - Developer Mailing List](https://lists.jboss.org/mailman/listinfo/keycloak-dev) *  [Mailing List Search](http://www.keycloak.org/search) *  [Keycloak Subreddit](https://www.reddit.com/r/keycloak)  ## Books * [Keycloak - Identity and Access Management for Modern Applications](https://www.packtpub.com/product/keycloak-identity-and-access-management-for-modern-applications/9781800562493)  ## Articles *  [How to get Keycloak working with Docker](https://www.ivonet.nl/2015/05/23/Keycloak-Docker/) *  [Single-Sign-On for Microservices and/or Java EE applications with Keycloak SSO](http://www.n-k.de/2016/06/keycloak-sso-for-microservices.html) *  [Keycloak Admin Client(s) - multiple ways to manage your SSO system](http://www.n-k.de/2016/08/keycloak-admin-client.html) *  [How to get the AccessToken of Keycloak in Spring Boot and/or Java EE](http://www.n-k.de/2016/05/how-to-get-accesstoken-from-keycloak-springboot-javaee.html) *  [JWT authentication with Vert.x, Keycloak and Angular 2](http://paulbakker.io/java/jwt-keycloak-angular2/) *  [Authenticating via Kerberos with Keycloak and Windows 2008 Active Directory](http://matthewcasperson.blogspot.de/2015/07/authenticating-via-kerberos-with.html) *  [Deploying Keycloak with Ansible](https://adam.younglogic.com/2016/01/deploying-keycloak-via-ansible/) *  [Easily secure your Spring Boot applications with Keycloak](https://developers.redhat.com/blog/2017/05/25/easily-secure-your-spring-boot-applications-with-keycloak/) *  [How Red Hat re-designed its Single Sign On (SSO) architecture, and why](https://developers.redhat.com/blog/2016/10/04/how-red-hat-re-designed-its-single-sign-on-sso-architecture-and-why/) *  [OAuth2, JWT, Open-ID Connect and other confusing things](http://giallone.blogspot.de/2017/06/oath2.html) *  [X509 Authentication with Keycloak and JBoss Fuse](https://sjhiggs.github.io/fuse/sso/x509/smartcard/2017/03/29/fuse-hawtio-keycloak.html) *  [Running Keycloak on OpenShift 3](https://medium.com/@sbose78/running-keycloak-on-openshift-3-8d195c0daaf6) *  [Introducing Keycloak for Identity and Access Management](https://www.thomasvitale.com/introducing-keycloak-identity-access-management/) *  [Keycloak Basic Configuration for Authentication and Authorisation](https://www.thomasvitale.com/keycloak-configuration-authentication-authorisation/) *  [Keycloak on OpenShift Origin](https://medium.com/@james_devcomb/keycloak-on-openshift-origin-ee81d01dac97) *  [Identity Management, One-Time-Passwords and Two-Factor-Auth with Spring Boot and Keycloak](http://www.hascode.com/2017/11/identity-management-one-time-passwords-and-two-factor-auth-with-spring-boot-and-keycloak/) *  [Keycloak Identity Brokering with Openshift](https://developers.redhat.com/blog/2017/12/06/keycloak-identity-brokering-openshift/) *  [OpenID Connect Identity Brokering with Red Hat Single Sign-On](https://developers.redhat.com/blog/2017/10/18/openid-connect-identity-brokering-red-hat-single-sign/) *  [Authentication &amp; user management is hard](https://eclipsesource.com/blogs/2018/01/11/authenticating-reverse-proxy-with-keycloak/) *  [Securing Nginx with Keycloak](https://edhull.co.uk/blog/2018-06-06/keycloak-nginx) *  [Secure kibana dashboards using keycloak](https://aboullaite.me/secure-kibana-keycloak/) *  [Configuring NGINX for OAuth/OpenID Connect SSO with Keycloak/Red Hat SSO](https://developers.redhat.com/blog/2018/10/08/configuring-nginx-keycloak-oauth-oidc/) *  [Keycloak Clustering Setup and Configuration Examples](https://github.com/fit2anything/keycloak-cluster-setup-and-configuration) *  [MicroProfile JWT with Keycloak](https://kodnito.com/posts/microprofile-jwt-with-keycloak/) *  [Keycloak Essentials](https://medium.com/keycloak/keycloak-essentials-86254b2f1872) *  [SSO-session failover with Keycloak and AWS S3](https://medium.com/@georgijsr/sso-session-failover-with-keycloak-and-aws-s3-e0b1db985e12) *  [KTOR and Keycloak: authentication with OpenId](https://medium.com/slickteam/ktor-and-keycloak-authentication-with-openid-ecd415d7a62e) * [Keycloak: Core concepts of open source identity and access management](https://developers.redhat.com/blog/2019/12/11/keycloak-core-concepts-of-open-source-identity-and-access-management) * [Who am I? Keycloak Impersonation API](https://blog.softwaremill.com/who-am-i-keycloak-impersonation-api-bfe7acaf051a) * [Setup Keycloak Server on Ubuntu 18.04](https://medium.com/@hasnat.saeed/setup-keycloak-server-on-ubuntu-18-04-ed8c7c79a2d9) * [Getting started with Keycloak](https://robferguson.org/blog/2019/12/24/getting-started-with-keycloak/) * [Angular, OpenID Connect and Keycloak](https://robferguson.org/blog/2019/12/29/angular-openid-connect-keycloak/) * [Angular, OAuth 2.0 Scopes and Keycloak](https://robferguson.org/blog/2019/12/31/angular-oauth2-keycloak/) * [Keycloak, Flowable and OpenLDAP](https://robferguson.org/blog/2020/01/03/keycloak-flowable-and-openldap/) * [How to exchange token from an external provider to a keycloak token](https://www.mathieupassenaud.fr/token-exchange-keycloak/) * [Building an Event Listener SPI (Plugin) for Keycloak](https://dev.to/adwaitthattey/building-an-event-listener-spi-plugin-for-keycloak-2044) * [Keycloak user migration – connect your legacy authentication system to Keycloak](https://codesoapbox.dev/keycloak-user-migration/) * [Keycloak Authentication and Authorization in GraphQL](https://medium.com/@darahayes/keycloak-authentication-and-authorization-in-graphql-ad0a1685f7da) * [Kong / Konga / Keycloak: securing API through OIDC](https://github.com/d4rkstar/kong-konga-keycloak) * [KeyCloak: Custom Login theme](https://codehumsafar.wordpress.com/2018/09/11/keycloak-custom-login-theme/) * [Keycloak: Use background color instead of background image in Custom Login theme](https://codehumsafar.wordpress.com/2018/09/21/keycloak-use-background-color-instead-of-background-image-in-custom-login-theme/) * [How to turn off the Keycloak theme cache](https://keycloakthemes.com/blog/how-to-turn-off-the-keycloak-theme-cache) * [How to add a custom field to the Keycloak registration page](https://keycloakthemes.com/blog/how-to-add-custom-field-keycloak-registration-page) * [How to setup Sign in with Google using Keycloak](https://keycloakthemes.com/blog/how-to-setup-sign-in-with-google-using-keycloak) * [How to sign in users on Keycloak using Github](https://keycloakthemes.com/blog/how-to-sign-in-users-on-keycloak-using-github) * [Extending Keycloak SSO Capabilities with IBM Security Verify](https://community.ibm.com/community/user/security/blogs/jason-choi1/2020/06/10/extending-keycloak-sso-capabilities-with-ibm-secur) * [AWS SAML based User Federation using Keycloak](https://medium.com/@karanbir.tech/aws-connect-saml-based-identity-provider-using-keycloak-9b3e6d0111e6) * [AWS user account OpenID federation using Keycloak](https://medium.com/@karanbir.tech/aws-account-openid-federation-using-keycloak-40d22b952a43) * [How to Run Keycloak in HA on Kubernetes](https://blog.sighup.io/keycloak-ha-on-kubernetes/) * [How to create a Keycloak authenticator as a microservice?](https://medium.com/application-security/how-to-create-a-keycloak-authenticator-as-a-microservice-ad332e287b58) * [keycloak.ch | Installing &amp; Running Keycloak](https://keycloak.ch/keycloak-tutorials/tutorial-1-installing-and-running-keycloak/) * [keycloak.ch | Configuring Token Exchange using the CLI](https://keycloak.ch/keycloak-tutorials/tutorial-token-exchange/) * [keycloak.ch | Configuring WebAuthn](https://keycloak.ch/keycloak-tutorials/tutorial-webauthn/) * [keycloak.ch | Configuring a SwissID integration](https://keycloak.ch/keycloak-tutorials/tutorial-swissid/) * [Getting Started with Service Accounts in Keycloak](https://medium.com/@mihirrajdixit/getting-started-with-service-accounts-in-keycloak-c8f6798a0675) * [Building cloud native apps: Identity and Access Management](https://dev.to/lukaszbudnik/building-cloud-native-apps-identity-and-access-management-1e5m) * [X.509 user certificate authentication with Red Hat’s single sign-on technology](https://developers.redhat.com/blog/2021/02/19/x-509-user-certificate-authentication-with-red-hats-single-sign-on-technology) * [Grafana OAuth with Keycloak and how to validate a JWT token](https://janikvonrotz.ch/2020/08/27/grafana-oauth-with-keycloak-and-how-to-validate-a-jwt-token/) * [How to setup a Keycloak server with external MySQL database on AWS ECS Fargate in clustered mode](https://jbjerksetmyr.medium.com/how-to-setup-a-keycloak-server-with-external-mysql-database-on-aws-ecs-fargate-in-clustered-mode-9775d01cd317) * [Extending Keycloak: adding API key authentication](http://www.zakariaamine.com/2019-06-14/extending-keycloak) * [Extending Keycloak: using a custom email sender](http://www.zakariaamine.com/2019-07-14/extending-keycloak2) * [Integrating Keycloak and OPA with Confluent](https://goraft.tech/2021/03/17/integrating-keycloak-and-opa-with-confluent.html) * [UMA 2.0 : User Managed Access - how to use it with bash](https://blog.please-open.it/uma/)  ## Talks *  [JDD2015 - Keycloak Open Source Identity and Access Management Solution](https://www.youtube.com/watch?v=TuEkj25lbd0) *  [2015 Using Tomcat and Keycloak in an iFrame](https://www.youtube.com/watch?v=nF_lw7uIxao) *  [2016 You've Got Microservices Now Secure Them](https://www.youtube.com/watch?v=SfVhqf-rMQY) *  [2016 Keycloak: Open Source Single Sign On - Sebastian Rose - AOE conf (german)](https://www.youtube.com/watch?v=wbKw0Bwyne4) *  [2016 Sécuriser ses applications back et front facilement avec Keycloak (french)](https://www.youtube.com/watch?v=bVidgluUcg0) *  [2016 Keycloak and Red Hat Mobile Application Platform](https://www.youtube.com/watch?v=4NBgiHM5aOA) *  [2016 Easily secure your Front and back applications with KeyCloak](https://www.youtube.com/watch?v=RGp4HUKikts) *  [2017 Easily secure your Spring Boot applications with Keycloak - Part 1](https://developers.redhat.com/video/youtube/vpgRTPFDHAw/) *  [2017 Easily secure your Spring Boot applications with Keycloak - Part 2](https://developers.redhat.com/video/youtube/O5ePCWON08Y/) *  [2018 How to secure your Spring Apps with Keycloak by Thomas Darimont @ Spring I/O 2018](https://www.youtube.com/watch?v=haHFoeWUj0w) *  [2018 DevNation Live | A Deep Dive into Keycloak](https://www.youtube.com/watch?v=ZxpY_zZ52kU) *  [2018 IDM Europe: WSO2 Identity Server vs. Keycloak (Dmitry Kann)](https://www.youtube.com/watch?v=hnjBiGsEDoU) *  [2018 JPrime|Building an effective identity and access management architecture with Keycloak (Sebastien Blanc)](https://www.youtube.com/watch?v=bMqcGkCvUVQ) *  [2018 WJAX| Sichere Spring-Anwendungen mit Keycloak](https://www.youtube.com/watch?v=6Z490EMcafs) *  [2019 Spring I/O | Secure your Spring Apps with Keycloak](https://www.youtube.com/watch?v=KrOd5wIkqls) *  [2019 DevoxxFR | Maitriser sa gestion de l'identité avec Keycloak (L. Benoit, T. Recloux, S. Blanc)](https://www.youtube.com/watch?v=0cziL__0-K8) *  [2019 DevConf | Fine - Grained Authorization with Keycloak SSO (Marek Posolda)](https://www.youtube.com/watch?v=yosg4St0iUw) *  [2019 VoxxedDays Minsk | Bilding an effective identity and access management architecture with Keycloak (Sebastien Blanc)](https://www.youtube.com/watch?v=RupQWmYhrLA) *  [2019 Single-Sign-On Authentifizierung mit dem Keycloak Identity Provider | jambit CoffeeTalk](https://www.youtube.com/watch?v=dnY6ORaFNY8) *  [2020 Keycloak Team | Keycloak Pitch](https://www.youtube.com/watch?v=GZTN_VXjoQw) *  [2020 Keycloak Team | Keycloak Overview](https://www.youtube.com/watch?v=duawSV69LDI) *  [2020 Please-open.it : oauth2 dans le monde des ops (french)](https://www.youtube.com/watch?v=S-9X50QajmY)  ## Presentations *  [Keycloak 101](https://stevenolen.github.io/kc101-talk/#1)  ## Video Playlists *  [Keycloak Identity and Access Management by Łukasz Budnik](https://www.youtube.com/playlist?list=PLPZal7ksxNs0mgScrJxrggEayV-TPZ9sA) *  [Keycloak by Niko Köbler](https://www.youtube.com/playlist?list=PLNn3plN7ZiaowUvKzKiJjYfWpp86u98iY) *  [Keycloak Playlist by hexaDefence](https://youtu.be/35bflT_zxXA) *  [Keycloak Tutorial Series by CodeLens](https://www.youtube.com/watch?v=Lr9WeIMtFow&amp;list=PLeGNmkzI56BTjRxNGxUhh4k30FD_gy0pC)  ## Clients *  [Official Keycloak Node.js Admin Client](https://github.com/keycloak/keycloak-admin-client/) ("Extremely Experimental") *  [Keycloak Node.js TypeScript Admin Client by Canner](https://github.com/Canner/keycloak-admin/) *  [Keycloak Go Client by Cloudtrust](https://github.com/cloudtrust/keycloak-client) *  [Keycloak Nest.js Admin Client by Relevant Fruit](https://github.com/relevantfruit/nestjs-keycloak-admin)  ## Community Extensions *  [Keycloak Extensions List](https://www.keycloak.org/extensions.html) *  [Keycloak Benchmark Project](https://github.com/keycloak/keycloak-benchmark) *  [Keycloak: Link IdP Login with User Provider](https://github.com/ohioit/keycloak-link-idp-with-user) *  [Client Owner Manager: Control who can edit a client](https://github.com/cyclone-project/cyclone-client-registration) *  [Keyloak Proxy written in Go](https://github.com/gambol99/keycloak-proxy) *  [Script based ProtocolMapper extension for SAML](https://github.com/cloudtrust/keycloak-client-mappers) *  [Realm export REST resource by Cloudtrust](https://github.com/cloudtrust/keycloak-export) *  [Keycloak JDBC Ping Setup by moremagic](https://github.com/moremagic/keycloak-jdbc-ping) *  [SMS 2 Factor Authentication for Keycloak via AWS SNS](https://github.com/nickpack/keycloak-sms-authenticator-sns) *  [SMS 2 Factor Authentiation for Keycloak via SMS by Alliander](https://github.com/Alliander/keycloak-sms-authenticator) *  [Identity Provider for vk.com](https://github.com/mrk08/keycloak-vk) *  [CAS Protocol Support](https://github.com/Doccrazy/keycloak-protocol-cas) *  [WS-FED Support](https://github.com/cloudtrust/keycloak-wsfed) *  [Keycloak Discord Support](https://github.com/wadahiro/keycloak-discord) *  [Keycloak Login with User Attribute](https://github.com/cnieg/keycloak-login-attribute) *  [zonaut/keycloak-extensions](https://github.com/zonaut/keycloak-extensions) *  [leroyguillaume/keycloak-bcrypt](https://github.com/leroyguillaume/keycloak-bcrypt) *  [SPI Authenticator in Nodejs](https://www.npmjs.com/package/keycloak-rest-authenticator) *  [Have I Been Pwned? Keycloak Password Policy](https://github.com/alexashley/keycloak-password-policy-have-i-been-pwned) *  [Keycloak Eventlistener for Google Cloud Pub Sub](https://github.com/acesso-io/keycloak-event-listener-gcpubsub) *  [Enforcing Password policy based on attributes of User Groups](https://github.com/sayedcsekuet/keycloak-user-group-based-password-policy) *  [Verify Email with Link or Code by hokumski](https://github.com/hokumski/keycloak-verifyemailwithcode) *  [Role-based Docker registry authentication](https://github.com/lifs-tools/keycloak-docker-role-mapper) *  [SCIM for keycloak](https://github.com/Captain-P-Goldfish/scim-for-keycloak) *  [Keycloak Kafka Module](https://github.com/SnuK87/keycloak-kafka)   ## Integrations *  [Official Keycloak Node.js Connect Adapter](https://github.com/keycloak/keycloak-nodejs-connect) *  [Keycloak support for Aurelia](https://github.com/waynepennington/aurelia-keycloak) *  [Keycloak OAuth2 Auth for PHP](https://github.com/stevenmaguire/oauth2-keycloak) *  [Jenkins Keycloak Authentication Plugin](https://github.com/jenkinsci/keycloak-plugin) *  [Meteor Keycloak Accounts](https://github.com/mxab/meteor-keycloak) *  [HapiJS Keycloak Auth](https://github.com/felixheck/hapi-auth-keycloak) *  [zmartzone mod_auth_openidc for Apache 2.x](https://github.com/zmartzone/mod_auth_openidc) *  [Duo Security MFA Authentication for Keycloak](https://github.com/mulesoft-labs/keycloak-duo-spi) *  [Extension Keycloak facilitant l'utilisation de FranceConnect](https://github.com/InseeFr/Keycloak-FranceConnect) *  [Ambassador Keycloak Support](https://www.getambassador.io/reference/idp-support/keycloak/) *  [Keycloak Python Client](https://github.com/akhilputhiry/keycloak-client) *  [Keycloak Terraform Provider](https://github.com/mrparkers/terraform-provider-keycloak) *  [Keycloak ADFS OpenID Connect](https://www.michaelboeynaems.com/keycloak-ADFS-OIDC.html) *  [React/NextJS Keycloak Bindings](https://github.com/panz3r/react-keycloak) *  [Keycloak Open-Shift integration](https://github.com/keycloak/openshift-integration) *  [Keycloak, Kong and Konga setup scripts (local development)](https://github.com/JaouherK/Kong-konga-Keycloak) *  [SSO for Keycloak and Nextcloud with SAML](https://stackoverflow.com/questions/48400812/sso-with-saml-keycloak-and-nextcloud) *  [Keycloak Connect GraphQL Adapter for Node.js](https://github.com/aerogear/keycloak-connect-graphql) *  [python-keycloak](https://github.com/marcospereirampj/python-keycloak) *  [Keycloak and PrivacyId3a docker-compose (local development)](https://github.com/JaouherK/keycloak-privacyIdea) *  [Nerzal/gocloak Golang Keycloak API Package](https://github.com/Nerzal/gocloak) *  [Apple Social Identity Provider for Keycloak](https://github.com/BenjaminFavre/keycloak-apple-social-identity-provider)  ## Quick demo Videos * [Keycloak with istio envoy jwt-auth proxy](https://www.youtube.com/watch?v=wscX7JMfuBI)  ## Themes *  [Community Keycloak Ionic Theme](https://github.com/lfryc/keycloak-ionic-theme) *  [A Keycloak theme based on the AdminLTE UI library](https://github.com/MAXIMUS-DeltaWare/adminlte-keycloak-theme) *  [GOV.UK Theme](https://github.com/UKHomeOffice/keycloak-theme-govuk) *  [Carbon Design](https://github.com/httpsOmkar/carbon-keycloak-theme) *  [Modern](https://keycloakthemes.com/themes/modern) *  [Adminlte](https://git.uptic.nl/uptic-public-projects/uptic-keyclock-theme-adminlte) *  [keycloakify: Create Keycloak themes using React](https://github.com/InseeFrLab/keycloakify)  ## Docker *  [Official Keycloak Docker Images](https://github.com/jboss-dockerfiles/keycloak) *  [Keycloak Examples as Docker Image](https://hub.docker.com/r/jboss/keycloak-examples) *  [Keycloak Maven SDK for managing the entire lifecycle of your extensions with Docker](https://github.com/OpenPj/keycloak-docker-quickstart)  ## Kubernetes *  [Deprecated Keycloak Helm Chart](https://github.com/codecentric/helm-charts/tree/master/charts/keycloak) *  [codecentric Keycloak Helm Chart](https://github.com/codecentric/helm-charts/tree/master/charts/keycloak) *  [Import / Export Keycloak Config](https://gist.github.com/unguiculus/19618ef57b1863145262191944565c9d) *  [keycloak-operator](https://github.com/keycloak/keycloak-operator)  ## Tools *  [keycloakmigration: Manage your Keycloak configuration with code](https://github.com/klg71/keycloakmigration) *  [tool to autogenerate an OpenAPI Specification for Keycloak's Admin API](https://github.com/ccouzens/keycloak-openapi) *  [oidc-bash-client](https://github.com/please-openit/oidc-bash-client) *  [louketo-proxy (FKA Gatekeeper)](https://github.com/louketo/louketo-proxy) *  [keycloak-config-cli: Configuration as Code for Keycloak](https://github.com/adorsys/keycloak-config-cli) *  [Keycloak Pulumi](https://github.com/pulumi/pulumi-keycloak) *  [Keycloak on AWS](https://github.com/aws-samples/keycloak-on-aws) *  [aws-cdk construct library that allows you to create KeyCloak on AWS in TypeScript or Python](https://github.com/aws-samples/cdk-keycloak) *  [keycloak-scanner Python CLI](https://github.com/NeuronAddict/keycloak-scanner)  ## Deployment Examples * [Keycloak deployment with CDK on AWS with Fargate](https://github.com/aws-samples/cdk-keycloak)  ## Example Projects *  [Examples from Keycloak Book: Keycloak - Identity and Access Management for Modern Applications](https://github.com/PacktPublishing/Keycloak-Identity-and-Access-Management-for-Modern-Applications) *  [Official Examples](https://github.com/keycloak/keycloak/tree/master/examples) *  [Keycloak Quickstarts](https://github.com/keycloak/keycloak-quickstarts) *  [Drupal 7.0 with Keycloak](https://gist.github.com/thomasdarimont/17fa146c4fb5440d7fc2ee6322ec392d) *  [Securing Realm Resources With Custom Roles](https://github.com/dteleguin/custom-admin-roles) *  [BeerCloak: a comprehensive KeyCloak extension example](https://github.com/dteleguin/beercloak) *  [KeyCloak Extensions: Securing Realm Resources With Custom Roles](https://github.com/dteleguin/custom-admin-roles) *  [Red Hat Single Sign-On Labs](https://github.com/RedHatWorkshops/red-hat-sso) *  [Spring Boot Keycloak Tutorial](https://github.com/sebastienblanc/spring-boot-keycloak-tutorial) *  [Custom Keycloak Docker Image of Computer Science House of RIT](https://github.com/ComputerScienceHouse/keycloak-docker) *  [Example of custom password hash SPI for Keycloak](https://github.com/pavelbogomolenko/keycloak-custom-password-hash) *  [Example for a custom http-client-provider with Proxy support](https://github.com/xiaoyvr/custom-http-client-provider) *  [Monitor your keycloak with prometheus](https://github.com/larscheid-schmitzhermes/keycloak-monitoring-prometheus) *  [Custom User Storage Provider .ear with jboss-cli setup](https://github.com/thomasdarimont/keycloak-user-storage-provider-demo) *  [Keycloak - Experimental extensions by Stian Thorgersen/Keycloak](https://github.com/stianst/keycloak-experimental) *  [Securing Spring Boot Admin &amp; Actuator Endpoints with Keycloak](https://github.com/thomasdarimont/spring-boot-admin-keycloak-example) *  [A Keycloak Mobile Implementation using Angular v4 and Ionic v3](https://github.com/tomjackman/keyonic-v2) *  [Example for Securing Apps with Keycloak on Kubernetes](https://github.com/stianst/demo-kubernetes) *  [Example for Securing AspDotNet Core Apps with Keycloak](https://github.com/thomasdarimont/kc-dnc-demo) *  [Example for passing custom URL parameters to a Keycloak theme for dynamic branding](https://github.com/dteleguin/keycloak-dynamic-branding) *  [Angular Webapp secured with Keycloak](https://github.com/CodepediaOrg/bookmarks.dev) *  [Keycloak Theme Development Kit](https://github.com/anthonny/kit-keycloak-theme) *  [Keycloak Clustering examples](https://github.com/ivangfr/keycloak-clustered) *  [Keycloak Last Login Date Event Listener](https://github.com/ThoreKr/keycloak-last-login-event-listener) *  [Keycloak Project Example (Customizations, Extensions, Configuration)](https://github.com/thomasdarimont/keycloak-project-example) *  [Example of adding API Key authentication to Keycloak](https://github.com/zak905/keycloak-api-key-demo)  ## Benchmarks *  [Gatling based Benchmark by @rvansa](https://github.com/rvansa/keycloak-benchmark)  ## Help * [Keycloak on Stackoverflow](https://stackoverflow.com/questions/tagged/keycloak)  ## Commercial Offerings *  [Red Hat Single Sign-On](https://access.redhat.com/products/red-hat-single-sign-on) *  [INTEGSOFT UNIFIED USER CREDENTIALS WITH KEYCLOAK SSO](https://www.integsoft.cz/en/sso.html#what-is-sso) *  [JIRA SSO Plugin by codecentric](https://marketplace.atlassian.com/plugins/de.codecentric.atlassian.oidc.jira-oidc-plugin/server/overview) *  [Keycloak Competence Center by Inventage AG](https://keycloak.ch/) *  [Keycloak as a Service](https://www.cloud-iam.com)  ## Miscellaneous *  [Find sites using Keycloak with google](https://www.google.de/search?q=inurl%3Aauth+inurl%3Arealms+inurl%3Aprotocol&amp;oq=inurl%3A&amp;client=ubuntu&amp;sourceid=chrome&amp;ie=UTF-8) *  [Keycloak Dev Bookmarks](http://bookmarks.dev/search?q=keycloak) - Use the tag [keycloak](https://www.bookmarks.dev/tagged/keycloak) *  [Use fail2ban to block brute-force attacks to keycloak server](https://gist.github.com/drmalex07/3eba8b98d0ac4a1e821e8e721b3e1816) *  [Pentest-Report Keycloak 8.0 Audit &amp; Pentest 11.2019 by Cure53](https://cure53.de/pentest-report_keycloak.pdf) *  [Keycloak - CNCF Security SIG - Self Assesment](https://docs.google.com/document/d/14IIGliP3BWjdS-0wfOk3l_1AU8kyoSiLUzpPImsz4R0/edit#)  # License  [![CC0](http://mirrors.creativecommons.org/presskit/buttons/88x31/svg/cc-zero.svg)](https://creativecommons.org/publicdomain/zero/1.0/)  To the extent possible under law, [Thomas Darimont](https://github.com/thomasdarimont) has waived all copyright and related or neighboring rights to this work.</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-bug-bounty</t>
+          <t>https://github.com/BabyJ723/blast-ON</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>2026-04-10T04:50:22Z</t>
+          <t>2026-06-01T20:23:48Z</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>BabyJ723/blast-ON</t>
+          <t>Viralmaniar/DDWPasteRecon</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -9760,29 +9760,29 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t># Awesome Keycloak [![Awesome](https://cdn.rawgit.com/sindresorhus/awesome/d7305f38d29fed78fa85652e3a63e154dd8e8829/media/badge.svg)](https://github.com/sindresorhus/awesome)  # [&lt;img src="https://www.keycloak.org/resources/images/keycloak_logo_480x108.png"&gt;](https://github.com/thomasdarimont/awesome-keycloak)  &gt; Carefully curated list of awesome Keycloak resources.  A curated list of resources for learning about the Open Source Identity and Access Management solution Keycloak.  Contains books, websites, blog posts, links to github Repositories.    # Contributing Contributions welcome. Add links through pull requests or create an issue to start a discussion. [Please refer to the contributing guide for details](CONTRIBUTING.md).  # Contents  * [General](#general)   * [Documentation](#docs)     * [Keycloak Website](http://www.keycloak.org)     * [Current Documentation](http://www.keycloak.org/documentation.html)     * [Archived Documentation](http://www.keycloak.org/documentation-archive.html)   * [Mailing Lists](#mailing-lists)     * [User Mailing List](#user-mailing-list)     * [Developer Mailing List](#dev-mailing-list)     * [Mailing List Search](#mailing-list-search) * [Books](#books) * [Articles](#articles) * [Talks](#talks) * [Presentations](#presentations) * [Video Playlists](#video-playlists) * [Community Extensions](#community-extensions) * [Integrations](#integrations) * [Themes](#themes) * [Docker](#docker) * [Deployment Examples](#deployment-examples) * [Example Projects](#example-projects) * [Benchmarks](#benchmarks) * [Help](#help) * [Commercial Offerings](#commercial-offerings) * [Miscellaneous](#miscellaneous)  # General  ## Documentation  *  [Keycloak Website](http://www.keycloak.org/) *  [Current Documentation](http://www.keycloak.org/documentation.html) *  [Archived Documentation](http://www.keycloak.org/documentation-archive.html) *  [Product Documentation for Red Hat Single Sign-On](https://access.redhat.com/documentation/en/red-hat-single-sign-on/)  ## Discussion Groups and Mailing Lists *  [Keycloak Users Google Group](https://groups.google.com/forum/#!forum/keycloak-user) *  [Keycloak Developers Google Group](https://groups.google.com/forum/#!forum/keycloak-dev) *  [Keycloak Discourse Group](https://keycloak.discourse.group/) *  [Keycloak Developer Chat](https://keycloak.zulipchat.com) *  [Inactive - User Mailing List](https://lists.jboss.org/mailman/listinfo/keycloak-user) *  [Inactive - Developer Mailing List](https://lists.jboss.org/mailman/listinfo/keycloak-dev) *  [Mailing List Search](http://www.keycloak.org/search) *  [Keycloak Subreddit](https://www.reddit.com/r/keycloak)  ## Books * [Keycloak - Identity and Access Management for Modern Applications](https://www.packtpub.com/product/keycloak-identity-and-access-management-for-modern-applications/9781800562493)  ## Articles *  [How to get Keycloak working with Docker](https://www.ivonet.nl/2015/05/23/Keycloak-Docker/) *  [Single-Sign-On for Microservices and/or Java EE applications with Keycloak SSO](http://www.n-k.de/2016/06/keycloak-sso-for-microservices.html) *  [Keycloak Admin Client(s) - multiple ways to manage your SSO system](http://www.n-k.de/2016/08/keycloak-admin-client.html) *  [How to get the AccessToken of Keycloak in Spring Boot and/or Java EE](http://www.n-k.de/2016/05/how-to-get-accesstoken-from-keycloak-springboot-javaee.html) *  [JWT authentication with Vert.x, Keycloak and Angular 2](http://paulbakker.io/java/jwt-keycloak-angular2/) *  [Authenticating via Kerberos with Keycloak and Windows 2008 Active Directory](http://matthewcasperson.blogspot.de/2015/07/authenticating-via-kerberos-with.html) *  [Deploying Keycloak with Ansible](https://adam.younglogic.com/2016/01/deploying-keycloak-via-ansible/) *  [Easily secure your Spring Boot applications with Keycloak](https://developers.redhat.com/blog/2017/05/25/easily-secure-your-spring-boot-applications-with-keycloak/) *  [How Red Hat re-designed its Single Sign On (SSO) architecture, and why](https://developers.redhat.com/blog/2016/10/04/how-red-hat-re-designed-its-single-sign-on-sso-architecture-and-why/) *  [OAuth2, JWT, Open-ID Connect and other confusing things](http://giallone.blogspot.de/2017/06/oath2.html) *  [X509 Authentication with Keycloak and JBoss Fuse](https://sjhiggs.github.io/fuse/sso/x509/smartcard/2017/03/29/fuse-hawtio-keycloak.html) *  [Running Keycloak on OpenShift 3](https://medium.com/@sbose78/running-keycloak-on-openshift-3-8d195c0daaf6) *  [Introducing Keycloak for Identity and Access Management](https://www.thomasvitale.com/introducing-keycloak-identity-access-management/) *  [Keycloak Basic Configuration for Authentication and Authorisation](https://www.thomasvitale.com/keycloak-configuration-authentication-authorisation/) *  [Keycloak on OpenShift Origin](https://medium.com/@james_devcomb/keycloak-on-openshift-origin-ee81d01dac97) *  [Identity Management, One-Time-Passwords and Two-Factor-Auth with Spring Boot and Keycloak](http://www.hascode.com/2017/11/identity-management-one-time-passwords-and-two-factor-auth-with-spring-boot-and-keycloak/) *  [Keycloak Identity Brokering with Openshift](https://developers.redhat.com/blog/2017/12/06/keycloak-identity-brokering-openshift/) *  [OpenID Connect Identity Brokering with Red Hat Single Sign-On](https://developers.redhat.com/blog/2017/10/18/openid-connect-identity-brokering-red-hat-single-sign/) *  [Authentication &amp; user management is hard](https://eclipsesource.com/blogs/2018/01/11/authenticating-reverse-proxy-with-keycloak/) *  [Securing Nginx with Keycloak](https://edhull.co.uk/blog/2018-06-06/keycloak-nginx) *  [Secure kibana dashboards using keycloak](https://aboullaite.me/secure-kibana-keycloak/) *  [Configuring NGINX for OAuth/OpenID Connect SSO with Keycloak/Red Hat SSO](https://developers.redhat.com/blog/2018/10/08/configuring-nginx-keycloak-oauth-oidc/) *  [Keycloak Clustering Setup and Configuration Examples](https://github.com/fit2anything/keycloak-cluster-setup-and-configuration) *  [MicroProfile JWT with Keycloak](https://kodnito.com/posts/microprofile-jwt-with-keycloak/) *  [Keycloak Essentials](https://medium.com/keycloak/keycloak-essentials-86254b2f1872) *  [SSO-session failover with Keycloak and AWS S3](https://medium.com/@georgijsr/sso-session-failover-with-keycloak-and-aws-s3-e0b1db985e12) *  [KTOR and Keycloak: authentication with OpenId](https://medium.com/slickteam/ktor-and-keycloak-authentication-with-openid-ecd415d7a62e) * [Keycloak: Core concepts of open source identity and access management](https://developers.redhat.com/blog/2019/12/11/keycloak-core-concepts-of-open-source-identity-and-access-management) * [Who am I? Keycloak Impersonation API](https://blog.softwaremill.com/who-am-i-keycloak-impersonation-api-bfe7acaf051a) * [Setup Keycloak Server on Ubuntu 18.04](https://medium.com/@hasnat.saeed/setup-keycloak-server-on-ubuntu-18-04-ed8c7c79a2d9) * [Getting started with Keycloak](https://robferguson.org/blog/2019/12/24/getting-started-with-keycloak/) * [Angular, OpenID Connect and Keycloak](https://robferguson.org/blog/2019/12/29/angular-openid-connect-keycloak/) * [Angular, OAuth 2.0 Scopes and Keycloak](https://robferguson.org/blog/2019/12/31/angular-oauth2-keycloak/) * [Keycloak, Flowable and OpenLDAP](https://robferguson.org/blog/2020/01/03/keycloak-flowable-and-openldap/) * [How to exchange token from an external provider to a keycloak token](https://www.mathieupassenaud.fr/token-exchange-keycloak/) * [Building an Event Listener SPI (Plugin) for Keycloak](https://dev.to/adwaitthattey/building-an-event-listener-spi-plugin-for-keycloak-2044) * [Keycloak user migration – connect your legacy authentication system to Keycloak](https://codesoapbox.dev/keycloak-user-migration/) * [Keycloak Authentication and Authorization in GraphQL](https://medium.com/@darahayes/keycloak-authentication-and-authorization-in-graphql-ad0a1685f7da) * [Kong / Konga / Keycloak: securing API through OIDC](https://github.com/d4rkstar/kong-konga-keycloak) * [KeyCloak: Custom Login theme](https://codehumsafar.wordpress.com/2018/09/11/keycloak-custom-login-theme/) * [Keycloak: Use background color instead of background image in Custom Login theme](https://codehumsafar.wordpress.com/2018/09/21/keycloak-use-background-color-instead-of-background-image-in-custom-login-theme/) * [How to turn off the Keycloak theme cache](https://keycloakthemes.com/blog/how-to-turn-off-the-keycloak-theme-cache) * [How to add a custom field to the Keycloak registration page](https://keycloakthemes.com/blog/how-to-add-custom-field-keycloak-registration-page) * [How to setup Sign in with Google using Keycloak](https://keycloakthemes.com/blog/how-to-setup-sign-in-with-google-using-keycloak) * [How to sign in users on Keycloak using Github](https://keycloakthemes.com/blog/how-to-sign-in-users-on-keycloak-using-github) * [Extending Keycloak SSO Capabilities with IBM Security Verify](https://community.ibm.com/community/user/security/blogs/jason-choi1/2020/06/10/extending-keycloak-sso-capabilities-with-ibm-secur) * [AWS SAML based User Federation using Keycloak](https://medium.com/@karanbir.tech/aws-connect-saml-based-identity-provider-using-keycloak-9b3e6d0111e6) * [AWS user account OpenID federation using Keycloak](https://medium.com/@karanbir.tech/aws-account-openid-federation-using-keycloak-40d22b952a43) * [How to Run Keycloak in HA on Kubernetes](https://blog.sighup.io/keycloak-ha-on-kubernetes/) * [How to create a Keycloak authenticator as a microservice?](https://medium.com/application-security/how-to-create-a-keycloak-authenticator-as-a-microservice-ad332e287b58) * [keycloak.ch | Installing &amp; Running Keycloak](https://keycloak.ch/keycloak-tutorials/tutorial-1-installing-and-running-keycloak/) * [keycloak.ch | Configuring Token Exchange using the CLI](https://keycloak.ch/keycloak-tutorials/tutorial-token-exchange/) * [keycloak.ch | Configuring WebAuthn](https://keycloak.ch/keycloak-tutorials/tutorial-webauthn/) * [keycloak.ch | Configuring a SwissID integration](https://keycloak.ch/keycloak-tutorials/tutorial-swissid/) * [Getting Started with Service Accounts in Keycloak](https://medium.com/@mihirrajdixit/getting-started-with-service-accounts-in-keycloak-c8f6798a0675) * [Building cloud native apps: Identity and Access Management](https://dev.to/lukaszbudnik/building-cloud-native-apps-identity-and-access-management-1e5m) * [X.509 user certificate authentication with Red Hat’s single sign-on technology](https://developers.redhat.com/blog/2021/02/19/x-509-user-certificate-authentication-with-red-hats-single-sign-on-technology) * [Grafana OAuth with Keycloak and how to validate a JWT token](https://janikvonrotz.ch/2020/08/27/grafana-oauth-with-keycloak-and-how-to-validate-a-jwt-token/) * [How to setup a Keycloak server with external MySQL database on AWS ECS Fargate in clustered mode](https://jbjerksetmyr.medium.com/how-to-setup-a-keycloak-server-with-external-mysql-database-on-aws-ecs-fargate-in-clustered-mode-9775d01cd317) * [Extending Keycloak: adding API key authentication](http://www.zakariaamine.com/2019-06-14/extending-keycloak) * [Extending Keycloak: using a custom email sender](http://www.zakariaamine.com/2019-07-14/extending-keycloak2) * [Integrating Keycloak and OPA with Confluent](https://goraft.tech/2021/03/17/integrating-keycloak-and-opa-with-confluent.html) * [UMA 2.0 : User Managed Access - how to use it with bash](https://blog.please-open.it/uma/)  ## Talks *  [JDD2015 - Keycloak Open Source Identity and Access Management Solution](https://www.youtube.com/watch?v=TuEkj25lbd0) *  [2015 Using Tomcat and Keycloak in an iFrame](https://www.youtube.com/watch?v=nF_lw7uIxao) *  [2016 You've Got Microservices Now Secure Them](https://www.youtube.com/watch?v=SfVhqf-rMQY) *  [2016 Keycloak: Open Source Single Sign On - Sebastian Rose - AOE conf (german)](https://www.youtube.com/watch?v=wbKw0Bwyne4) *  [2016 Sécuriser ses applications back et front facilement avec Keycloak (french)](https://www.youtube.com/watch?v=bVidgluUcg0) *  [2016 Keycloak and Red Hat Mobile Application Platform](https://www.youtube.com/watch?v=4NBgiHM5aOA) *  [2016 Easily secure your Front and back applications with KeyCloak](https://www.youtube.com/watch?v=RGp4HUKikts) *  [2017 Easily secure your Spring Boot applications with Keycloak - Part 1](https://developers.redhat.com/video/youtube/vpgRTPFDHAw/) *  [2017 Easily secure your Spring Boot applications with Keycloak - Part 2](https://developers.redhat.com/video/youtube/O5ePCWON08Y/) *  [2018 How to secure your Spring Apps with Keycloak by Thomas Darimont @ Spring I/O 2018](https://www.youtube.com/watch?v=haHFoeWUj0w) *  [2018 DevNation Live | A Deep Dive into Keycloak](https://www.youtube.com/watch?v=ZxpY_zZ52kU) *  [2018 IDM Europe: WSO2 Identity Server vs. Keycloak (Dmitry Kann)](https://www.youtube.com/watch?v=hnjBiGsEDoU) *  [2018 JPrime|Building an effective identity and access management architecture with Keycloak (Sebastien Blanc)](https://www.youtube.com/watch?v=bMqcGkCvUVQ) *  [2018 WJAX| Sichere Spring-Anwendungen mit Keycloak](https://www.youtube.com/watch?v=6Z490EMcafs) *  [2019 Spring I/O | Secure your Spring Apps with Keycloak](https://www.youtube.com/watch?v=KrOd5wIkqls) *  [2019 DevoxxFR | Maitriser sa gestion de l'identité avec Keycloak (L. Benoit, T. Recloux, S. Blanc)](https://www.youtube.com/watch?v=0cziL__0-K8) *  [2019 DevConf | Fine - Grained Authorization with Keycloak SSO (Marek Posolda)](https://www.youtube.com/watch?v=yosg4St0iUw) *  [2019 VoxxedDays Minsk | Bilding an effective identity and access management architecture with Keycloak (Sebastien Blanc)](https://www.youtube.com/watch?v=RupQWmYhrLA) *  [2019 Single-Sign-On Authentifizierung mit dem Keycloak Identity Provider | jambit CoffeeTalk](https://www.youtube.com/watch?v=dnY6ORaFNY8) *  [2020 Keycloak Team | Keycloak Pitch](https://www.youtube.com/watch?v=GZTN_VXjoQw) *  [2020 Keycloak Team | Keycloak Overview](https://www.youtube.com/watch?v=duawSV69LDI) *  [2020 Please-open.it : oauth2 dans le monde des ops (french)](https://www.youtube.com/watch?v=S-9X50QajmY)  ## Presentations *  [Keycloak 101](https://stevenolen.github.io/kc101-talk/#1)  ## Video Playlists *  [Keycloak Identity and Access Management by Łukasz Budnik](https://www.youtube.com/playlist?list=PLPZal7ksxNs0mgScrJxrggEayV-TPZ9sA) *  [Keycloak by Niko Köbler](https://www.youtube.com/playlist?list=PLNn3plN7ZiaowUvKzKiJjYfWpp86u98iY) *  [Keycloak Playlist by hexaDefence](https://youtu.be/35bflT_zxXA) *  [Keycloak Tutorial Series by CodeLens](https://www.youtube.com/watch?v=Lr9WeIMtFow&amp;list=PLeGNmkzI56BTjRxNGxUhh4k30FD_gy0pC)  ## Clients *  [Official Keycloak Node.js Admin Client](https://github.com/keycloak/keycloak-admin-client/) ("Extremely Experimental") *  [Keycloak Node.js TypeScript Admin Client by Canner](https://github.com/Canner/keycloak-admin/) *  [Keycloak Go Client by Cloudtrust](https://github.com/cloudtrust/keycloak-client) *  [Keycloak Nest.js Admin Client by Relevant Fruit](https://github.com/relevantfruit/nestjs-keycloak-admin)  ## Community Extensions *  [Keycloak Extensions List](https://www.keycloak.org/extensions.html) *  [Keycloak Benchmark Project](https://github.com/keycloak/keycloak-benchmark) *  [Keycloak: Link IdP Login with User Provider](https://github.com/ohioit/keycloak-link-idp-with-user) *  [Client Owner Manager: Control who can edit a client](https://github.com/cyclone-project/cyclone-client-registration) *  [Keyloak Proxy written in Go](https://github.com/gambol99/keycloak-proxy) *  [Script based ProtocolMapper extension for SAML](https://github.com/cloudtrust/keycloak-client-mappers) *  [Realm export REST resource by Cloudtrust](https://github.com/cloudtrust/keycloak-export) *  [Keycloak JDBC Ping Setup by moremagic](https://github.com/moremagic/keycloak-jdbc-ping) *  [SMS 2 Factor Authentication for Keycloak via AWS SNS](https://github.com/nickpack/keycloak-sms-authenticator-sns) *  [SMS 2 Factor Authentiation for Keycloak via SMS by Alliander](https://github.com/Alliander/keycloak-sms-authenticator) *  [Identity Provider for vk.com](https://github.com/mrk08/keycloak-vk) *  [CAS Protocol Support](https://github.com/Doccrazy/keycloak-protocol-cas) *  [WS-FED Support](https://github.com/cloudtrust/keycloak-wsfed) *  [Keycloak Discord Support](https://github.com/wadahiro/keycloak-discord) *  [Keycloak Login with User Attribute](https://github.com/cnieg/keycloak-login-attribute) *  [zonaut/keycloak-extensions](https://github.com/zonaut/keycloak-extensions) *  [leroyguillaume/keycloak-bcrypt](https://github.com/leroyguillaume/keycloak-bcrypt) *  [SPI Authenticator in Nodejs](https://www.npmjs.com/package/keycloak-rest-authenticator) *  [Have I Been Pwned? Keycloak Password Policy](https://github.com/alexashley/keycloak-password-policy-have-i-been-pwned) *  [Keycloak Eventlistener for Google Cloud Pub Sub](https://github.com/acesso-io/keycloak-event-listener-gcpubsub) *  [Enforcing Password policy based on attributes of User Groups](https://github.com/sayedcsekuet/keycloak-user-group-based-password-policy) *  [Verify Email with Link or Code by hokumski](https://github.com/hokumski/keycloak-verifyemailwithcode) *  [Role-based Docker registry authentication](https://github.com/lifs-tools/keycloak-docker-role-mapper) *  [SCIM for keycloak](https://github.com/Captain-P-Goldfish/scim-for-keycloak) *  [Keycloak Kafka Module](https://github.com/SnuK87/keycloak-kafka)   ## Integrations *  [Official Keycloak Node.js Connect Adapter](https://github.com/keycloak/keycloak-nodejs-connect) *  [Keycloak support for Aurelia](https://github.com/waynepennington/aurelia-keycloak) *  [Keycloak OAuth2 Auth for PHP](https://github.com/stevenmaguire/oauth2-keycloak) *  [Jenkins Keycloak Authentication Plugin](https://github.com/jenkinsci/keycloak-plugin) *  [Meteor Keycloak Accounts](https://github.com/mxab/meteor-keycloak) *  [HapiJS Keycloak Auth](https://github.com/felixheck/hapi-auth-keycloak) *  [zmartzone mod_auth_openidc for Apache 2.x](https://github.com/zmartzone/mod_auth_openidc) *  [Duo Security MFA Authentication for Keycloak](https://github.com/mulesoft-labs/keycloak-duo-spi) *  [Extension Keycloak facilitant l'utilisation de FranceConnect](https://github.com/InseeFr/Keycloak-FranceConnect) *  [Ambassador Keycloak Support](https://www.getambassador.io/reference/idp-support/keycloak/) *  [Keycloak Python Client](https://github.com/akhilputhiry/keycloak-client) *  [Keycloak Terraform Provider](https://github.com/mrparkers/terraform-provider-keycloak) *  [Keycloak ADFS OpenID Connect](https://www.michaelboeynaems.com/keycloak-ADFS-OIDC.html) *  [React/NextJS Keycloak Bindings](https://github.com/panz3r/react-keycloak) *  [Keycloak Open-Shift integration](https://github.com/keycloak/openshift-integration) *  [Keycloak, Kong and Konga setup scripts (local development)](https://github.com/JaouherK/Kong-konga-Keycloak) *  [SSO for Keycloak and Nextcloud with SAML](https://stackoverflow.com/questions/48400812/sso-with-saml-keycloak-and-nextcloud) *  [Keycloak Connect GraphQL Adapter for Node.js](https://github.com/aerogear/keycloak-connect-graphql) *  [python-keycloak](https://github.com/marcospereirampj/python-keycloak) *  [Keycloak and PrivacyId3a docker-compose (local development)](https://github.com/JaouherK/keycloak-privacyIdea) *  [Nerzal/gocloak Golang Keycloak API Package](https://github.com/Nerzal/gocloak) *  [Apple Social Identity Provider for Keycloak](https://github.com/BenjaminFavre/keycloak-apple-social-identity-provider)  ## Quick demo Videos * [Keycloak with istio envoy jwt-auth proxy](https://www.youtube.com/watch?v=wscX7JMfuBI)  ## Themes *  [Community Keycloak Ionic Theme](https://github.com/lfryc/keycloak-ionic-theme) *  [A Keycloak theme based on the AdminLTE UI library](https://github.com/MAXIMUS-DeltaWare/adminlte-keycloak-theme) *  [GOV.UK Theme](https://github.com/UKHomeOffice/keycloak-theme-govuk) *  [Carbon Design](https://github.com/httpsOmkar/carbon-keycloak-theme) *  [Modern](https://keycloakthemes.com/themes/modern) *  [Adminlte](https://git.uptic.nl/uptic-public-projects/uptic-keyclock-theme-adminlte) *  [keycloakify: Create Keycloak themes using React](https://github.com/InseeFrLab/keycloakify)  ## Docker *  [Official Keycloak Docker Images](https://github.com/jboss-dockerfiles/keycloak) *  [Keycloak Examples as Docker Image](https://hub.docker.com/r/jboss/keycloak-examples) *  [Keycloak Maven SDK for managing the entire lifecycle of your extensions with Docker](https://github.com/OpenPj/keycloak-docker-quickstart)  ## Kubernetes *  [Deprecated Keycloak Helm Chart](https://github.com/codecentric/helm-charts/tree/master/charts/keycloak) *  [codecentric Keycloak Helm Chart](https://github.com/codecentric/helm-charts/tree/master/charts/keycloak) *  [Import / Export Keycloak Config](https://gist.github.com/unguiculus/19618ef57b1863145262191944565c9d) *  [keycloak-operator](https://github.com/keycloak/keycloak-operator)  ## Tools *  [keycloakmigration: Manage your Keycloak configuration with code](https://github.com/klg71/keycloakmigration) *  [tool to autogenerate an OpenAPI Specification for Keycloak's Admin API](https://github.com/ccouzens/keycloak-openapi) *  [oidc-bash-client](https://github.com/please-openit/oidc-bash-client) *  [louketo-proxy (FKA Gatekeeper)](https://github.com/louketo/louketo-proxy) *  [keycloak-config-cli: Configuration as Code for Keycloak](https://github.com/adorsys/keycloak-config-cli) *  [Keycloak Pulumi](https://github.com/pulumi/pulumi-keycloak) *  [Keycloak on AWS](https://github.com/aws-samples/keycloak-on-aws) *  [aws-cdk construct library that allows you to create KeyCloak on AWS in TypeScript or Python](https://github.com/aws-samples/cdk-keycloak) *  [keycloak-scanner Python CLI](https://github.com/NeuronAddict/keycloak-scanner)  ## Deployment Examples * [Keycloak deployment with CDK on AWS with Fargate](https://github.com/aws-samples/cdk-keycloak)  ## Example Projects *  [Examples from Keycloak Book: Keycloak - Identity and Access Management for Modern Applications](https://github.com/PacktPublishing/Keycloak-Identity-and-Access-Management-for-Modern-Applications) *  [Official Examples](https://github.com/keycloak/keycloak/tree/master/examples) *  [Keycloak Quickstarts](https://github.com/keycloak/keycloak-quickstarts) *  [Drupal 7.0 with Keycloak](https://gist.github.com/thomasdarimont/17fa146c4fb5440d7fc2ee6322ec392d) *  [Securing Realm Resources With Custom Roles](https://github.com/dteleguin/custom-admin-roles) *  [BeerCloak: a comprehensive KeyCloak extension example](https://github.com/dteleguin/beercloak) *  [KeyCloak Extensions: Securing Realm Resources With Custom Roles](https://github.com/dteleguin/custom-admin-roles) *  [Red Hat Single Sign-On Labs](https://github.com/RedHatWorkshops/red-hat-sso) *  [Spring Boot Keycloak Tutorial](https://github.com/sebastienblanc/spring-boot-keycloak-tutorial) *  [Custom Keycloak Docker Image of Computer Science House of RIT](https://github.com/ComputerScienceHouse/keycloak-docker) *  [Example of custom password hash SPI for Keycloak](https://github.com/pavelbogomolenko/keycloak-custom-password-hash) *  [Example for a custom http-client-provider with Proxy support](https://github.com/xiaoyvr/custom-http-client-provider) *  [Monitor your keycloak with prometheus](https://github.com/larscheid-schmitzhermes/keycloak-monitoring-prometheus) *  [Custom User Storage Provider .ear with jboss-cli setup](https://github.com/thomasdarimont/keycloak-user-storage-provider-demo) *  [Keycloak - Experimental extensions by Stian Thorgersen/Keycloak](https://github.com/stianst/keycloak-experimental) *  [Securing Spring Boot Admin &amp; Actuator Endpoints with Keycloak](https://github.com/thomasdarimont/spring-boot-admin-keycloak-example) *  [A Keycloak Mobile Implementation using Angular v4 and Ionic v3](https://github.com/tomjackman/keyonic-v2) *  [Example for Securing Apps with Keycloak on Kubernetes](https://github.com/stianst/demo-kubernetes) *  [Example for Securing AspDotNet Core Apps with Keycloak](https://github.com/thomasdarimont/kc-dnc-demo) *  [Example for passing custom URL parameters to a Keycloak theme for dynamic branding](https://github.com/dteleguin/keycloak-dynamic-branding) *  [Angular Webapp secured with Keycloak](https://github.com/CodepediaOrg/bookmarks.dev) *  [Keycloak Theme Development Kit](https://github.com/anthonny/kit-keycloak-theme) *  [Keycloak Clustering examples](https://github.com/ivangfr/keycloak-clustered) *  [Keycloak Last Login Date Event Listener](https://github.com/ThoreKr/keycloak-last-login-event-listener) *  [Keycloak Project Example (Customizations, Extensions, Configuration)](https://github.com/thomasdarimont/keycloak-project-example) *  [Example of adding API Key authentication to Keycloak](https://github.com/zak905/keycloak-api-key-demo)  ## Benchmarks *  [Gatling based Benchmark by @rvansa](https://github.com/rvansa/keycloak-benchmark)  ## Help * [Keycloak on Stackoverflow](https://stackoverflow.com/questions/tagged/keycloak)  ## Commercial Offerings *  [Red Hat Single Sign-On](https://access.redhat.com/products/red-hat-single-sign-on) *  [INTEGSOFT UNIFIED USER CREDENTIALS WITH KEYCLOAK SSO](https://www.integsoft.cz/en/sso.html#what-is-sso) *  [JIRA SSO Plugin by codecentric](https://marketplace.atlassian.com/plugins/de.codecentric.atlassian.oidc.jira-oidc-plugin/server/overview) *  [Keycloak Competence Center by Inventage AG](https://keycloak.ch/) *  [Keycloak as a Service](https://www.cloud-iam.com)  ## Miscellaneous *  [Find sites using Keycloak with google](https://www.google.de/search?q=inurl%3Aauth+inurl%3Arealms+inurl%3Aprotocol&amp;oq=inurl%3A&amp;client=ubuntu&amp;sourceid=chrome&amp;ie=UTF-8) *  [Keycloak Dev Bookmarks](http://bookmarks.dev/search?q=keycloak) - Use the tag [keycloak](https://www.bookmarks.dev/tagged/keycloak) *  [Use fail2ban to block brute-force attacks to keycloak server](https://gist.github.com/drmalex07/3eba8b98d0ac4a1e821e8e721b3e1816) *  [Pentest-Report Keycloak 8.0 Audit &amp; Pentest 11.2019 by Cure53](https://cure53.de/pentest-report_keycloak.pdf) *  [Keycloak - CNCF Security SIG - Self Assesment](https://docs.google.com/document/d/14IIGliP3BWjdS-0wfOk3l_1AU8kyoSiLUzpPImsz4R0/edit#)  # License  [![CC0](http://mirrors.creativecommons.org/presskit/buttons/88x31/svg/cc-zero.svg)](https://creativecommons.org/publicdomain/zero/1.0/)  To the extent possible under law, [Thomas Darimont](https://github.com/thomasdarimont) has waived all copyright and related or neighboring rights to this work.</t>
+          <t>DDWPasteRecon tool will help you identify code leak, sensitive files, plaintext passwords, password hashes. It also allow member of SOC &amp; Blue Team to gain situational awareness of the organisation's web exposure on the pastesites. It Utilises Google's indexing of pastesites to gain targeted intelligence of the organisation. Blue &amp; SOC teams can collect and analyse data from these indexed pastesites to better protect against unknown threats.</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>https://github.com/BabyJ723/blast-ON</t>
+          <t>https://github.com/Viralmaniar/DDWPasteRecon</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>C#</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>2026-06-01T20:23:48Z</t>
+          <t>2026-05-05T03:46:12Z</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Viralmaniar/DDWPasteRecon</t>
+          <t>paulveillard/cybersecurity-bug-bounty</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -9790,22 +9790,22 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>DDWPasteRecon tool will help you identify code leak, sensitive files, plaintext passwords, password hashes. It also allow member of SOC &amp; Blue Team to gain situational awareness of the organisation's web exposure on the pastesites. It Utilises Google's indexing of pastesites to gain targeted intelligence of the organisation. Blue &amp; SOC teams can collect and analyse data from these indexed pastesites to better protect against unknown threats.</t>
+          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Bug Bounty in Cybersecurity.</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>https://github.com/Viralmaniar/DDWPasteRecon</t>
+          <t>https://github.com/paulveillard/cybersecurity-bug-bounty</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>C#</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>2026-05-05T03:46:12Z</t>
+          <t>2026-04-10T04:50:22Z</t>
         </is>
       </c>
     </row>
@@ -9842,7 +9842,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>usr2r00t/ChatGTP3-Prompts_Bug-Bounty</t>
+          <t>Prathamrajgor/hacking_books</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -9850,12 +9850,12 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>A list of ChatGPT Prompts for Web Application Security, Bug Bounty, and Pentesting</t>
+          <t>Books on Hacking and pen-testing</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>https://github.com/usr2r00t/ChatGTP3-Prompts_Bug-Bounty</t>
+          <t>https://github.com/Prathamrajgor/hacking_books</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -9865,14 +9865,14 @@
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>2026-06-12T23:01:18Z</t>
+          <t>2026-06-13T04:18:19Z</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Prathamrajgor/hacking_books</t>
+          <t>Xservus/PenTestTools</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -9880,12 +9880,12 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Books on Hacking and pen-testing</t>
+          <t>A currated list of pentest tools that are in active use by the twitter infosec community.</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>https://github.com/Prathamrajgor/hacking_books</t>
+          <t>https://github.com/Xservus/PenTestTools</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -9895,7 +9895,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>2026-06-13T04:18:19Z</t>
+          <t>2025-04-20T01:07:07Z</t>
         </is>
       </c>
     </row>
@@ -9932,7 +9932,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Xservus/PenTestTools</t>
+          <t>usr2r00t/ChatGTP3-Prompts_Bug-Bounty</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -9940,12 +9940,12 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>A currated list of pentest tools that are in active use by the twitter infosec community.</t>
+          <t>A list of ChatGPT Prompts for Web Application Security, Bug Bounty, and Pentesting</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>https://github.com/Xservus/PenTestTools</t>
+          <t>https://github.com/usr2r00t/ChatGTP3-Prompts_Bug-Bounty</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -9955,14 +9955,14 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>2025-04-20T01:07:07Z</t>
+          <t>2026-06-12T23:01:18Z</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>RITRedteam/StreetCred</t>
+          <t>Aryia-Behroziuan/Other-sources</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -9970,29 +9970,29 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Tool created for Red Team to test default credentials on SSH and WinRM and then execute scripts with those credentials before the password can be changed by Blue Team.</t>
+          <t>Asada, M.; Hosoda, K.; Kuniyoshi, Y.; Ishiguro, H.; Inui, T.; Yoshikawa, Y.; Ogino, M.; Yoshida, C. (2009). "Cognitive developmental robotics: a survey". IEEE Transactions on Autonomous Mental Development. 1 (1): 12–34. doi:10.1109/tamd.2009.2021702. S2CID 10168773. "ACM Computing Classification System: Artificial intelligence". ACM. 1998. Archived from the original on 12 October 2007. Retrieved 30 August 2007. Goodman, Joanna (2016). Robots in Law: How Artificial Intelligence is Transforming Legal Services (1st ed.). Ark Group. ISBN 978-1-78358-264-8. Archived from the original on 8 November 2016. Retrieved 7 November 2016. Albus, J. S. (2002). "4-D/RCS: A Reference Model Architecture for Intelligent Unmanned Ground Vehicles" (PDF). In Gerhart, G.; Gunderson, R.; Shoemaker, C. (eds.). Proceedings of the SPIE AeroSense Session on Unmanned Ground Vehicle Technology. Unmanned Ground Vehicle Technology IV. 3693. pp. 11–20. Bibcode:2002SPIE.4715..303A. CiteSeerX 10.1.1.15.14. doi:10.1117/12.474462. S2CID 63339739. Archived from the original (PDF) on 25 July 2004. Aleksander, Igor (1995). Artificial Neuroconsciousness: An Update. IWANN. Archived from the original on 2 March 1997. BibTex Archived 2 March 1997 at the Wayback Machine. Bach, Joscha (2008). "Seven Principles of Synthetic Intelligence". In Wang, Pei; Goertzel, Ben; Franklin, Stan (eds.). Artificial General Intelligence, 2008: Proceedings of the First AGI Conference. IOS Press. pp. 63–74. ISBN 978-1-58603-833-5. Archived from the original on 8 July 2016. Retrieved 16 February 2016. "Robots could demand legal rights". BBC News. 21 December 2006. Archived from the original on 15 October 2019. Retrieved 3 February 2011. Brooks, Rodney (1990). "Elephants Don't Play Chess" (PDF). Robotics and Autonomous Systems. 6 (1–2): 3–15. CiteSeerX 10.1.1.588.7539. doi:10.1016/S0921-8890(05)80025-9. Archived (PDF) from the original on 9 August 2007. Brooks, R. A. (1991). "How to build complete creatures rather than isolated cognitive simulators". In VanLehn, K. (ed.). Architectures for Intelligence. Hillsdale, NJ: Lawrence Erlbaum Associates. pp. 225–239. CiteSeerX 10.1.1.52.9510. Buchanan, Bruce G. (2005). "A (Very) Brief History of Artificial Intelligence" (PDF). AI Magazine: 53–60. Archived from the original (PDF) on 26 September 2007. Butler, Samuel (13 June 1863). "Darwin among the Machines". Letters to the Editor. The Press. Christchurch, New Zealand. Archived from the original on 19 September 2008. Retrieved 16 October 2014 – via Victoria University of Wellington. Clark, Jack (8 December 2015). "Why 2015 Was a Breakthrough Year in Artificial Intelligence". Bloomberg News. Archived from the original on 23 November 2016. Retrieved 23 November 2016. After a half-decade of quiet breakthroughs in artificial intelligence, 2015 has been a landmark year. Computers are smarter and learning faster than ever. "AI set to exceed human brain power". CNN. 26 July 2006. Archived from the original on 19 February 2008. Dennett, Daniel (1991). Consciousness Explained. The Penguin Press. ISBN 978-0-7139-9037-9. Domingos, Pedro (2015). The Master Algorithm: How the Quest for the Ultimate Learning Machine Will Remake Our World. Basic Books. ISBN 978-0-465-06192-1. Dowe, D. L.; Hajek, A. R. (1997). "A computational extension to the Turing Test". Proceedings of the 4th Conference of the Australasian Cognitive Science Society. Archived from the original on 28 June 2011. Dreyfus, Hubert (1972). What Computers Can't Do. New York: MIT Press. ISBN 978-0-06-011082-6. Dreyfus, Hubert; Dreyfus, Stuart (1986). Mind over Machine: The Power of Human Intuition and Expertise in the Era of the Computer. Oxford, UK: Blackwell. ISBN 978-0-02-908060-3. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Dreyfus, Hubert (1992). What Computers Still Can't Do. New York: MIT Press. ISBN 978-0-262-54067-4. Dyson, George (1998). Darwin among the Machines. Allan Lane Science. ISBN 978-0-7382-0030-9. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Edelman, Gerald (23 November 2007). "Gerald Edelman – Neural Darwinism and Brain-based Devices". Talking Robots. Archived from the original on 8 October 2009. Edelson, Edward (1991). The Nervous System. New York: Chelsea House. ISBN 978-0-7910-0464-7. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Fearn, Nicholas (2007). The Latest Answers to the Oldest Questions: A Philosophical Adventure with the World's Greatest Thinkers. New York: Grove Press. ISBN 978-0-8021-1839-4. Gladwell, Malcolm (2005). Blink. New York: Little, Brown and Co. ISBN 978-0-316-17232-5. Gödel, Kurt (1951). Some basic theorems on the foundations of mathematics and their implications. Gibbs Lecture. In Feferman, Solomon, ed. (1995). Kurt Gödel: Collected Works, Vol. III: Unpublished Essays and Lectures. Oxford University Press. pp. 304–23. ISBN 978-0-19-514722-3. Haugeland, John (1985). Artificial Intelligence: The Very Idea. Cambridge, Mass.: MIT Press. ISBN 978-0-262-08153-5. Hawkins, Jeff; Blakeslee, Sandra (2005). On Intelligence. New York, NY: Owl Books. ISBN 978-0-8050-7853-4. Henderson, Mark (24 April 2007). "Human rights for robots? We're getting carried away". The Times Online. London. Archived from the original on 31 May 2014. Retrieved 31 May 2014. Hernandez-Orallo, Jose (2000). "Beyond the Turing Test". Journal of Logic, Language and Information. 9 (4): 447–466. doi:10.1023/A:1008367325700. S2CID 14481982. Hernandez-Orallo, J.; Dowe, D. L. (2010). "Measuring Universal Intelligence: Towards an Anytime Intelligence Test". Artificial Intelligence. 174 (18): 1508–1539. CiteSeerX 10.1.1.295.9079. doi:10.1016/j.artint.2010.09.006. Hinton, G. E. (2007). "Learning multiple layers of representation". Trends in Cognitive Sciences. 11 (10): 428–434. doi:10.1016/j.tics.2007.09.004. PMID 17921042. S2CID 15066318. Hofstadter, Douglas (1979). Gödel, Escher, Bach: an Eternal Golden Braid. New York, NY: Vintage Books. ISBN 978-0-394-74502-2. Holland, John H. (1975). Adaptation in Natural and Artificial Systems. University of Michigan Press. ISBN 978-0-262-58111-0. Archived from the original on 26 July 2020. Retrieved 17 December 2019. Howe, J. (November 1994). "Artificial Intelligence at Edinburgh University: a Perspective". Archived from the original on 15 May 2007. Retrieved 30 August 2007. Hutter, M. (2012). "One Decade of Universal Artificial Intelligence". Theoretical Foundations of Artificial General Intelligence. Atlantis Thinking Machines. 4. pp. 67–88. CiteSeerX 10.1.1.228.8725. doi:10.2991/978-94-91216-62-6_5. ISBN 978-94-91216-61-9. S2CID 8888091. Kahneman, Daniel; Slovic, D.; Tversky, Amos (1982). Judgment under uncertainty: Heuristics and biases. Science. 185. New York: Cambridge University Press. pp. 1124–31. doi:10.1126/science.185.4157.1124. ISBN 978-0-521-28414-1. PMID 17835457. S2CID 143452957. Kaplan, Andreas; Haenlein, Michael (2019). "Siri, Siri in my Hand, who's the Fairest in the Land? On the Interpretations, Illustrations and Implications of Artificial Intelligence". Business Horizons. 62: 15–25. doi:10.1016/j.bushor.2018.08.004. Katz, Yarden (1 November 2012). "Noam Chomsky on Where Artificial Intelligence Went Wrong". The Atlantic. Archived from the original on 28 February 2019. Retrieved 26 October 2014. "Kismet". MIT Artificial Intelligence Laboratory, Humanoid Robotics Group. Archived from the original on 17 October 2014. Retrieved 25 October 2014. Koza, John R. (1992). Genetic Programming (On the Programming of Computers by Means of Natural Selection). MIT Press. Bibcode:1992gppc.book.....K. ISBN 978-0-262-11170-6. Kolata, G. (1982). "How can computers get common sense?". Science. 217 (4566): 1237–1238. Bibcode:1982Sci...217.1237K. doi:10.1126/science.217.4566.1237. PMID 17837639. Kumar, Gulshan; Kumar, Krishan (2012). "The Use of Artificial-Intelligence-Based Ensembles for Intrusion Detection: A Review". Applied Computational Intelligence and Soft Computing. 2012: 1–20. doi:10.1155/2012/850160. Kurzweil, Ray (1999). The Age of Spiritual Machines. Penguin Books. ISBN 978-0-670-88217-5. Kurzweil, Ray (2005). The Singularity is Near. Penguin Books. ISBN 978-0-670-03384-3. Lakoff, George; Núñez, Rafael E. (2000). Where Mathematics Comes From: How the Embodied Mind Brings Mathematics into Being. Basic Books. ISBN 978-0-465-03771-1. Langley, Pat (2011). "The changing science of machine learning". Machine Learning. 82 (3): 275–279. doi:10.1007/s10994-011-5242-y. Law, Diane (June 1994). Searle, Subsymbolic Functionalism and Synthetic Intelligence (Technical report). University of Texas at Austin. p. AI94-222. CiteSeerX 10.1.1.38.8384. Legg, Shane; Hutter, Marcus (15 June 2007). A Collection of Definitions of Intelligence (Technical report). IDSIA. arXiv:0706.3639. Bibcode:2007arXiv0706.3639L. 07-07. Lenat, Douglas; Guha, R. V. (1989). Building Large Knowledge-Based Systems. Addison-Wesley. ISBN 978-0-201-51752-1. Lighthill, James (1973). "Artificial Intelligence: A General Survey". Artificial Intelligence: a paper symposium. Science Research Council. Lucas, John (1961). "Minds, Machines and Gödel". In Anderson, A.R. (ed.). Minds and Machines. Archived from the original on 19 August 2007. Retrieved 30 August 2007. Lungarella, M.; Metta, G.; Pfeifer, R.; Sandini, G. (2003). "Developmental robotics: a survey". Connection Science. 15 (4): 151–190. CiteSeerX 10.1.1.83.7615. doi:10.1080/09540090310001655110. S2CID 1452734. Maker, Meg Houston (2006). "AI@50: AI Past, Present, Future". Dartmouth College. Archived from the original on 3 January 2007. Retrieved 16 October 2008. Markoff, John (16 February 2011). "Computer Wins on 'Jeopardy!': Trivial, It's Not". The New York Times. Archived from the original on 22 October 2014. Retrieved 25 October 2014. McCarthy, John; Minsky, Marvin; Rochester, Nathan; Shannon, Claude (1955). "A Proposal for the Dartmouth Summer Research Project on Artificial Intelligence". Archived from the original on 26 August 2007. Retrieved 30 August 2007.. McCarthy, John; Hayes, P. J. (1969). "Some philosophical problems from the standpoint of artificial intelligence". Machine Intelligence. 4: 463–502. CiteSeerX 10.1.1.85.5082. Archived from the original on 10 August 2007. Retrieved 30 August 2007. McCarthy, John (12 November 2007). "What Is Artificial Intelligence?". Archived from the original on 18 November 2015. Minsky, Marvin (1967). Computation: Finite and Infinite Machines. Englewood Cliffs, N.J.: Prentice-Hall. ISBN 978-0-13-165449-5. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Minsky, Marvin (2006). The Emotion Machine. New York, NY: Simon &amp; Schusterl. ISBN 978-0-7432-7663-4. Moravec, Hans (1988). Mind Children. Harvard University Press. ISBN 978-0-674-57616-2. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Norvig, Peter (25 June 2012). "On Chomsky and the Two Cultures of Statistical Learning". Peter Norvig. Archived from the original on 19 October 2014. NRC (United States National Research Council) (1999). "Developments in Artificial Intelligence". Funding a Revolution: Government Support for Computing Research. National Academy Press. Needham, Joseph (1986). Science and Civilization in China: Volume 2. Caves Books Ltd. Newell, Allen; Simon, H. A. (1976). "Computer Science as Empirical Inquiry: Symbols and Search". Communications of the ACM. 19 (3): 113–126. doi:10.1145/360018.360022.. Nilsson, Nils (1983). "Artificial Intelligence Prepares for 2001" (PDF). AI Magazine. 1 (1). Archived (PDF) from the original on 17 August 2020. Retrieved 22 August 2020. Presidential Address to the Association for the Advancement of Artificial Intelligence. O'Brien, James; Marakas, George (2011). Management Information Systems (10th ed.). McGraw-Hill/Irwin. ISBN 978-0-07-337681-3. O'Connor, Kathleen Malone (1994). "The alchemical creation of life (takwin) and other concepts of Genesis in medieval Islam". University of Pennsylvania: 1–435. Archived from the original on 5 December 2019. Retrieved 27 August 2008. Oudeyer, P-Y. (2010). "On the impact of robotics in behavioral and cognitive sciences: from insect navigation to human cognitive development" (PDF). IEEE Transactions on Autonomous Mental Development. 2 (1): 2–16. doi:10.1109/tamd.2009.2039057. S2CID 6362217. Archived (PDF) from the original on 3 October 2018. Retrieved 4 June 2013. Penrose, Roger (1989). The Emperor's New Mind: Concerning Computer, Minds and The Laws of Physics. Oxford University Press. ISBN 978-0-19-851973-7. Poli, R.; Langdon, W. B.; McPhee, N. F. (2008). A Field Guide to Genetic Programming. Lulu.com. ISBN 978-1-4092-0073-4. Archived from the original on 8 August 2015. Retrieved 21 April 2008 – via gp-field-guide.org.uk. Rajani, Sandeep (2011). "Artificial Intelligence – Man or Machine" (PDF). International Journal of Information Technology and Knowledge Management. 4 (1): 173–176. Archived from the original (PDF) on 18 January 2013. Ronald, E. M. A. and Sipper, M. Intelligence is not enough: On the socialization of talking machines, Minds and Machines Archived 25 July 2020 at the Wayback Machine, vol. 11, no. 4, pp. 567–576, November 2001. Ronald, E. M. A. and Sipper, M. What use is a Turing chatterbox? Archived 25 July 2020 at the Wayback Machine, Communications of the ACM, vol. 43, no. 10, pp. 21–23, October 2000. "Science". August 1982. Archived from the original on 25 July 2020. Retrieved 16 February 2016. Searle, John (1980). "Minds, Brains and Programs" (PDF). Behavioral and Brain Sciences. 3 (3): 417–457. doi:10.1017/S0140525X00005756. Archived (PDF) from the original on 17 March 2019. Retrieved 22 August 2020. Searle, John (1999). Mind, language and society. New York, NY: Basic Books. ISBN 978-0-465-04521-1. OCLC 231867665. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Shapiro, Stuart C. (1992). "Artificial Intelligence". In Shapiro, Stuart C. (ed.). Encyclopedia of Artificial Intelligence (PDF) (2nd ed.). New York: John Wiley. pp. 54–57. ISBN 978-0-471-50306-4. Archived (PDF) from the original on 1 February 2016. Retrieved 29 May 2009. Simon, H. A. (1965). The Shape of Automation for Men and Management. New York: Harper &amp; Row. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Skillings, Jonathan (3 July 2006). "Getting Machines to Think Like Us". cnet. Archived from the original on 16 November 2011. Retrieved 3 February 2011. Solomonoff, Ray (1956). An Inductive Inference Machine (PDF). Dartmouth Summer Research Conference on Artificial Intelligence. Archived (PDF) from the original on 26 April 2011. Retrieved 22 March 2011 – via std.com, pdf scanned copy of the original. Later published as Solomonoff, Ray (1957). "An Inductive Inference Machine". IRE Convention Record. Section on Information Theory, part 2. pp. 56–62. Tao, Jianhua; Tan, Tieniu (2005). Affective Computing and Intelligent Interaction. Affective Computing: A Review. LNCS 3784. Springer. pp. 981–995. doi:10.1007/11573548. Tecuci, Gheorghe (March–April 2012). "Artificial Intelligence". Wiley Interdisciplinary Reviews: Computational Statistics. 4 (2): 168–180. doi:10.1002/wics.200. Thro, Ellen (1993). Robotics: The Marriage of Computers and Machines. New York: Facts on File. ISBN 978-0-8160-2628-9. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Turing, Alan (October 1950), "Computing Machinery and Intelligence", Mind, LIX (236): 433–460, doi:10.1093/mind/LIX.236.433, ISSN 0026-4423. van der Walt, Christiaan; Bernard, Etienne (2006). "Data characteristics that determine classifier performance" (PDF). Archived from the original (PDF) on 25 March 2009. Retrieved 5 August 2009. Vinge, Vernor (1993). "The Coming Technological Singularity: How to Survive in the Post-Human Era". Vision 21: Interdisciplinary Science and Engineering in the Era of Cyberspace: 11. Bibcode:1993vise.nasa...11V. Archived from the original on 1 January 2007. Retrieved 14 November 2011. Wason, P. C.; Shapiro, D. (1966). "Reasoning". In Foss, B. M. (ed.). New horizons in psychology. Harmondsworth: Penguin. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Weizenbaum, Joseph (1976). Computer Power and Human Reason. San Francisco: W.H. Freeman &amp; Company. ISBN 978-0-7167-0464-5. Weng, J.; McClelland; Pentland, A.; Sporns, O.; Stockman, I.; Sur, M.; Thelen, E. (2001). "Autonomous mental development by robots and animals" (PDF). Science. 291 (5504): 599–600. doi:10.1126/science.291.5504.599. PMID 11229402. S2CID 54131797. Archived (PDF) from the original on 4 September 2013. Retrieved 4 June 2013 – via msu.edu. "Applications of AI". www-formal.stanford.edu. Archived from the original on 28 August 2016. Retrieved 25 September 2016. Further reading DH Author, 'Why Are There Still So Many Jobs? The History and Future of Workplace Automation' (2015) 29(3) Journal of Economic Perspectives 3. Boden, Margaret, Mind As Machine, Oxford University Press, 2006. Cukier, Kenneth, "Ready for Robots? How to Think about the Future of AI", Foreign Affairs, vol. 98, no. 4 (July/August 2019), pp. 192–98. George Dyson, historian of computing, writes (in what might be called "Dyson's Law") that "Any system simple enough to be understandable will not be complicated enough to behave intelligently, while any system complicated enough to behave intelligently will be too complicated to understand." (p. 197.) Computer scientist Alex Pentland writes: "Current AI machine-learning algorithms are, at their core, dead simple stupid. They work, but they work by brute force." (p. 198.) Domingos, Pedro, "Our Digital Doubles: AI will serve our species, not control it", Scientific American, vol. 319, no. 3 (September 2018), pp. 88–93. Gopnik, Alison, "Making AI More Human: Artificial intelligence has staged a revival by starting to incorporate what we know about how children learn", Scientific American, vol. 316, no. 6 (June 2017), pp. 60–65. Johnston, John (2008) The Allure of Machinic Life: Cybernetics, Artificial Life, and the New AI, MIT Press. Koch, Christof, "Proust among the Machines", Scientific American, vol. 321, no. 6 (December 2019), pp. 46–49. Christof Koch doubts the possibility of "intelligent" machines attaining consciousness, because "[e]ven the most sophisticated brain simulations are unlikely to produce conscious feelings." (p. 48.) According to Koch, "Whether machines can become sentient [is important] for ethical reasons. If computers experience life through their own senses, they cease to be purely a means to an end determined by their usefulness to... humans. Per GNW [the Global Neuronal Workspace theory], they turn from mere objects into subjects... with a point of view.... Once computers' cognitive abilities rival those of humanity, their impulse to push for legal and political rights will become irresistible – the right not to be deleted, not to have their memories wiped clean, not to suffer pain and degradation. The alternative, embodied by IIT [Integrated Information Theory], is that computers will remain only supersophisticated machinery, ghostlike empty shells, devoid of what we value most: the feeling of life itself." (p. 49.) Marcus, Gary, "Am I Human?: Researchers need new ways to distinguish artificial intelligence from the natural kind", Scientific American, vol. 316, no. 3 (March 2017), pp. 58–63. A stumbling block to AI has been an incapacity for reliable disambiguation. An example is the "pronoun disambiguation problem": a machine has no way of determining to whom or what a pronoun in a sentence refers. (p. 61.) E McGaughey, 'Will Robots Automate Your Job Away? Full Employment, Basic Income, and Economic Democracy' (2018) SSRN, part 2(3) Archived 24 May 2018 at the Wayback Machine. George Musser, "Artificial Imagination: How machines could learn creativity and common sense, among other human qualities", Scientific American, vol. 320, no. 5 (May 2019), pp. 58–63. Myers, Courtney Boyd ed. (2009). "The AI Report" Archived 29 July 2017 at the Wayback Machine. Forbes June 2009 Raphael, Bertram (1976). The Thinking Computer. W.H.Freeman and Company. ISBN 978-0-7167-0723-3. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Scharre, Paul, "Killer Apps: The Real Dangers of an AI Arms Race", Foreign Affairs, vol. 98, no. 3 (May/June 2019), pp. 135–44. "Today's AI technologies are powerful but unreliable. Rules-based systems cannot deal with circumstances their programmers did not anticipate. Learning systems are limited by the data on which they were trained. AI failures have already led to tragedy. Advanced autopilot features in cars, although they perform well in some circumstances, have driven cars without warning into trucks, concrete barriers, and parked cars. In the wrong situation, AI systems go from supersmart to superdumb in an instant. When an enemy is trying to manipulate and hack an AI system, the risks are even greater." (p. 140.) Serenko, Alexander (2010). "The development of an AI journal ranking based on the revealed preference approach" (PDF). Journal of Informetrics. 4 (4): 447–459. doi:10.1016/j.joi.2010.04.001. Archived (PDF) from the original on 4 October 2013. Retrieved 24 August 2013. Serenko, Alexander; Michael Dohan (2011). "Comparing the expert survey and citation impact journal ranking methods: Example from the field of Artificial Intelligence" (PDF). Journal of Informetrics. 5 (4): 629–649. doi:10.1016/j.joi.2011.06.002. Archived (PDF) from the original on 4 October 2013. Retrieved 12 September 2013. Sun, R. &amp; Bookman, L. (eds.), Computational Architectures: Integrating Neural and Symbolic Processes. Kluwer Academic Publishers, Needham, MA. 1994. Tom Simonite (29 December 2014). "2014 in Computing: Breakthroughs in Artificial Intelligence". MIT Technology Review. Tooze, Adam, "Democracy and Its Discontents", The New York Review of Books, vol. LXVI, no. 10 (6 June 2019), pp. 52–53, 56–57. "Democracy has no clear answer for the mindless operation of bureaucratic and technological power. We may indeed be witnessing its extension in the form of artificial intelligence and robotics. Likewise, after decades of dire warning, the environmental problem remains fundamentally unaddressed.... Bureaucratic overreach and environmental catastrophe are precisely the kinds of slow-moving existential challenges that democracies deal with very badly.... Finally, there is the threat du jour: corporations and the technologies they promote." (pp. 56–57.)</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>https://github.com/RITRedteam/StreetCred</t>
+          <t>https://github.com/Aryia-Behroziuan/Other-sources</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Go</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>2026-05-23T10:52:29Z</t>
+          <t>2026-06-07T17:35:25Z</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>clides/Hacking-Books</t>
+          <t>kayranfatih/awesome-iot-and-hardware-security</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -10000,12 +10000,12 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>My collection of hacking books for learning information security</t>
+          <t>A collection of awesome tools, books, resources, software, documents and cool stuff about IoT and HW security.</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>https://github.com/clides/Hacking-Books</t>
+          <t>https://github.com/kayranfatih/awesome-iot-and-hardware-security</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10015,14 +10015,14 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>2026-06-06T12:48:50Z</t>
+          <t>2026-06-13T04:39:34Z</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Aryia-Behroziuan/Other-sources</t>
+          <t>clides/Hacking-Books</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -10030,12 +10030,12 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Asada, M.; Hosoda, K.; Kuniyoshi, Y.; Ishiguro, H.; Inui, T.; Yoshikawa, Y.; Ogino, M.; Yoshida, C. (2009). "Cognitive developmental robotics: a survey". IEEE Transactions on Autonomous Mental Development. 1 (1): 12–34. doi:10.1109/tamd.2009.2021702. S2CID 10168773. "ACM Computing Classification System: Artificial intelligence". ACM. 1998. Archived from the original on 12 October 2007. Retrieved 30 August 2007. Goodman, Joanna (2016). Robots in Law: How Artificial Intelligence is Transforming Legal Services (1st ed.). Ark Group. ISBN 978-1-78358-264-8. Archived from the original on 8 November 2016. Retrieved 7 November 2016. Albus, J. S. (2002). "4-D/RCS: A Reference Model Architecture for Intelligent Unmanned Ground Vehicles" (PDF). In Gerhart, G.; Gunderson, R.; Shoemaker, C. (eds.). Proceedings of the SPIE AeroSense Session on Unmanned Ground Vehicle Technology. Unmanned Ground Vehicle Technology IV. 3693. pp. 11–20. Bibcode:2002SPIE.4715..303A. CiteSeerX 10.1.1.15.14. doi:10.1117/12.474462. S2CID 63339739. Archived from the original (PDF) on 25 July 2004. Aleksander, Igor (1995). Artificial Neuroconsciousness: An Update. IWANN. Archived from the original on 2 March 1997. BibTex Archived 2 March 1997 at the Wayback Machine. Bach, Joscha (2008). "Seven Principles of Synthetic Intelligence". In Wang, Pei; Goertzel, Ben; Franklin, Stan (eds.). Artificial General Intelligence, 2008: Proceedings of the First AGI Conference. IOS Press. pp. 63–74. ISBN 978-1-58603-833-5. Archived from the original on 8 July 2016. Retrieved 16 February 2016. "Robots could demand legal rights". BBC News. 21 December 2006. Archived from the original on 15 October 2019. Retrieved 3 February 2011. Brooks, Rodney (1990). "Elephants Don't Play Chess" (PDF). Robotics and Autonomous Systems. 6 (1–2): 3–15. CiteSeerX 10.1.1.588.7539. doi:10.1016/S0921-8890(05)80025-9. Archived (PDF) from the original on 9 August 2007. Brooks, R. A. (1991). "How to build complete creatures rather than isolated cognitive simulators". In VanLehn, K. (ed.). Architectures for Intelligence. Hillsdale, NJ: Lawrence Erlbaum Associates. pp. 225–239. CiteSeerX 10.1.1.52.9510. Buchanan, Bruce G. (2005). "A (Very) Brief History of Artificial Intelligence" (PDF). AI Magazine: 53–60. Archived from the original (PDF) on 26 September 2007. Butler, Samuel (13 June 1863). "Darwin among the Machines". Letters to the Editor. The Press. Christchurch, New Zealand. Archived from the original on 19 September 2008. Retrieved 16 October 2014 – via Victoria University of Wellington. Clark, Jack (8 December 2015). "Why 2015 Was a Breakthrough Year in Artificial Intelligence". Bloomberg News. Archived from the original on 23 November 2016. Retrieved 23 November 2016. After a half-decade of quiet breakthroughs in artificial intelligence, 2015 has been a landmark year. Computers are smarter and learning faster than ever. "AI set to exceed human brain power". CNN. 26 July 2006. Archived from the original on 19 February 2008. Dennett, Daniel (1991). Consciousness Explained. The Penguin Press. ISBN 978-0-7139-9037-9. Domingos, Pedro (2015). The Master Algorithm: How the Quest for the Ultimate Learning Machine Will Remake Our World. Basic Books. ISBN 978-0-465-06192-1. Dowe, D. L.; Hajek, A. R. (1997). "A computational extension to the Turing Test". Proceedings of the 4th Conference of the Australasian Cognitive Science Society. Archived from the original on 28 June 2011. Dreyfus, Hubert (1972). What Computers Can't Do. New York: MIT Press. ISBN 978-0-06-011082-6. Dreyfus, Hubert; Dreyfus, Stuart (1986). Mind over Machine: The Power of Human Intuition and Expertise in the Era of the Computer. Oxford, UK: Blackwell. ISBN 978-0-02-908060-3. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Dreyfus, Hubert (1992). What Computers Still Can't Do. New York: MIT Press. ISBN 978-0-262-54067-4. Dyson, George (1998). Darwin among the Machines. Allan Lane Science. ISBN 978-0-7382-0030-9. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Edelman, Gerald (23 November 2007). "Gerald Edelman – Neural Darwinism and Brain-based Devices". Talking Robots. Archived from the original on 8 October 2009. Edelson, Edward (1991). The Nervous System. New York: Chelsea House. ISBN 978-0-7910-0464-7. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Fearn, Nicholas (2007). The Latest Answers to the Oldest Questions: A Philosophical Adventure with the World's Greatest Thinkers. New York: Grove Press. ISBN 978-0-8021-1839-4. Gladwell, Malcolm (2005). Blink. New York: Little, Brown and Co. ISBN 978-0-316-17232-5. Gödel, Kurt (1951). Some basic theorems on the foundations of mathematics and their implications. Gibbs Lecture. In Feferman, Solomon, ed. (1995). Kurt Gödel: Collected Works, Vol. III: Unpublished Essays and Lectures. Oxford University Press. pp. 304–23. ISBN 978-0-19-514722-3. Haugeland, John (1985). Artificial Intelligence: The Very Idea. Cambridge, Mass.: MIT Press. ISBN 978-0-262-08153-5. Hawkins, Jeff; Blakeslee, Sandra (2005). On Intelligence. New York, NY: Owl Books. ISBN 978-0-8050-7853-4. Henderson, Mark (24 April 2007). "Human rights for robots? We're getting carried away". The Times Online. London. Archived from the original on 31 May 2014. Retrieved 31 May 2014. Hernandez-Orallo, Jose (2000). "Beyond the Turing Test". Journal of Logic, Language and Information. 9 (4): 447–466. doi:10.1023/A:1008367325700. S2CID 14481982. Hernandez-Orallo, J.; Dowe, D. L. (2010). "Measuring Universal Intelligence: Towards an Anytime Intelligence Test". Artificial Intelligence. 174 (18): 1508–1539. CiteSeerX 10.1.1.295.9079. doi:10.1016/j.artint.2010.09.006. Hinton, G. E. (2007). "Learning multiple layers of representation". Trends in Cognitive Sciences. 11 (10): 428–434. doi:10.1016/j.tics.2007.09.004. PMID 17921042. S2CID 15066318. Hofstadter, Douglas (1979). Gödel, Escher, Bach: an Eternal Golden Braid. New York, NY: Vintage Books. ISBN 978-0-394-74502-2. Holland, John H. (1975). Adaptation in Natural and Artificial Systems. University of Michigan Press. ISBN 978-0-262-58111-0. Archived from the original on 26 July 2020. Retrieved 17 December 2019. Howe, J. (November 1994). "Artificial Intelligence at Edinburgh University: a Perspective". Archived from the original on 15 May 2007. Retrieved 30 August 2007. Hutter, M. (2012). "One Decade of Universal Artificial Intelligence". Theoretical Foundations of Artificial General Intelligence. Atlantis Thinking Machines. 4. pp. 67–88. CiteSeerX 10.1.1.228.8725. doi:10.2991/978-94-91216-62-6_5. ISBN 978-94-91216-61-9. S2CID 8888091. Kahneman, Daniel; Slovic, D.; Tversky, Amos (1982). Judgment under uncertainty: Heuristics and biases. Science. 185. New York: Cambridge University Press. pp. 1124–31. doi:10.1126/science.185.4157.1124. ISBN 978-0-521-28414-1. PMID 17835457. S2CID 143452957. Kaplan, Andreas; Haenlein, Michael (2019). "Siri, Siri in my Hand, who's the Fairest in the Land? On the Interpretations, Illustrations and Implications of Artificial Intelligence". Business Horizons. 62: 15–25. doi:10.1016/j.bushor.2018.08.004. Katz, Yarden (1 November 2012). "Noam Chomsky on Where Artificial Intelligence Went Wrong". The Atlantic. Archived from the original on 28 February 2019. Retrieved 26 October 2014. "Kismet". MIT Artificial Intelligence Laboratory, Humanoid Robotics Group. Archived from the original on 17 October 2014. Retrieved 25 October 2014. Koza, John R. (1992). Genetic Programming (On the Programming of Computers by Means of Natural Selection). MIT Press. Bibcode:1992gppc.book.....K. ISBN 978-0-262-11170-6. Kolata, G. (1982). "How can computers get common sense?". Science. 217 (4566): 1237–1238. Bibcode:1982Sci...217.1237K. doi:10.1126/science.217.4566.1237. PMID 17837639. Kumar, Gulshan; Kumar, Krishan (2012). "The Use of Artificial-Intelligence-Based Ensembles for Intrusion Detection: A Review". Applied Computational Intelligence and Soft Computing. 2012: 1–20. doi:10.1155/2012/850160. Kurzweil, Ray (1999). The Age of Spiritual Machines. Penguin Books. ISBN 978-0-670-88217-5. Kurzweil, Ray (2005). The Singularity is Near. Penguin Books. ISBN 978-0-670-03384-3. Lakoff, George; Núñez, Rafael E. (2000). Where Mathematics Comes From: How the Embodied Mind Brings Mathematics into Being. Basic Books. ISBN 978-0-465-03771-1. Langley, Pat (2011). "The changing science of machine learning". Machine Learning. 82 (3): 275–279. doi:10.1007/s10994-011-5242-y. Law, Diane (June 1994). Searle, Subsymbolic Functionalism and Synthetic Intelligence (Technical report). University of Texas at Austin. p. AI94-222. CiteSeerX 10.1.1.38.8384. Legg, Shane; Hutter, Marcus (15 June 2007). A Collection of Definitions of Intelligence (Technical report). IDSIA. arXiv:0706.3639. Bibcode:2007arXiv0706.3639L. 07-07. Lenat, Douglas; Guha, R. V. (1989). Building Large Knowledge-Based Systems. Addison-Wesley. ISBN 978-0-201-51752-1. Lighthill, James (1973). "Artificial Intelligence: A General Survey". Artificial Intelligence: a paper symposium. Science Research Council. Lucas, John (1961). "Minds, Machines and Gödel". In Anderson, A.R. (ed.). Minds and Machines. Archived from the original on 19 August 2007. Retrieved 30 August 2007. Lungarella, M.; Metta, G.; Pfeifer, R.; Sandini, G. (2003). "Developmental robotics: a survey". Connection Science. 15 (4): 151–190. CiteSeerX 10.1.1.83.7615. doi:10.1080/09540090310001655110. S2CID 1452734. Maker, Meg Houston (2006). "AI@50: AI Past, Present, Future". Dartmouth College. Archived from the original on 3 January 2007. Retrieved 16 October 2008. Markoff, John (16 February 2011). "Computer Wins on 'Jeopardy!': Trivial, It's Not". The New York Times. Archived from the original on 22 October 2014. Retrieved 25 October 2014. McCarthy, John; Minsky, Marvin; Rochester, Nathan; Shannon, Claude (1955). "A Proposal for the Dartmouth Summer Research Project on Artificial Intelligence". Archived from the original on 26 August 2007. Retrieved 30 August 2007.. McCarthy, John; Hayes, P. J. (1969). "Some philosophical problems from the standpoint of artificial intelligence". Machine Intelligence. 4: 463–502. CiteSeerX 10.1.1.85.5082. Archived from the original on 10 August 2007. Retrieved 30 August 2007. McCarthy, John (12 November 2007). "What Is Artificial Intelligence?". Archived from the original on 18 November 2015. Minsky, Marvin (1967). Computation: Finite and Infinite Machines. Englewood Cliffs, N.J.: Prentice-Hall. ISBN 978-0-13-165449-5. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Minsky, Marvin (2006). The Emotion Machine. New York, NY: Simon &amp; Schusterl. ISBN 978-0-7432-7663-4. Moravec, Hans (1988). Mind Children. Harvard University Press. ISBN 978-0-674-57616-2. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Norvig, Peter (25 June 2012). "On Chomsky and the Two Cultures of Statistical Learning". Peter Norvig. Archived from the original on 19 October 2014. NRC (United States National Research Council) (1999). "Developments in Artificial Intelligence". Funding a Revolution: Government Support for Computing Research. National Academy Press. Needham, Joseph (1986). Science and Civilization in China: Volume 2. Caves Books Ltd. Newell, Allen; Simon, H. A. (1976). "Computer Science as Empirical Inquiry: Symbols and Search". Communications of the ACM. 19 (3): 113–126. doi:10.1145/360018.360022.. Nilsson, Nils (1983). "Artificial Intelligence Prepares for 2001" (PDF). AI Magazine. 1 (1). Archived (PDF) from the original on 17 August 2020. Retrieved 22 August 2020. Presidential Address to the Association for the Advancement of Artificial Intelligence. O'Brien, James; Marakas, George (2011). Management Information Systems (10th ed.). McGraw-Hill/Irwin. ISBN 978-0-07-337681-3. O'Connor, Kathleen Malone (1994). "The alchemical creation of life (takwin) and other concepts of Genesis in medieval Islam". University of Pennsylvania: 1–435. Archived from the original on 5 December 2019. Retrieved 27 August 2008. Oudeyer, P-Y. (2010). "On the impact of robotics in behavioral and cognitive sciences: from insect navigation to human cognitive development" (PDF). IEEE Transactions on Autonomous Mental Development. 2 (1): 2–16. doi:10.1109/tamd.2009.2039057. S2CID 6362217. Archived (PDF) from the original on 3 October 2018. Retrieved 4 June 2013. Penrose, Roger (1989). The Emperor's New Mind: Concerning Computer, Minds and The Laws of Physics. Oxford University Press. ISBN 978-0-19-851973-7. Poli, R.; Langdon, W. B.; McPhee, N. F. (2008). A Field Guide to Genetic Programming. Lulu.com. ISBN 978-1-4092-0073-4. Archived from the original on 8 August 2015. Retrieved 21 April 2008 – via gp-field-guide.org.uk. Rajani, Sandeep (2011). "Artificial Intelligence – Man or Machine" (PDF). International Journal of Information Technology and Knowledge Management. 4 (1): 173–176. Archived from the original (PDF) on 18 January 2013. Ronald, E. M. A. and Sipper, M. Intelligence is not enough: On the socialization of talking machines, Minds and Machines Archived 25 July 2020 at the Wayback Machine, vol. 11, no. 4, pp. 567–576, November 2001. Ronald, E. M. A. and Sipper, M. What use is a Turing chatterbox? Archived 25 July 2020 at the Wayback Machine, Communications of the ACM, vol. 43, no. 10, pp. 21–23, October 2000. "Science". August 1982. Archived from the original on 25 July 2020. Retrieved 16 February 2016. Searle, John (1980). "Minds, Brains and Programs" (PDF). Behavioral and Brain Sciences. 3 (3): 417–457. doi:10.1017/S0140525X00005756. Archived (PDF) from the original on 17 March 2019. Retrieved 22 August 2020. Searle, John (1999). Mind, language and society. New York, NY: Basic Books. ISBN 978-0-465-04521-1. OCLC 231867665. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Shapiro, Stuart C. (1992). "Artificial Intelligence". In Shapiro, Stuart C. (ed.). Encyclopedia of Artificial Intelligence (PDF) (2nd ed.). New York: John Wiley. pp. 54–57. ISBN 978-0-471-50306-4. Archived (PDF) from the original on 1 February 2016. Retrieved 29 May 2009. Simon, H. A. (1965). The Shape of Automation for Men and Management. New York: Harper &amp; Row. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Skillings, Jonathan (3 July 2006). "Getting Machines to Think Like Us". cnet. Archived from the original on 16 November 2011. Retrieved 3 February 2011. Solomonoff, Ray (1956). An Inductive Inference Machine (PDF). Dartmouth Summer Research Conference on Artificial Intelligence. Archived (PDF) from the original on 26 April 2011. Retrieved 22 March 2011 – via std.com, pdf scanned copy of the original. Later published as Solomonoff, Ray (1957). "An Inductive Inference Machine". IRE Convention Record. Section on Information Theory, part 2. pp. 56–62. Tao, Jianhua; Tan, Tieniu (2005). Affective Computing and Intelligent Interaction. Affective Computing: A Review. LNCS 3784. Springer. pp. 981–995. doi:10.1007/11573548. Tecuci, Gheorghe (March–April 2012). "Artificial Intelligence". Wiley Interdisciplinary Reviews: Computational Statistics. 4 (2): 168–180. doi:10.1002/wics.200. Thro, Ellen (1993). Robotics: The Marriage of Computers and Machines. New York: Facts on File. ISBN 978-0-8160-2628-9. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Turing, Alan (October 1950), "Computing Machinery and Intelligence", Mind, LIX (236): 433–460, doi:10.1093/mind/LIX.236.433, ISSN 0026-4423. van der Walt, Christiaan; Bernard, Etienne (2006). "Data characteristics that determine classifier performance" (PDF). Archived from the original (PDF) on 25 March 2009. Retrieved 5 August 2009. Vinge, Vernor (1993). "The Coming Technological Singularity: How to Survive in the Post-Human Era". Vision 21: Interdisciplinary Science and Engineering in the Era of Cyberspace: 11. Bibcode:1993vise.nasa...11V. Archived from the original on 1 January 2007. Retrieved 14 November 2011. Wason, P. C.; Shapiro, D. (1966). "Reasoning". In Foss, B. M. (ed.). New horizons in psychology. Harmondsworth: Penguin. Archived from the original on 26 July 2020. Retrieved 18 November 2019. Weizenbaum, Joseph (1976). Computer Power and Human Reason. San Francisco: W.H. Freeman &amp; Company. ISBN 978-0-7167-0464-5. Weng, J.; McClelland; Pentland, A.; Sporns, O.; Stockman, I.; Sur, M.; Thelen, E. (2001). "Autonomous mental development by robots and animals" (PDF). Science. 291 (5504): 599–600. doi:10.1126/science.291.5504.599. PMID 11229402. S2CID 54131797. Archived (PDF) from the original on 4 September 2013. Retrieved 4 June 2013 – via msu.edu. "Applications of AI". www-formal.stanford.edu. Archived from the original on 28 August 2016. Retrieved 25 September 2016. Further reading DH Author, 'Why Are There Still So Many Jobs? The History and Future of Workplace Automation' (2015) 29(3) Journal of Economic Perspectives 3. Boden, Margaret, Mind As Machine, Oxford University Press, 2006. Cukier, Kenneth, "Ready for Robots? How to Think about the Future of AI", Foreign Affairs, vol. 98, no. 4 (July/August 2019), pp. 192–98. George Dyson, historian of computing, writes (in what might be called "Dyson's Law") that "Any system simple enough to be understandable will not be complicated enough to behave intelligently, while any system complicated enough to behave intelligently will be too complicated to understand." (p. 197.) Computer scientist Alex Pentland writes: "Current AI machine-learning algorithms are, at their core, dead simple stupid. They work, but they work by brute force." (p. 198.) Domingos, Pedro, "Our Digital Doubles: AI will serve our species, not control it", Scientific American, vol. 319, no. 3 (September 2018), pp. 88–93. Gopnik, Alison, "Making AI More Human: Artificial intelligence has staged a revival by starting to incorporate what we know about how children learn", Scientific American, vol. 316, no. 6 (June 2017), pp. 60–65. Johnston, John (2008) The Allure of Machinic Life: Cybernetics, Artificial Life, and the New AI, MIT Press. Koch, Christof, "Proust among the Machines", Scientific American, vol. 321, no. 6 (December 2019), pp. 46–49. Christof Koch doubts the possibility of "intelligent" machines attaining consciousness, because "[e]ven the most sophisticated brain simulations are unlikely to produce conscious feelings." (p. 48.) According to Koch, "Whether machines can become sentient [is important] for ethical reasons. If computers experience life through their own senses, they cease to be purely a means to an end determined by their usefulness to... humans. Per GNW [the Global Neuronal Workspace theory], they turn from mere objects into subjects... with a point of view.... Once computers' cognitive abilities rival those of humanity, their impulse to push for legal and political rights will become irresistible – the right not to be deleted, not to have their memories wiped clean, not to suffer pain and degradation. The alternative, embodied by IIT [Integrated Information Theory], is that computers will remain only supersophisticated machinery, ghostlike empty shells, devoid of what we value most: the feeling of life itself." (p. 49.) Marcus, Gary, "Am I Human?: Researchers need new ways to distinguish artificial intelligence from the natural kind", Scientific American, vol. 316, no. 3 (March 2017), pp. 58–63. A stumbling block to AI has been an incapacity for reliable disambiguation. An example is the "pronoun disambiguation problem": a machine has no way of determining to whom or what a pronoun in a sentence refers. (p. 61.) E McGaughey, 'Will Robots Automate Your Job Away? Full Employment, Basic Income, and Economic Democracy' (2018) SSRN, part 2(3) Archived 24 May 2018 at the Wayback Machine. George Musser, "Artificial Imagination: How machines could learn creativity and common sense, among other human qualities", Scientific American, vol. 320, no. 5 (May 2019), pp. 58–63. Myers, Courtney Boyd ed. (2009). "The AI Report" Archived 29 July 2017 at the Wayback Machine. Forbes June 2009 Raphael, Bertram (1976). The Thinking Computer. W.H.Freeman and Company. ISBN 978-0-7167-0723-3. Archived from the original on 26 July 2020. Retrieved 22 August 2020. Scharre, Paul, "Killer Apps: The Real Dangers of an AI Arms Race", Foreign Affairs, vol. 98, no. 3 (May/June 2019), pp. 135–44. "Today's AI technologies are powerful but unreliable. Rules-based systems cannot deal with circumstances their programmers did not anticipate. Learning systems are limited by the data on which they were trained. AI failures have already led to tragedy. Advanced autopilot features in cars, although they perform well in some circumstances, have driven cars without warning into trucks, concrete barriers, and parked cars. In the wrong situation, AI systems go from supersmart to superdumb in an instant. When an enemy is trying to manipulate and hack an AI system, the risks are even greater." (p. 140.) Serenko, Alexander (2010). "The development of an AI journal ranking based on the revealed preference approach" (PDF). Journal of Informetrics. 4 (4): 447–459. doi:10.1016/j.joi.2010.04.001. Archived (PDF) from the original on 4 October 2013. Retrieved 24 August 2013. Serenko, Alexander; Michael Dohan (2011). "Comparing the expert survey and citation impact journal ranking methods: Example from the field of Artificial Intelligence" (PDF). Journal of Informetrics. 5 (4): 629–649. doi:10.1016/j.joi.2011.06.002. Archived (PDF) from the original on 4 October 2013. Retrieved 12 September 2013. Sun, R. &amp; Bookman, L. (eds.), Computational Architectures: Integrating Neural and Symbolic Processes. Kluwer Academic Publishers, Needham, MA. 1994. Tom Simonite (29 December 2014). "2014 in Computing: Breakthroughs in Artificial Intelligence". MIT Technology Review. Tooze, Adam, "Democracy and Its Discontents", The New York Review of Books, vol. LXVI, no. 10 (6 June 2019), pp. 52–53, 56–57. "Democracy has no clear answer for the mindless operation of bureaucratic and technological power. We may indeed be witnessing its extension in the form of artificial intelligence and robotics. Likewise, after decades of dire warning, the environmental problem remains fundamentally unaddressed.... Bureaucratic overreach and environmental catastrophe are precisely the kinds of slow-moving existential challenges that democracies deal with very badly.... Finally, there is the threat du jour: corporations and the technologies they promote." (pp. 56–57.)</t>
+          <t>My collection of hacking books for learning information security</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>https://github.com/Aryia-Behroziuan/Other-sources</t>
+          <t>https://github.com/clides/Hacking-Books</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10045,14 +10045,14 @@
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-06-07T17:35:25Z</t>
+          <t>2026-06-06T12:48:50Z</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>ShoshinMaster/cybersec-hub-2026</t>
+          <t>h33tlit/SniffCon-Ultimate-Recon-Dashboard-For-Bug-Bounty-And-Pentesting</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -10060,29 +10060,29 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Self-hosted cybersecurity dashboard to organize learning resources, tools, news and certifications. A personal hub to centralize and manage all cybersecurity resources.</t>
+          <t>Sniffcon has a wide list of powerful online bug bounty tools which can be used to find security vulnerabilities.</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>https://github.com/ShoshinMaster/cybersec-hub-2026</t>
+          <t>https://github.com/h33tlit/SniffCon-Ultimate-Recon-Dashboard-For-Bug-Bounty-And-Pentesting</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>JavaScript</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>2026-05-06T19:31:38Z</t>
+          <t>2026-05-27T11:49:20Z</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>h33tlit/SniffCon-Ultimate-Recon-Dashboard-For-Bug-Bounty-And-Pentesting</t>
+          <t>RITRedteam/StreetCred</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -10090,29 +10090,29 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Sniffcon has a wide list of powerful online bug bounty tools which can be used to find security vulnerabilities.</t>
+          <t>Tool created for Red Team to test default credentials on SSH and WinRM and then execute scripts with those credentials before the password can be changed by Blue Team.</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>https://github.com/h33tlit/SniffCon-Ultimate-Recon-Dashboard-For-Bug-Bounty-And-Pentesting</t>
+          <t>https://github.com/RITRedteam/StreetCred</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Go</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>2026-05-27T11:49:20Z</t>
+          <t>2026-05-23T10:52:29Z</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>kayranfatih/awesome-iot-and-hardware-security</t>
+          <t>ShoshinMaster/cybersec-hub-2026</t>
         </is>
       </c>
       <c r="B324" t="n">
@@ -10120,22 +10120,22 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>A collection of awesome tools, books, resources, software, documents and cool stuff about IoT and HW security.</t>
+          <t>Self-hosted cybersecurity dashboard to organize learning resources, tools, news and certifications. A personal hub to centralize and manage all cybersecurity resources.</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>https://github.com/kayranfatih/awesome-iot-and-hardware-security</t>
+          <t>https://github.com/ShoshinMaster/cybersec-hub-2026</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>JavaScript</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>2026-06-13T04:39:34Z</t>
+          <t>2026-05-06T19:31:38Z</t>
         </is>
       </c>
     </row>
@@ -10172,7 +10172,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Asterisk369/Top-20-Free-H4CKING-learn-books</t>
+          <t>ryanmrestivo/blue-team</t>
         </is>
       </c>
       <c r="B326" t="n">
@@ -10180,29 +10180,29 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>A curated list of 20 free hacking books that cover various aspects of cybersecurity, ethical hacking, and penetration testing. This repository aims to provide valuable resources for beginners and experienced professionals alike.</t>
+          <t>Some portable tools, some YARA, some Python, and a little bit of love.  Not all of these tools can be used in incident response.  Use PEs with caution.</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>https://github.com/Asterisk369/Top-20-Free-H4CKING-learn-books</t>
+          <t>https://github.com/ryanmrestivo/blue-team</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>YARA</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>2026-06-07T14:29:06Z</t>
+          <t>2026-02-18T05:25:13Z</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>brinhosa/awesome-pentest-tools-in-colab</t>
+          <t>Asterisk369/Top-20-Free-H4CKING-learn-books</t>
         </is>
       </c>
       <c r="B327" t="n">
@@ -10210,29 +10210,29 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>A curated list of awesome Penetration Testing Tools ported to Google Colab to make faster and easier to execute and test.</t>
+          <t>A curated list of 20 free hacking books that cover various aspects of cybersecurity, ethical hacking, and penetration testing. This repository aims to provide valuable resources for beginners and experienced professionals alike.</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>https://github.com/brinhosa/awesome-pentest-tools-in-colab</t>
+          <t>https://github.com/Asterisk369/Top-20-Free-H4CKING-learn-books</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Jupyter Notebook</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>2026-05-05T01:10:09Z</t>
+          <t>2026-06-07T14:29:06Z</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>ryanmrestivo/blue-team</t>
+          <t>brinhosa/awesome-pentest-tools-in-colab</t>
         </is>
       </c>
       <c r="B328" t="n">
@@ -10240,29 +10240,29 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Some portable tools, some YARA, some Python, and a little bit of love.  Not all of these tools can be used in incident response.  Use PEs with caution.</t>
+          <t>A curated list of awesome Penetration Testing Tools ported to Google Colab to make faster and easier to execute and test.</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>https://github.com/ryanmrestivo/blue-team</t>
+          <t>https://github.com/brinhosa/awesome-pentest-tools-in-colab</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>YARA</t>
+          <t>Jupyter Notebook</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>2026-02-18T05:25:13Z</t>
+          <t>2026-05-05T01:10:09Z</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-security-harderning</t>
+          <t>paulveillard/cybersecurity-dast</t>
         </is>
       </c>
       <c r="B329" t="n">
@@ -10270,29 +10270,29 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>A collection of awesome security hardening software, libraries, learning tutorials &amp; documents, e-books, best practices, checklists, benchmarks about hardening in Cybersecurity</t>
+          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Dynamic Application Security Testing (DAST) Tools.</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-security-harderning</t>
+          <t>https://github.com/paulveillard/cybersecurity-dast</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>2026-05-04T17:14:15Z</t>
+          <t>2026-06-01T12:21:26Z</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-dast</t>
+          <t>paulveillard/cybersecurity-security-harderning</t>
         </is>
       </c>
       <c r="B330" t="n">
@@ -10300,22 +10300,22 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Dynamic Application Security Testing (DAST) Tools.</t>
+          <t>A collection of awesome security hardening software, libraries, learning tutorials &amp; documents, e-books, best practices, checklists, benchmarks about hardening in Cybersecurity</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-dast</t>
+          <t>https://github.com/paulveillard/cybersecurity-security-harderning</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>2026-06-01T12:21:26Z</t>
+          <t>2026-05-04T17:14:15Z</t>
         </is>
       </c>
     </row>
@@ -10382,7 +10382,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>lugnitdgp/CTF-Learning-Resources</t>
+          <t>kraloveckey/venom</t>
         </is>
       </c>
       <c r="B333" t="n">
@@ -10390,29 +10390,29 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>All kinds of infosec learning related stuff.</t>
+          <t>👽 The collection of awesome software, tools, libraries, documents, books, resources and cool stuff about information security, penetration testing and offensive cybersecurity.</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>https://github.com/lugnitdgp/CTF-Learning-Resources</t>
+          <t>https://github.com/kraloveckey/venom</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>2026-03-22T21:39:01Z</t>
+          <t>2026-05-30T14:32:35Z</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>verylazytech/Hacking-Books-2024</t>
+          <t>lugnitdgp/CTF-Learning-Resources</t>
         </is>
       </c>
       <c r="B334" t="n">
@@ -10420,12 +10420,12 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Top Hacking Books for 2024 (plus Resources): FREE and Paid</t>
+          <t>All kinds of infosec learning related stuff.</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>https://github.com/verylazytech/Hacking-Books-2024</t>
+          <t>https://github.com/lugnitdgp/CTF-Learning-Resources</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -10435,14 +10435,14 @@
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>2026-04-30T18:38:58Z</t>
+          <t>2026-03-22T21:39:01Z</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>kraloveckey/venom</t>
+          <t>verylazytech/Hacking-Books-2024</t>
         </is>
       </c>
       <c r="B335" t="n">
@@ -10450,22 +10450,22 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>👽 The collection of awesome software, tools, libraries, documents, books, resources and cool stuff about information security, penetration testing and offensive cybersecurity.</t>
+          <t>Top Hacking Books for 2024 (plus Resources): FREE and Paid</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>https://github.com/kraloveckey/venom</t>
+          <t>https://github.com/verylazytech/Hacking-Books-2024</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>2026-05-30T14:32:35Z</t>
+          <t>2026-04-30T18:38:58Z</t>
         </is>
       </c>
     </row>
@@ -10502,7 +10502,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>keitersecurity/awesome-infosec</t>
+          <t>legoffant/reverseengineering</t>
         </is>
       </c>
       <c r="B337" t="n">
@@ -10510,12 +10510,12 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>A curated list of information security resources</t>
+          <t>Books for hacker in reverse engineering</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>https://github.com/keitersecurity/awesome-infosec</t>
+          <t>https://github.com/legoffant/reverseengineering</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -10525,7 +10525,7 @@
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>2026-05-20T13:22:34Z</t>
+          <t>2026-03-19T19:11:47Z</t>
         </is>
       </c>
     </row>
@@ -10562,7 +10562,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>legoffant/reverseengineering</t>
+          <t>dcarlin/Blue-Team-Tools</t>
         </is>
       </c>
       <c r="B339" t="n">
@@ -10570,12 +10570,12 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Books for hacker in reverse engineering</t>
+          <t>This contains a list of Blue Team Tools that I use daily, and have stored here for reference.</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>https://github.com/legoffant/reverseengineering</t>
+          <t>https://github.com/dcarlin/Blue-Team-Tools</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -10585,14 +10585,14 @@
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>2026-03-19T19:11:47Z</t>
+          <t>2025-11-28T19:59:04Z</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>dcarlin/Blue-Team-Tools</t>
+          <t>keitersecurity/awesome-infosec</t>
         </is>
       </c>
       <c r="B340" t="n">
@@ -10600,12 +10600,12 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>This contains a list of Blue Team Tools that I use daily, and have stored here for reference.</t>
+          <t>A curated list of information security resources</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>https://github.com/dcarlin/Blue-Team-Tools</t>
+          <t>https://github.com/keitersecurity/awesome-infosec</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -10615,7 +10615,7 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>2025-11-28T19:59:04Z</t>
+          <t>2026-05-20T13:22:34Z</t>
         </is>
       </c>
     </row>
@@ -10652,7 +10652,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-exploit-development</t>
+          <t>keraattin/Blue-Team-Roadmap</t>
         </is>
       </c>
       <c r="B342" t="n">
@@ -10660,12 +10660,12 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Exploit Development.</t>
+          <t>The most comprehensive, step-by-step roadmap for breaking into defensive cybersecurity. From absolute zero to your first Blue Team role. Every skill, tool, certification, and resource you need. No experience required.</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-exploit-development</t>
+          <t>https://github.com/keraattin/Blue-Team-Roadmap</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -10675,14 +10675,14 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>2026-06-06T21:46:39Z</t>
+          <t>2026-06-13T15:25:40Z</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>pascalschulz/Infosec-Resources</t>
+          <t>paulveillard/cybersecurity-exploit-development</t>
         </is>
       </c>
       <c r="B343" t="n">
@@ -10690,12 +10690,12 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>just a little treasure chest of stuff I need to watch / read later</t>
+          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Exploit Development.</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>https://github.com/pascalschulz/Infosec-Resources</t>
+          <t>https://github.com/paulveillard/cybersecurity-exploit-development</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -10705,14 +10705,14 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>2025-03-19T06:51:25Z</t>
+          <t>2026-06-06T21:46:39Z</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>keraattin/Blue-Team-Roadmap</t>
+          <t>pascalschulz/Infosec-Resources</t>
         </is>
       </c>
       <c r="B344" t="n">
@@ -10720,12 +10720,12 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>The most comprehensive, step-by-step roadmap for breaking into defensive cybersecurity. From absolute zero to your first Blue Team role. Every skill, tool, certification, and resource you need. No experience required.</t>
+          <t>just a little treasure chest of stuff I need to watch / read later</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>https://github.com/keraattin/Blue-Team-Roadmap</t>
+          <t>https://github.com/pascalschulz/Infosec-Resources</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -10735,7 +10735,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>2026-06-13T15:25:40Z</t>
+          <t>2025-03-19T06:51:25Z</t>
         </is>
       </c>
     </row>
@@ -10802,7 +10802,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>pwnwriter/ebooks</t>
+          <t>paulveillard/cybersecurity-pcap-tools</t>
         </is>
       </c>
       <c r="B347" t="n">
@@ -10810,22 +10810,22 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Random pdfs and books which i may need later and forever.</t>
+          <t>A collection of awesome software, libraries, documents, books, resources and cool stuff about cybersecurity packet capture (PCAP) tools.</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>https://github.com/pwnwriter/ebooks</t>
+          <t>https://github.com/paulveillard/cybersecurity-pcap-tools</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>2026-01-26T19:21:12Z</t>
+          <t>2026-05-02T08:27:37Z</t>
         </is>
       </c>
     </row>
@@ -10862,7 +10862,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-pcap-tools</t>
+          <t>pwnwriter/ebooks</t>
         </is>
       </c>
       <c r="B349" t="n">
@@ -10870,22 +10870,22 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>A collection of awesome software, libraries, documents, books, resources and cool stuff about cybersecurity packet capture (PCAP) tools.</t>
+          <t>Random pdfs and books which i may need later and forever.</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-pcap-tools</t>
+          <t>https://github.com/pwnwriter/ebooks</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>2026-05-02T08:27:37Z</t>
+          <t>2026-01-26T19:21:12Z</t>
         </is>
       </c>
     </row>
@@ -10982,7 +10982,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>paulveillard/cybersecurity-pam</t>
+          <t>SagarBiswas-MultiHAT/Library-of-Cybersecurity-Books</t>
         </is>
       </c>
       <c r="B353" t="n">
@@ -10990,29 +10990,29 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Privileged Access Management (PAM) in Cybersecurity.</t>
+          <t>A free, no-paywall cybersecurity self-study library covering foundations, pentesting, web security, exploit development, malware analysis, cryptography, defense, and programming. Books are organized by domain and difficulty with a guided learning path so beginners can progress to advanced security skills independently.</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>https://github.com/paulveillard/cybersecurity-pam</t>
+          <t>https://github.com/SagarBiswas-MultiHAT/Library-of-Cybersecurity-Books</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-05-04T18:18:48Z</t>
+          <t>2026-06-09T05:19:39Z</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>SagarBiswas-MultiHAT/Library-of-Cybersecurity-Books</t>
+          <t>paulveillard/cybersecurity-pam</t>
         </is>
       </c>
       <c r="B354" t="n">
@@ -11020,22 +11020,22 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>A free, no-paywall cybersecurity self-study library covering foundations, pentesting, web security, exploit development, malware analysis, cryptography, defense, and programming. Books are organized by domain and difficulty with a guided learning path so beginners can progress to advanced security skills independently.</t>
+          <t>An ongoing &amp; curated collection of awesome software best practices and techniques, libraries and frameworks, E-books and videos, websites, blog posts, links to github Repositories, technical guidelines and important resources about Privileged Access Management (PAM) in Cybersecurity.</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>https://github.com/SagarBiswas-MultiHAT/Library-of-Cybersecurity-Books</t>
+          <t>https://github.com/paulveillard/cybersecurity-pam</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>PHP</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>2026-06-09T05:19:39Z</t>
+          <t>2026-05-04T18:18:48Z</t>
         </is>
       </c>
     </row>
@@ -11072,7 +11072,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>nerov103/Book</t>
+          <t>Errum/Intelligence-and-Cybersecurity-Peer-Reviewed-sources</t>
         </is>
       </c>
       <c r="B356" t="n">
@@ -11080,12 +11080,12 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Hacking Books</t>
+          <t>A list of Per-Reviewed Journals, Books and Blogs on intelligence and Cybersecurity</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>https://github.com/nerov103/Book</t>
+          <t>https://github.com/Errum/Intelligence-and-Cybersecurity-Peer-Reviewed-sources</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -11095,14 +11095,14 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>2026-06-09T00:07:25Z</t>
+          <t>2026-05-25T09:22:01Z</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Errum/Intelligence-and-Cybersecurity-Peer-Reviewed-sources</t>
+          <t>nerov103/Book</t>
         </is>
       </c>
       <c r="B357" t="n">
@@ -11110,12 +11110,12 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>A list of Per-Reviewed Journals, Books and Blogs on intelligence and Cybersecurity</t>
+          <t>Hacking Books</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>https://github.com/Errum/Intelligence-and-Cybersecurity-Peer-Reviewed-sources</t>
+          <t>https://github.com/nerov103/Book</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -11125,14 +11125,14 @@
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>2026-05-25T09:22:01Z</t>
+          <t>2026-06-09T00:07:25Z</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>SofianeHamlaoui/b-ok-scraper</t>
+          <t>binarymist/HolisticInfoSec-For-WebDevelopers-Fascicle1</t>
         </is>
       </c>
       <c r="B358" t="n">
@@ -11140,29 +11140,29 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>A b-ok.cc Simple Python Scraper</t>
+          <t>:books: VPS :lock: Network :lock: Cloud :lock: Web Applications :books:</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>https://github.com/SofianeHamlaoui/b-ok-scraper</t>
+          <t>https://github.com/binarymist/HolisticInfoSec-For-WebDevelopers-Fascicle1</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>2024-10-27T04:19:42Z</t>
+          <t>2026-05-04T10:51:37Z</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>binarymist/HolisticInfoSec-For-WebDevelopers-Fascicle1</t>
+          <t>SofianeHamlaoui/b-ok-scraper</t>
         </is>
       </c>
       <c r="B359" t="n">
@@ -11170,22 +11170,22 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>:books: VPS :lock: Network :lock: Cloud :lock: Web Applications :books:</t>
+          <t>A b-ok.cc Simple Python Scraper</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>https://github.com/binarymist/HolisticInfoSec-For-WebDevelopers-Fascicle1</t>
+          <t>https://github.com/SofianeHamlaoui/b-ok-scraper</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>2026-05-04T10:51:37Z</t>
+          <t>2024-10-27T04:19:42Z</t>
         </is>
       </c>
     </row>
@@ -11282,7 +11282,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>lsszz2100/VibeHacking</t>
+          <t>jassics/awesome-genai-security</t>
         </is>
       </c>
       <c r="B363" t="n">
@@ -11290,29 +11290,29 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>A Collection of Repositories, Videos, Books, and Lecture Materials to Learn Security &amp; Hacking with AI in a Fun Way</t>
+          <t>Curated list of links, references, books videos, tutorials (Free or Paid), Exploit, CTFs, Hacking Practices etc. which are related to GenAI and LLM Security</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>https://github.com/lsszz2100/VibeHacking</t>
+          <t>https://github.com/jassics/awesome-genai-security</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>2026-06-12T15:00:45Z</t>
+          <t>2026-06-11T08:54:48Z</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>N30nHaCkZ/linux</t>
+          <t>AlessandroMozzato/hn_books</t>
         </is>
       </c>
       <c r="B364" t="n">
@@ -11320,29 +11320,29 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Linux kernel release 3.x &lt;http://kernel.org/&gt;  These are the release notes for Linux version 3.  Read them carefully, as they tell you what this is all about, explain how to install the kernel, and what to do if something goes wrong.   WHAT IS LINUX?    Linux is a clone of the operating system Unix, written from scratch by   Linus Torvalds with assistance from a loosely-knit team of hackers across   the Net. It aims towards POSIX and Single UNIX Specification compliance.    It has all the features you would expect in a modern fully-fledged Unix,   including true multitasking, virtual memory, shared libraries, demand   loading, shared copy-on-write executables, proper memory management,   and multistack networking including IPv4 and IPv6.    It is distributed under the GNU General Public License - see the   accompanying COPYING file for more details.   ON WHAT HARDWARE DOES IT RUN?    Although originally developed first for 32-bit x86-based PCs (386 or higher),   today Linux also runs on (at least) the Compaq Alpha AXP, Sun SPARC and   UltraSPARC, Motorola 68000, PowerPC, PowerPC64, ARM, Hitachi SuperH, Cell,   IBM S/390, MIPS, HP PA-RISC, Intel IA-64, DEC VAX, AMD x86-64, AXIS CRIS,   Xtensa, Tilera TILE, AVR32 and Renesas M32R architectures.    Linux is easily portable to most general-purpose 32- or 64-bit architectures   as long as they have a paged memory management unit (PMMU) and a port of the   GNU C compiler (gcc) (part of The GNU Compiler Collection, GCC). Linux has   also been ported to a number of architectures without a PMMU, although   functionality is then obviously somewhat limited.   Linux has also been ported to itself. You can now run the kernel as a   userspace application - this is called UserMode Linux (UML).  DOCUMENTATION:   - There is a lot of documentation available both in electronic form on    the Internet and in books, both Linux-specific and pertaining to    general UNIX questions.  I'd recommend looking into the documentation    subdirectories on any Linux FTP site for the LDP (Linux Documentation    Project) books.  This README is not meant to be documentation on the    system: there are much better sources available.   - There are various README files in the Documentation/ subdirectory:    these typically contain kernel-specific installation notes for some     drivers for example. See Documentation/00-INDEX for a list of what    is contained in each file.  Please read the Changes file, as it    contains information about the problems, which may result by upgrading    your kernel.   - The Documentation/DocBook/ subdirectory contains several guides for    kernel developers and users.  These guides can be rendered in a    number of formats:  PostScript (.ps), PDF, HTML, &amp; man-pages, among others.    After installation, "make psdocs", "make pdfdocs", "make htmldocs",    or "make mandocs" will render the documentation in the requested format.  INSTALLING the kernel source:   - If you install the full sources, put the kernel tarball in a    directory where you have permissions (eg. your home directory) and    unpack it:       gzip -cd linux-3.X.tar.gz | tar xvf -     or       bzip2 -dc linux-3.X.tar.bz2 | tar xvf -     Replace "X" with the version number of the latest kernel.     Do NOT use the /usr/src/linux area! This area has a (usually    incomplete) set of kernel headers that are used by the library header    files.  They should match the library, and not get messed up by    whatever the kernel-du-jour happens to be.   - You can also upgrade between 3.x releases by patching.  Patches are    distributed in the traditional gzip and the newer bzip2 format.  To    install by patching, get all the newer patch files, enter the    top level directory of the kernel source (linux-3.X) and execute:       gzip -cd ../patch-3.x.gz | patch -p1     or       bzip2 -dc ../patch-3.x.bz2 | patch -p1     Replace "x" for all versions bigger than the version "X" of your current    source tree, _in_order_, and you should be ok.  You may want to remove    the backup files (some-file-name~ or some-file-name.orig), and make sure    that there are no failed patches (some-file-name# or some-file-name.rej).    If there are, either you or I have made a mistake.     Unlike patches for the 3.x kernels, patches for the 3.x.y kernels    (also known as the -stable kernels) are not incremental but instead apply    directly to the base 3.x kernel.  For example, if your base kernel is 3.0    and you want to apply the 3.0.3 patch, you must not first apply the 3.0.1    and 3.0.2 patches. Similarly, if you are running kernel version 3.0.2 and    want to jump to 3.0.3, you must first reverse the 3.0.2 patch (that is,    patch -R) _before_ applying the 3.0.3 patch. You can read more on this in    Documentation/applying-patches.txt     Alternatively, the script patch-kernel can be used to automate this    process.  It determines the current kernel version and applies any    patches found.       linux/scripts/patch-kernel linux     The first argument in the command above is the location of the    kernel source.  Patches are applied from the current directory, but    an alternative directory can be specified as the second argument.   - Make sure you have no stale .o files and dependencies lying around:       cd linux      make mrproper     You should now have the sources correctly installed.  SOFTWARE REQUIREMENTS     Compiling and running the 3.x kernels requires up-to-date    versions of various software packages.  Consult    Documentation/Changes for the minimum version numbers required    and how to get updates for these packages.  Beware that using    excessively old versions of these packages can cause indirect    errors that are very difficult to track down, so don't assume that    you can just update packages when obvious problems arise during    build or operation.  BUILD directory for the kernel:     When compiling the kernel, all output files will per default be    stored together with the kernel source code.    Using the option "make O=output/dir" allow you to specify an alternate    place for the output files (including .config).    Example:       kernel source code: /usr/src/linux-3.X      build directory:    /home/name/build/kernel     To configure and build the kernel, use:       cd /usr/src/linux-3.X      make O=/home/name/build/kernel menuconfig      make O=/home/name/build/kernel      sudo make O=/home/name/build/kernel modules_install install     Please note: If the 'O=output/dir' option is used, then it must be    used for all invocations of make.  CONFIGURING the kernel:     Do not skip this step even if you are only upgrading one minor    version.  New configuration options are added in each release, and    odd problems will turn up if the configuration files are not set up    as expected.  If you want to carry your existing configuration to a    new version with minimal work, use "make oldconfig", which will    only ask you for the answers to new questions.   - Alternative configuration commands are:       "make config"      Plain text interface.       "make menuconfig"  Text based color menus, radiolists &amp; dialogs.       "make nconfig"     Enhanced text based color menus.       "make xconfig"     X windows (Qt) based configuration tool.       "make gconfig"     X windows (Gtk) based configuration tool.       "make oldconfig"   Default all questions based on the contents of                         your existing ./.config file and asking about                         new config symbols.       "make silentoldconfig"                         Like above, but avoids cluttering the screen                         with questions already answered.                         Additionally updates the dependencies.       "make olddefconfig"                         Like above, but sets new symbols to their default                         values without prompting.       "make defconfig"   Create a ./.config file by using the default                         symbol values from either arch/$ARCH/defconfig                         or arch/$ARCH/configs/${PLATFORM}_defconfig,                         depending on the architecture.       "make ${PLATFORM}_defconfig"                         Create a ./.config file by using the default                         symbol values from                         arch/$ARCH/configs/${PLATFORM}_defconfig.                         Use "make help" to get a list of all available                         platforms of your architecture.       "make allyesconfig"                         Create a ./.config file by setting symbol                         values to 'y' as much as possible.       "make allmodconfig"                         Create a ./.config file by setting symbol                         values to 'm' as much as possible.       "make allnoconfig" Create a ./.config file by setting symbol                         values to 'n' as much as possible.       "make randconfig"  Create a ./.config file by setting symbol                         values to random values.       "make localmodconfig" Create a config based on current config and                            loaded modules (lsmod). Disables any module                            option that is not needed for the loaded modules.                             To create a localmodconfig for another machine,                            store the lsmod of that machine into a file                            and pass it in as a LSMOD parameter.                     target$ lsmod &gt; /tmp/mylsmod                    target$ scp /tmp/mylsmod host:/tmp                     host$ make LSMOD=/tmp/mylsmod localmodconfig                             The above also works when cross compiling.       "make localyesconfig" Similar to localmodconfig, except it will convert                            all module options to built in (=y) options.     You can find more information on using the Linux kernel config tools    in Documentation/kbuild/kconfig.txt.   - NOTES on "make config":      - Having unnecessary drivers will make the kernel bigger, and can       under some circumstances lead to problems: probing for a       nonexistent controller card may confuse your other controllers      - Compiling the kernel with "Processor type" set higher than 386       will result in a kernel that does NOT work on a 386.  The       kernel will detect this on bootup, and give up.      - A kernel with math-emulation compiled in will still use the       coprocessor if one is present: the math emulation will just       never get used in that case.  The kernel will be slightly larger,       but will work on different machines regardless of whether they       have a math coprocessor or not.      - The "kernel hacking" configuration details usually result in a       bigger or slower kernel (or both), and can even make the kernel       less stable by configuring some routines to actively try to       break bad code to find kernel problems (kmalloc()).  Thus you       should probably answer 'n' to the questions for "development",       "experimental", or "debugging" features.  COMPILING the kernel:   - Make sure you have at least gcc 3.2 available.    For more information, refer to Documentation/Changes.     Please note that you can still run a.out user programs with this kernel.   - Do a "make" to create a compressed kernel image. It is also    possible to do "make install" if you have lilo installed to suit the    kernel makefiles, but you may want to check your particular lilo setup first.     To do the actual install, you have to be root, but none of the normal    build should require that. Don't take the name of root in vain.   - If you configured any of the parts of the kernel as `modules', you    will also have to do "make modules_install".   - Verbose kernel compile/build output:     Normally, the kernel build system runs in a fairly quiet mode (but not    totally silent).  However, sometimes you or other kernel developers need    to see compile, link, or other commands exactly as they are executed.    For this, use "verbose" build mode.  This is done by inserting    "V=1" in the "make" command.  E.g.:       make V=1 all     To have the build system also tell the reason for the rebuild of each    target, use "V=2".  The default is "V=0".   - Keep a backup kernel handy in case something goes wrong.  This is     especially true for the development releases, since each new release    contains new code which has not been debugged.  Make sure you keep a    backup of the modules corresponding to that kernel, as well.  If you    are installing a new kernel with the same version number as your    working kernel, make a backup of your modules directory before you    do a "make modules_install".     Alternatively, before compiling, use the kernel config option    "LOCALVERSION" to append a unique suffix to the regular kernel version.    LOCALVERSION can be set in the "General Setup" menu.   - In order to boot your new kernel, you'll need to copy the kernel    image (e.g. .../linux/arch/i386/boot/bzImage after compilation)    to the place where your regular bootable kernel is found.    - Booting a kernel directly from a floppy without the assistance of a    bootloader such as LILO, is no longer supported.     If you boot Linux from the hard drive, chances are you use LILO, which    uses the kernel image as specified in the file /etc/lilo.conf.  The    kernel image file is usually /vmlinuz, /boot/vmlinuz, /bzImage or    /boot/bzImage.  To use the new kernel, save a copy of the old image    and copy the new image over the old one.  Then, you MUST RERUN LILO    to update the loading map!! If you don't, you won't be able to boot    the new kernel image.     Reinstalling LILO is usually a matter of running /sbin/lilo.     You may wish to edit /etc/lilo.conf to specify an entry for your    old kernel image (say, /vmlinux.old) in case the new one does not    work.  See the LILO docs for more information.      After reinstalling LILO, you should be all set.  Shutdown the system,    reboot, and enjoy!     If you ever need to change the default root device, video mode,    ramdisk size, etc.  in the kernel image, use the 'rdev' program (or    alternatively the LILO boot options when appropriate).  No need to    recompile the kernel to change these parameters.    - Reboot with the new kernel and enjoy.   IF SOMETHING GOES WRONG:   - If you have problems that seem to be due to kernel bugs, please check    the file MAINTAINERS to see if there is a particular person associated    with the part of the kernel that you are having trouble with. If there    isn't anyone listed there, then the second best thing is to mail    them to me (torvalds@linux-foundation.org), and possibly to any other    relevant mailing-list or to the newsgroup.   - In all bug-reports, *please* tell what kernel you are talking about,    how to duplicate the problem, and what your setup is (use your common    sense).  If the problem is new, tell me so, and if the problem is    old, please try to tell me when you first noticed it.   - If the bug results in a message like       unable to handle kernel paging request at address C0000010      Oops: 0002      EIP:   0010:XXXXXXXX      eax: xxxxxxxx   ebx: xxxxxxxx   ecx: xxxxxxxx   edx: xxxxxxxx      esi: xxxxxxxx   edi: xxxxxxxx   ebp: xxxxxxxx      ds: xxxx  es: xxxx  fs: xxxx  gs: xxxx      Pid: xx, process nr: xx      xx xx xx xx xx xx xx xx xx xx     or similar kernel debugging information on your screen or in your    system log, please duplicate it *exactly*.  The dump may look    incomprehensible to you, but it does contain information that may    help debugging the problem.  The text above the dump is also    important: it tells something about why the kernel dumped code (in    the above example, it's due to a bad kernel pointer). More information    on making sense of the dump is in Documentation/oops-tracing.txt   - If you compiled the kernel with CONFIG_KALLSYMS you can send the dump    as is, otherwise you will have to use the "ksymoops" program to make    sense of the dump (but compiling with CONFIG_KALLSYMS is usually preferred).    This utility can be downloaded from    ftp://ftp.&lt;country&gt;.kernel.org/pub/linux/utils/kernel/ksymoops/ .    Alternatively, you can do the dump lookup by hand:   - In debugging dumps like the above, it helps enormously if you can    look up what the EIP value means.  The hex value as such doesn't help    me or anybody else very much: it will depend on your particular    kernel setup.  What you should do is take the hex value from the EIP    line (ignore the "0010:"), and look it up in the kernel namelist to    see which kernel function contains the offending address.     To find out the kernel function name, you'll need to find the system    binary associated with the kernel that exhibited the symptom.  This is    the file 'linux/vmlinux'.  To extract the namelist and match it against    the EIP from the kernel crash, do:       nm vmlinux | sort | less     This will give you a list of kernel addresses sorted in ascending    order, from which it is simple to find the function that contains the    offending address.  Note that the address given by the kernel    debugging messages will not necessarily match exactly with the    function addresses (in fact, that is very unlikely), so you can't    just 'grep' the list: the list will, however, give you the starting    point of each kernel function, so by looking for the function that    has a starting address lower than the one you are searching for but    is followed by a function with a higher address you will find the one    you want.  In fact, it may be a good idea to include a bit of    "context" in your problem report, giving a few lines around the    interesting one.      If you for some reason cannot do the above (you have a pre-compiled    kernel image or similar), telling me as much about your setup as    possible will help.  Please read the REPORTING-BUGS document for details.   - Alternatively, you can use gdb on a running kernel. (read-only; i.e. you    cannot change values or set break points.) To do this, first compile the    kernel with -g; edit arch/i386/Makefile appropriately, then do a "make    clean". You'll also need to enable CONFIG_PROC_FS (via "make config").     After you've rebooted with the new kernel, do "gdb vmlinux /proc/kcore".    You can now use all the usual gdb commands. The command to look up the    point where your system crashed is "l *0xXXXXXXXX". (Replace the XXXes    with the EIP value.)     gdb'ing a non-running kernel currently fails because gdb (wrongly)    disregards the starting offset for which the kernel is compiled.</t>
+          <t>This is a quick analysis on books suggestions from hacker news</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>https://github.com/N30nHaCkZ/linux</t>
+          <t>https://github.com/AlessandroMozzato/hn_books</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Jupyter Notebook</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2026-06-01T18:47:21Z</t>
+          <t>2026-01-26T19:16:03Z</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>jassics/awesome-genai-security</t>
+          <t>N30nHaCkZ/linux</t>
         </is>
       </c>
       <c r="B365" t="n">
@@ -11350,12 +11350,12 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Curated list of links, references, books videos, tutorials (Free or Paid), Exploit, CTFs, Hacking Practices etc. which are related to GenAI and LLM Security</t>
+          <t xml:space="preserve">  Linux kernel release 3.x &lt;http://kernel.org/&gt;  These are the release notes for Linux version 3.  Read them carefully, as they tell you what this is all about, explain how to install the kernel, and what to do if something goes wrong.   WHAT IS LINUX?    Linux is a clone of the operating system Unix, written from scratch by   Linus Torvalds with assistance from a loosely-knit team of hackers across   the Net. It aims towards POSIX and Single UNIX Specification compliance.    It has all the features you would expect in a modern fully-fledged Unix,   including true multitasking, virtual memory, shared libraries, demand   loading, shared copy-on-write executables, proper memory management,   and multistack networking including IPv4 and IPv6.    It is distributed under the GNU General Public License - see the   accompanying COPYING file for more details.   ON WHAT HARDWARE DOES IT RUN?    Although originally developed first for 32-bit x86-based PCs (386 or higher),   today Linux also runs on (at least) the Compaq Alpha AXP, Sun SPARC and   UltraSPARC, Motorola 68000, PowerPC, PowerPC64, ARM, Hitachi SuperH, Cell,   IBM S/390, MIPS, HP PA-RISC, Intel IA-64, DEC VAX, AMD x86-64, AXIS CRIS,   Xtensa, Tilera TILE, AVR32 and Renesas M32R architectures.    Linux is easily portable to most general-purpose 32- or 64-bit architectures   as long as they have a paged memory management unit (PMMU) and a port of the   GNU C compiler (gcc) (part of The GNU Compiler Collection, GCC). Linux has   also been ported to a number of architectures without a PMMU, although   functionality is then obviously somewhat limited.   Linux has also been ported to itself. You can now run the kernel as a   userspace application - this is called UserMode Linux (UML).  DOCUMENTATION:   - There is a lot of documentation available both in electronic form on    the Internet and in books, both Linux-specific and pertaining to    general UNIX questions.  I'd recommend looking into the documentation    subdirectories on any Linux FTP site for the LDP (Linux Documentation    Project) books.  This README is not meant to be documentation on the    system: there are much better sources available.   - There are various README files in the Documentation/ subdirectory:    these typically contain kernel-specific installation notes for some     drivers for example. See Documentation/00-INDEX for a list of what    is contained in each file.  Please read the Changes file, as it    contains information about the problems, which may result by upgrading    your kernel.   - The Documentation/DocBook/ subdirectory contains several guides for    kernel developers and users.  These guides can be rendered in a    number of formats:  PostScript (.ps), PDF, HTML, &amp; man-pages, among others.    After installation, "make psdocs", "make pdfdocs", "make htmldocs",    or "make mandocs" will render the documentation in the requested format.  INSTALLING the kernel source:   - If you install the full sources, put the kernel tarball in a    directory where you have permissions (eg. your home directory) and    unpack it:       gzip -cd linux-3.X.tar.gz | tar xvf -     or       bzip2 -dc linux-3.X.tar.bz2 | tar xvf -     Replace "X" with the version number of the latest kernel.     Do NOT use the /usr/src/linux area! This area has a (usually    incomplete) set of kernel headers that are used by the library header    files.  They should match the library, and not get messed up by    whatever the kernel-du-jour happens to be.   - You can also upgrade between 3.x releases by patching.  Patches are    distributed in the traditional gzip and the newer bzip2 format.  To    install by patching, get all the newer patch files, enter the    top level directory of the kernel source (linux-3.X) and execute:       gzip -cd ../patch-3.x.gz | patch -p1     or       bzip2 -dc ../patch-3.x.bz2 | patch -p1     Replace "x" for all versions bigger than the version "X" of your current    source tree, _in_order_, and you should be ok.  You may want to remove    the backup files (some-file-name~ or some-file-name.orig), and make sure    that there are no failed patches (some-file-name# or some-file-name.rej).    If there are, either you or I have made a mistake.     Unlike patches for the 3.x kernels, patches for the 3.x.y kernels    (also known as the -stable kernels) are not incremental but instead apply    directly to the base 3.x kernel.  For example, if your base kernel is 3.0    and you want to apply the 3.0.3 patch, you must not first apply the 3.0.1    and 3.0.2 patches. Similarly, if you are running kernel version 3.0.2 and    want to jump to 3.0.3, you must first reverse the 3.0.2 patch (that is,    patch -R) _before_ applying the 3.0.3 patch. You can read more on this in    Documentation/applying-patches.txt     Alternatively, the script patch-kernel can be used to automate this    process.  It determines the current kernel version and applies any    patches found.       linux/scripts/patch-kernel linux     The first argument in the command above is the location of the    kernel source.  Patches are applied from the current directory, but    an alternative directory can be specified as the second argument.   - Make sure you have no stale .o files and dependencies lying around:       cd linux      make mrproper     You should now have the sources correctly installed.  SOFTWARE REQUIREMENTS     Compiling and running the 3.x kernels requires up-to-date    versions of various software packages.  Consult    Documentation/Changes for the minimum version numbers required    and how to get updates for these packages.  Beware that using    excessively old versions of these packages can cause indirect    errors that are very difficult to track down, so don't assume that    you can just update packages when obvious problems arise during    build or operation.  BUILD directory for the kernel:     When compiling the kernel, all output files will per default be    stored together with the kernel source code.    Using the option "make O=output/dir" allow you to specify an alternate    place for the output files (including .config).    Example:       kernel source code: /usr/src/linux-3.X      build directory:    /home/name/build/kernel     To configure and build the kernel, use:       cd /usr/src/linux-3.X      make O=/home/name/build/kernel menuconfig      make O=/home/name/build/kernel      sudo make O=/home/name/build/kernel modules_install install     Please note: If the 'O=output/dir' option is used, then it must be    used for all invocations of make.  CONFIGURING the kernel:     Do not skip this step even if you are only upgrading one minor    version.  New configuration options are added in each release, and    odd problems will turn up if the configuration files are not set up    as expected.  If you want to carry your existing configuration to a    new version with minimal work, use "make oldconfig", which will    only ask you for the answers to new questions.   - Alternative configuration commands are:       "make config"      Plain text interface.       "make menuconfig"  Text based color menus, radiolists &amp; dialogs.       "make nconfig"     Enhanced text based color menus.       "make xconfig"     X windows (Qt) based configuration tool.       "make gconfig"     X windows (Gtk) based configuration tool.       "make oldconfig"   Default all questions based on the contents of                         your existing ./.config file and asking about                         new config symbols.       "make silentoldconfig"                         Like above, but avoids cluttering the screen                         with questions already answered.                         Additionally updates the dependencies.       "make olddefconfig"                         Like above, but sets new symbols to their default                         values without prompting.       "make defconfig"   Create a ./.config file by using the default                         symbol values from either arch/$ARCH/defconfig                         or arch/$ARCH/configs/${PLATFORM}_defconfig,                         depending on the architecture.       "make ${PLATFORM}_defconfig"                         Create a ./.config file by using the default                         symbol values from                         arch/$ARCH/configs/${PLATFORM}_defconfig.                         Use "make help" to get a list of all available                         platforms of your architecture.       "make allyesconfig"                         Create a ./.config file by setting symbol                         values to 'y' as much as possible.       "make allmodconfig"                         Create a ./.config file by setting symbol                         values to 'm' as much as possible.       "make allnoconfig" Create a ./.config file by setting symbol                         values to 'n' as much as possible.       "make randconfig"  Create a ./.config file by setting symbol                         values to random values.       "make localmodconfig" Create a config based on current config and                            loaded modules (lsmod). Disables any module                            option that is not needed for the loaded modules.                             To create a localmodconfig for another machine,                            store the lsmod of that machine into a file                            and pass it in as a LSMOD parameter.                     target$ lsmod &gt; /tmp/mylsmod                    target$ scp /tmp/mylsmod host:/tmp                     host$ make LSMOD=/tmp/mylsmod localmodconfig                             The above also works when cross compiling.       "make localyesconfig" Similar to localmodconfig, except it will convert                            all module options to built in (=y) options.     You can find more information on using the Linux kernel config tools    in Documentation/kbuild/kconfig.txt.   - NOTES on "make config":      - Having unnecessary drivers will make the kernel bigger, and can       under some circumstances lead to problems: probing for a       nonexistent controller card may confuse your other controllers      - Compiling the kernel with "Processor type" set higher than 386       will result in a kernel that does NOT work on a 386.  The       kernel will detect this on bootup, and give up.      - A kernel with math-emulation compiled in will still use the       coprocessor if one is present: the math emulation will just       never get used in that case.  The kernel will be slightly larger,       but will work on different machines regardless of whether they       have a math coprocessor or not.      - The "kernel hacking" configuration details usually result in a       bigger or slower kernel (or both), and can even make the kernel       less stable by configuring some routines to actively try to       break bad code to find kernel problems (kmalloc()).  Thus you       should probably answer 'n' to the questions for "development",       "experimental", or "debugging" features.  COMPILING the kernel:   - Make sure you have at least gcc 3.2 available.    For more information, refer to Documentation/Changes.     Please note that you can still run a.out user programs with this kernel.   - Do a "make" to create a compressed kernel image. It is also    possible to do "make install" if you have lilo installed to suit the    kernel makefiles, but you may want to check your particular lilo setup first.     To do the actual install, you have to be root, but none of the normal    build should require that. Don't take the name of root in vain.   - If you configured any of the parts of the kernel as `modules', you    will also have to do "make modules_install".   - Verbose kernel compile/build output:     Normally, the kernel build system runs in a fairly quiet mode (but not    totally silent).  However, sometimes you or other kernel developers need    to see compile, link, or other commands exactly as they are executed.    For this, use "verbose" build mode.  This is done by inserting    "V=1" in the "make" command.  E.g.:       make V=1 all     To have the build system also tell the reason for the rebuild of each    target, use "V=2".  The default is "V=0".   - Keep a backup kernel handy in case something goes wrong.  This is     especially true for the development releases, since each new release    contains new code which has not been debugged.  Make sure you keep a    backup of the modules corresponding to that kernel, as well.  If you    are installing a new kernel with the same version number as your    working kernel, make a backup of your modules directory before you    do a "make modules_install".     Alternatively, before compiling, use the kernel config option    "LOCALVERSION" to append a unique suffix to the regular kernel version.    LOCALVERSION can be set in the "General Setup" menu.   - In order to boot your new kernel, you'll need to copy the kernel    image (e.g. .../linux/arch/i386/boot/bzImage after compilation)    to the place where your regular bootable kernel is found.    - Booting a kernel directly from a floppy without the assistance of a    bootloader such as LILO, is no longer supported.     If you boot Linux from the hard drive, chances are you use LILO, which    uses the kernel image as specified in the file /etc/lilo.conf.  The    kernel image file is usually /vmlinuz, /boot/vmlinuz, /bzImage or    /boot/bzImage.  To use the new kernel, save a copy of the old image    and copy the new image over the old one.  Then, you MUST RERUN LILO    to update the loading map!! If you don't, you won't be able to boot    the new kernel image.     Reinstalling LILO is usually a matter of running /sbin/lilo.     You may wish to edit /etc/lilo.conf to specify an entry for your    old kernel image (say, /vmlinux.old) in case the new one does not    work.  See the LILO docs for more information.      After reinstalling LILO, you should be all set.  Shutdown the system,    reboot, and enjoy!     If you ever need to change the default root device, video mode,    ramdisk size, etc.  in the kernel image, use the 'rdev' program (or    alternatively the LILO boot options when appropriate).  No need to    recompile the kernel to change these parameters.    - Reboot with the new kernel and enjoy.   IF SOMETHING GOES WRONG:   - If you have problems that seem to be due to kernel bugs, please check    the file MAINTAINERS to see if there is a particular person associated    with the part of the kernel that you are having trouble with. If there    isn't anyone listed there, then the second best thing is to mail    them to me (torvalds@linux-foundation.org), and possibly to any other    relevant mailing-list or to the newsgroup.   - In all bug-reports, *please* tell what kernel you are talking about,    how to duplicate the problem, and what your setup is (use your common    sense).  If the problem is new, tell me so, and if the problem is    old, please try to tell me when you first noticed it.   - If the bug results in a message like       unable to handle kernel paging request at address C0000010      Oops: 0002      EIP:   0010:XXXXXXXX      eax: xxxxxxxx   ebx: xxxxxxxx   ecx: xxxxxxxx   edx: xxxxxxxx      esi: xxxxxxxx   edi: xxxxxxxx   ebp: xxxxxxxx      ds: xxxx  es: xxxx  fs: xxxx  gs: xxxx      Pid: xx, process nr: xx      xx xx xx xx xx xx xx xx xx xx     or similar kernel debugging information on your screen or in your    system log, please duplicate it *exactly*.  The dump may look    incomprehensible to you, but it does contain information that may    help debugging the problem.  The text above the dump is also    important: it tells something about why the kernel dumped code (in    the above example, it's due to a bad kernel pointer). More information    on making sense of the dump is in Documentation/oops-tracing.txt   - If you compiled the kernel with CONFIG_KALLSYMS you can send the dump    as is, otherwise you will have to use the "ksymoops" program to make    sense of the dump (but compiling with CONFIG_KALLSYMS is usually preferred).    This utility can be downloaded from    ftp://ftp.&lt;country&gt;.kernel.org/pub/linux/utils/kernel/ksymoops/ .    Alternatively, you can do the dump lookup by hand:   - In debugging dumps like the above, it helps enormously if you can    look up what the EIP value means.  The hex value as such doesn't help    me or anybody else very much: it will depend on your particular    kernel setup.  What you should do is take the hex value from the EIP    line (ignore the "0010:"), and look it up in the kernel namelist to    see which kernel function contains the offending address.     To find out the kernel function name, you'll need to find the system    binary associated with the kernel that exhibited the symptom.  This is    the file 'linux/vmlinux'.  To extract the namelist and match it against    the EIP from the kernel crash, do:       nm vmlinux | sort | less     This will give you a list of kernel addresses sorted in ascending    order, from which it is simple to find the function that contains the    offending address.  Note that the address given by the kernel    debugging messages will not necessarily match exactly with the    function addresses (in fact, that is very unlikely), so you can't    just 'grep' the list: the list will, however, give you the starting    point of each kernel function, so by looking for the function that    has a starting address lower than the one you are searching for but    is followed by a function with a higher address you will find the one    you want.  In fact, it may be a good idea to include a bit of    "context" in your problem report, giving a few lines around the    interesting one.      If you for some reason cannot do the above (you have a pre-compiled    kernel image or similar), telling me as much about your setup as    possible will help.  Please read the REPORTING-BUGS document for details.   - Alternatively, you can use gdb on a running kernel. (read-only; i.e. you    cannot change values or set break points.) To do this, first compile the    kernel with -g; edit arch/i386/Makefile appropriately, then do a "make    clean". You'll also need to enable CONFIG_PROC_FS (via "make config").     After you've rebooted with the new kernel, do "gdb vmlinux /proc/kcore".    You can now use all the usual gdb commands. The command to look up the    point where your system crashed is "l *0xXXXXXXXX". (Replace the XXXes    with the EIP value.)     gdb'ing a non-running kernel currently fails because gdb (wrongly)    disregards the starting offset for which the kernel is compiled.</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>https://github.com/jassics/awesome-genai-security</t>
+          <t>https://github.com/N30nHaCkZ/linux</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -11365,14 +11365,14 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>2026-06-11T08:54:48Z</t>
+          <t>2026-06-01T18:47:21Z</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>AlessandroMozzato/hn_books</t>
+          <t>DigitalQuinn/InfosecCompilation</t>
         </is>
       </c>
       <c r="B366" t="n">
@@ -11380,29 +11380,29 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>This is a quick analysis on books suggestions from hacker news</t>
+          <t>Infosec Compilation is an information security repository for offensive, defensive, and purple-teaming resources, along with guides designed for advanced penetration testing tactics, techniques, and procedures (TTPs) based on the MITRE framework</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>https://github.com/AlessandroMozzato/hn_books</t>
+          <t>https://github.com/DigitalQuinn/InfosecCompilation</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Jupyter Notebook</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>2026-01-26T19:16:03Z</t>
+          <t>2026-03-27T08:33:56Z</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>DigitalQuinn/InfosecCompilation</t>
+          <t>lsszz2100/VibeHacking</t>
         </is>
       </c>
       <c r="B367" t="n">
@@ -11410,29 +11410,29 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Infosec Compilation is an information security repository for offensive, defensive, and purple-teaming resources, along with guides designed for advanced penetration testing tactics, techniques, and procedures (TTPs) based on the MITRE framework</t>
+          <t>A Collection of Repositories, Videos, Books, and Lecture Materials to Learn Security &amp; Hacking with AI in a Fun Way</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>https://github.com/DigitalQuinn/InfosecCompilation</t>
+          <t>https://github.com/lsszz2100/VibeHacking</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>2026-03-27T08:33:56Z</t>
+          <t>2026-06-12T15:00:45Z</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>RamiBotAI/ramibot</t>
+          <t>dionmulaj/EnumVolcano</t>
         </is>
       </c>
       <c r="B368" t="n">
@@ -11440,29 +11440,29 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>RamiBot v3.8.0 is a local-first AI security operations platform integrating multi-LLM support, a dynamic red/blue team skill pipeline, MCP tool orchestration, Docker terminal access, Tor proxy management, and an auto-integrated Kali-based tool server (rami-kali) for controlled, extensible offensive and defensive workflows</t>
+          <t>EnumVolcano is an open source Bash script which is used to perform automated enumeration for privilege escalation. This tool is dedicated to ethical hackers, red teamers, blue teamers &amp; security analysts.</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>https://github.com/RamiBotAI/ramibot</t>
+          <t>https://github.com/dionmulaj/EnumVolcano</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>2026-06-09T09:45:33Z</t>
+          <t>2026-04-23T21:15:04Z</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>neonoatmeal/Coder-Everyday-Resource-Pack-</t>
+          <t>RamiBotAI/ramibot</t>
         </is>
       </c>
       <c r="B369" t="n">
@@ -11470,29 +11470,29 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>This Resource Pack comes with ethical hacking and unethical eBooks and other things such as programming Anarchism to Survival books to lock picking it also comes with a collection of Kevin mitnick books most of the eBook are the hacking for dummies , programming for dummies etc it also comes with books like how to build your network aka networking and Linux books and more my resource pack contains about 2,780 files Still Adding More I hope you enjoy!!!!</t>
+          <t>RamiBot v3.8.0 is a local-first AI security operations platform integrating multi-LLM support, a dynamic red/blue team skill pipeline, MCP tool orchestration, Docker terminal access, Tor proxy management, and an auto-integrated Kali-based tool server (rami-kali) for controlled, extensible offensive and defensive workflows</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>https://github.com/neonoatmeal/Coder-Everyday-Resource-Pack-</t>
+          <t>https://github.com/RamiBotAI/ramibot</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>2026-04-19T15:05:22Z</t>
+          <t>2026-06-09T09:45:33Z</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>mr-r3b00t/kerberoast_audit</t>
+          <t>neonoatmeal/Coder-Everyday-Resource-Pack-</t>
         </is>
       </c>
       <c r="B370" t="n">
@@ -11500,29 +11500,29 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>A blue team tool to help audit kerberoasting vulnerability status</t>
+          <t>This Resource Pack comes with ethical hacking and unethical eBooks and other things such as programming Anarchism to Survival books to lock picking it also comes with a collection of Kevin mitnick books most of the eBook are the hacking for dummies , programming for dummies etc it also comes with books like how to build your network aka networking and Linux books and more my resource pack contains about 2,780 files Still Adding More I hope you enjoy!!!!</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>https://github.com/mr-r3b00t/kerberoast_audit</t>
+          <t>https://github.com/neonoatmeal/Coder-Everyday-Resource-Pack-</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>PowerShell</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>2026-05-18T10:37:52Z</t>
+          <t>2026-04-19T15:05:22Z</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>dionmulaj/EnumVolcano</t>
+          <t>mr-r3b00t/kerberoast_audit</t>
         </is>
       </c>
       <c r="B371" t="n">
@@ -11530,22 +11530,22 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>EnumVolcano is an open source Bash script which is used to perform automated enumeration for privilege escalation. This tool is dedicated to ethical hackers, red teamers, blue teamers &amp; security analysts.</t>
+          <t>A blue team tool to help audit kerberoasting vulnerability status</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>https://github.com/dionmulaj/EnumVolcano</t>
+          <t>https://github.com/mr-r3b00t/kerberoast_audit</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>PowerShell</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>2026-04-23T21:15:04Z</t>
+          <t>2026-05-18T10:37:52Z</t>
         </is>
       </c>
     </row>
@@ -11582,7 +11582,7 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>alperunal/hacking_booksrc</t>
+          <t>Blizzo/tools</t>
         </is>
       </c>
       <c r="B373" t="n">
@@ -11590,29 +11590,29 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>book source codes from _Hacking: The Art of Exploitation_ 2nd edition by Jon Erickson</t>
+          <t>Simple, useful scripts for red/blue team situations</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>https://github.com/alperunal/hacking_booksrc</t>
+          <t>https://github.com/Blizzo/tools</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>2026-01-27T06:09:55Z</t>
+          <t>2023-12-12T18:00:12Z</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>Blizzo/tools</t>
+          <t>alperunal/hacking_booksrc</t>
         </is>
       </c>
       <c r="B374" t="n">
@@ -11620,22 +11620,22 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Simple, useful scripts for red/blue team situations</t>
+          <t>book source codes from _Hacking: The Art of Exploitation_ 2nd edition by Jon Erickson</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>https://github.com/Blizzo/tools</t>
+          <t>https://github.com/alperunal/hacking_booksrc</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>2023-12-12T18:00:12Z</t>
+          <t>2026-01-27T06:09:55Z</t>
         </is>
       </c>
     </row>
@@ -11882,7 +11882,7 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>bob-reis/SafeSpray</t>
+          <t>digitalarche/OnlineToolsForBlueTeam</t>
         </is>
       </c>
       <c r="B383" t="n">
@@ -11890,29 +11890,29 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>SafeSpray is a client-side tool for studies, awareness, and authorized authentication testing (pentest/OSINT/blue team). Everything runs in the browser: no data is sent to servers. The focus is educational and ethical, with internal limits to prevent abuse and practical documentation.</t>
+          <t>By Categories all online tools for blueteam</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>https://github.com/bob-reis/SafeSpray</t>
+          <t>https://github.com/digitalarche/OnlineToolsForBlueTeam</t>
         </is>
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>2026-02-09T23:46:20Z</t>
+          <t>2026-01-29T17:11:06Z</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>ilyess-sellami/BlueTeam-Handbook</t>
+          <t>chousensha/cyber-support-base</t>
         </is>
       </c>
       <c r="B384" t="n">
@@ -11920,12 +11920,12 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>BlueTeam-Handbook – A complete SOC1/2 interview and Blue Team guide with categorized questions, case studies, tools, and real-world defensive security scenarios.</t>
+          <t>Collection of bookmarked tools for security, red teaming, blue teaming, pentesting and other</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>https://github.com/ilyess-sellami/BlueTeam-Handbook</t>
+          <t>https://github.com/chousensha/cyber-support-base</t>
         </is>
       </c>
       <c r="E384" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>2026-04-11T18:07:15Z</t>
+          <t>2025-05-25T11:57:17Z</t>
         </is>
       </c>
     </row>
@@ -11972,7 +11972,7 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>pentestify/omgeasymon</t>
+          <t>ilyess-sellami/BlueTeam-Handbook</t>
         </is>
       </c>
       <c r="B386" t="n">
@@ -11980,29 +11980,29 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Simple CCDC monitoring tool for red or blue teams</t>
+          <t>BlueTeam-Handbook – A complete SOC1/2 interview and Blue Team guide with categorized questions, case studies, tools, and real-world defensive security scenarios.</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>https://github.com/pentestify/omgeasymon</t>
+          <t>https://github.com/ilyess-sellami/BlueTeam-Handbook</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Ruby</t>
+          <t>Non spécifiée</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>2024-02-19T18:12:41Z</t>
+          <t>2026-04-11T18:07:15Z</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>digitalarche/OnlineToolsForBlueTeam</t>
+          <t>pentestify/omgeasymon</t>
         </is>
       </c>
       <c r="B387" t="n">
@@ -12010,29 +12010,29 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>By Categories all online tools for blueteam</t>
+          <t>Simple CCDC monitoring tool for red or blue teams</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>https://github.com/digitalarche/OnlineToolsForBlueTeam</t>
+          <t>https://github.com/pentestify/omgeasymon</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>Ruby</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>2026-01-29T17:11:06Z</t>
+          <t>2024-02-19T18:12:41Z</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>chousensha/cyber-support-base</t>
+          <t>bob-reis/SafeSpray</t>
         </is>
       </c>
       <c r="B388" t="n">
@@ -12040,22 +12040,22 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Collection of bookmarked tools for security, red teaming, blue teaming, pentesting and other</t>
+          <t>SafeSpray is a client-side tool for studies, awareness, and authorized authentication testing (pentest/OSINT/blue team). Everything runs in the browser: no data is sent to servers. The focus is educational and ethical, with internal limits to prevent abuse and practical documentation.</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>https://github.com/chousensha/cyber-support-base</t>
+          <t>https://github.com/bob-reis/SafeSpray</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Non spécifiée</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>2025-05-25T11:57:17Z</t>
+          <t>2026-02-09T23:46:20Z</t>
         </is>
       </c>
     </row>
@@ -13522,7 +13522,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -13792,7 +13792,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -14170,7 +14170,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -14926,7 +14926,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -15520,7 +15520,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -18436,7 +18436,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -20731,7 +20731,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -21892,7 +21892,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -21946,7 +21946,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Hors ligne</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -22162,7 +22162,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
@@ -22432,7 +22432,7 @@
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E384" t="inlineStr">
@@ -26968,7 +26968,7 @@
       </c>
       <c r="D552" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E552" t="inlineStr">
@@ -28075,7 +28075,7 @@
       </c>
       <c r="D593" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E593" t="inlineStr">
@@ -28102,7 +28102,7 @@
       </c>
       <c r="D594" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E594" t="inlineStr">
@@ -28156,7 +28156,7 @@
       </c>
       <c r="D596" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E596" t="inlineStr">
@@ -28723,7 +28723,7 @@
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E617" t="inlineStr">
@@ -28804,7 +28804,7 @@
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E620" t="inlineStr">
@@ -29317,7 +29317,7 @@
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E639" t="inlineStr">
@@ -29479,7 +29479,7 @@
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Hors ligne</t>
         </is>
       </c>
       <c r="E645" t="inlineStr">
@@ -29965,7 +29965,7 @@
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Hors ligne</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
@@ -33205,7 +33205,7 @@
       </c>
       <c r="D783" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E783" t="inlineStr">
@@ -33232,7 +33232,7 @@
       </c>
       <c r="D784" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E784" t="inlineStr">
@@ -33799,7 +33799,7 @@
       </c>
       <c r="D805" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E805" t="inlineStr">
@@ -34528,7 +34528,7 @@
       </c>
       <c r="D832" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E832" t="inlineStr">
@@ -34582,7 +34582,7 @@
       </c>
       <c r="D834" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E834" t="inlineStr">
@@ -34690,7 +34690,7 @@
       </c>
       <c r="D838" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E838" t="inlineStr">
@@ -36148,7 +36148,7 @@
       </c>
       <c r="D892" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E892" t="inlineStr">
@@ -36283,7 +36283,7 @@
       </c>
       <c r="D897" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E897" t="inlineStr">
@@ -36391,7 +36391,7 @@
       </c>
       <c r="D901" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E901" t="inlineStr">
@@ -36418,7 +36418,7 @@
       </c>
       <c r="D902" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E902" t="inlineStr">
@@ -36796,7 +36796,7 @@
       </c>
       <c r="D916" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E916" t="inlineStr">
@@ -37120,7 +37120,7 @@
       </c>
       <c r="D928" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E928" t="inlineStr">
@@ -37147,7 +37147,7 @@
       </c>
       <c r="D929" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E929" t="inlineStr">
@@ -37741,7 +37741,7 @@
       </c>
       <c r="D951" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Hors ligne</t>
         </is>
       </c>
       <c r="E951" t="inlineStr">
@@ -38794,7 +38794,7 @@
       </c>
       <c r="D990" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E990" t="inlineStr">
@@ -38821,7 +38821,7 @@
       </c>
       <c r="D991" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E991" t="inlineStr">
@@ -39172,7 +39172,7 @@
       </c>
       <c r="D1004" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1004" t="inlineStr">
@@ -40171,7 +40171,7 @@
       </c>
       <c r="D1041" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1041" t="inlineStr">
@@ -40468,7 +40468,7 @@
       </c>
       <c r="D1052" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1052" t="inlineStr">
@@ -41845,7 +41845,7 @@
       </c>
       <c r="D1103" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1103" t="inlineStr">
@@ -41980,7 +41980,7 @@
       </c>
       <c r="D1108" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1108" t="inlineStr">
@@ -42196,7 +42196,7 @@
       </c>
       <c r="D1116" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1116" t="inlineStr">
@@ -43087,7 +43087,7 @@
       </c>
       <c r="D1149" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1149" t="inlineStr">
@@ -43492,7 +43492,7 @@
       </c>
       <c r="D1164" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1164" t="inlineStr">
@@ -44005,7 +44005,7 @@
       </c>
       <c r="D1183" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1183" t="inlineStr">
@@ -44059,7 +44059,7 @@
       </c>
       <c r="D1185" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1185" t="inlineStr">
@@ -44113,7 +44113,7 @@
       </c>
       <c r="D1187" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1187" t="inlineStr">
@@ -44599,7 +44599,7 @@
       </c>
       <c r="D1205" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1205" t="inlineStr">
@@ -45868,7 +45868,7 @@
       </c>
       <c r="D1252" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1252" t="inlineStr">
@@ -46192,7 +46192,7 @@
       </c>
       <c r="D1264" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1264" t="inlineStr">
@@ -46462,7 +46462,7 @@
       </c>
       <c r="D1274" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1274" t="inlineStr">
@@ -46516,7 +46516,7 @@
       </c>
       <c r="D1276" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1276" t="inlineStr">
@@ -46651,7 +46651,7 @@
       </c>
       <c r="D1281" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1281" t="inlineStr">
@@ -47029,7 +47029,7 @@
       </c>
       <c r="D1295" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1295" t="inlineStr">
@@ -47326,7 +47326,7 @@
       </c>
       <c r="D1306" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1306" t="inlineStr">
@@ -47515,7 +47515,7 @@
       </c>
       <c r="D1313" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1313" t="inlineStr">
@@ -47677,7 +47677,7 @@
       </c>
       <c r="D1319" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1319" t="inlineStr">
@@ -47839,7 +47839,7 @@
       </c>
       <c r="D1325" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Hors ligne</t>
         </is>
       </c>
       <c r="E1325" t="inlineStr">
@@ -48244,7 +48244,7 @@
       </c>
       <c r="D1340" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1340" t="inlineStr">
@@ -48298,7 +48298,7 @@
       </c>
       <c r="D1342" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1342" t="inlineStr">
@@ -48487,7 +48487,7 @@
       </c>
       <c r="D1349" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1349" t="inlineStr">
@@ -48514,7 +48514,7 @@
       </c>
       <c r="D1350" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1350" t="inlineStr">
@@ -49135,7 +49135,7 @@
       </c>
       <c r="D1373" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1373" t="inlineStr">
@@ -49405,7 +49405,7 @@
       </c>
       <c r="D1383" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1383" t="inlineStr">
@@ -49621,7 +49621,7 @@
       </c>
       <c r="D1391" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1391" t="inlineStr">
@@ -49783,7 +49783,7 @@
       </c>
       <c r="D1397" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1397" t="inlineStr">
@@ -50512,7 +50512,7 @@
       </c>
       <c r="D1424" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Hors ligne</t>
         </is>
       </c>
       <c r="E1424" t="inlineStr">
@@ -50782,7 +50782,7 @@
       </c>
       <c r="D1434" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1434" t="inlineStr">
@@ -50863,7 +50863,7 @@
       </c>
       <c r="D1437" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1437" t="inlineStr">
@@ -56425,7 +56425,7 @@
       </c>
       <c r="D1643" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1643" t="inlineStr">
@@ -56938,7 +56938,7 @@
       </c>
       <c r="D1662" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1662" t="inlineStr">
@@ -57370,7 +57370,7 @@
       </c>
       <c r="D1678" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1678" t="inlineStr">
@@ -57748,7 +57748,7 @@
       </c>
       <c r="D1692" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Hors ligne</t>
         </is>
       </c>
       <c r="E1692" t="inlineStr">
@@ -58666,7 +58666,7 @@
       </c>
       <c r="D1726" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1726" t="inlineStr">
@@ -58774,7 +58774,7 @@
       </c>
       <c r="D1730" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1730" t="inlineStr">
@@ -59422,7 +59422,7 @@
       </c>
       <c r="D1754" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1754" t="inlineStr">
@@ -59476,7 +59476,7 @@
       </c>
       <c r="D1756" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1756" t="inlineStr">
@@ -59530,7 +59530,7 @@
       </c>
       <c r="D1758" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1758" t="inlineStr">
@@ -60043,7 +60043,7 @@
       </c>
       <c r="D1777" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1777" t="inlineStr">
@@ -60232,7 +60232,7 @@
       </c>
       <c r="D1784" t="inlineStr">
         <is>
-          <t>Non vérifié</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="E1784" t="inlineStr">

</xml_diff>